<commit_message>
Modelar los escenarios optimista y pesimista y su evaluación comparada
- La planilla suma las hojas Optimista y Pesimista, con la misma estructura
  que la Neutral, y una hoja Resumen con los indicadores de los tres.
- El validador controla los tres escenarios y escribe la tabla comparada
  financiero-comparada.tex; se agregan dos tests.
- El cap. 3 incorpora los escenarios optimista y pesimista y la subsección
  «Evaluación financiera de escenarios» con la conclusión de viabilidad.
- Se actualizan analisis-financiero.md, index.md y log.md.

Refs #53

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -9,7 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="Supuestos" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Neutral" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Optimista" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Neutral" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Pesimista" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="ajuste_sueldo" vbProcedure="false">Supuestos!$D$24</definedName>
@@ -92,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="293">
   <si>
     <t xml:space="preserve">clave</t>
   </si>
@@ -757,202 +760,220 @@
     <t xml:space="preserve">Churn anual: agencias</t>
   </si>
   <si>
+    <t xml:space="preserve">Indicador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pesimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAN (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payback simple (años)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payback descontado (años)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Punto de equilibrio (clientes B2B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingreso medio por cliente B2B en el año 5 (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escenario optimista (USD nominales; todo lo derivado es fórmula)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columna de escenario en Supuestos (1 = optimista, 2 = neutral, 3 = pesimista)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año calendario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Año electoral (1 = sí)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventas B2B habilitadas (1 = sí)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuarios activos mensuales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios de gran porte: activos al inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios de gran porte: bajas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios de gran porte: altas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios de gran porte: activos al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios de gran porte: promedio del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios socios de ADEPA (resto): activos al inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios socios de ADEPA (resto): bajas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios socios de ADEPA (resto): altas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios socios de ADEPA (resto): activos al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medios socios de ADEPA (resto): promedio del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificadores: activos al inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificadores: bajas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificadores: altas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificadores: activos al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificadores: promedio del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidades y observatorios: activos al inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidades y observatorios: bajas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidades y observatorios: altas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidades y observatorios: activos al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidades y observatorios: promedio del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agencias: activos al inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agencias: bajas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agencias: altas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agencias: activos al cierre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agencias: promedio del año</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organismos y ONG: contratos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clientes B2B (promedio del año, con contratos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos por producto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos: API nivel superior (Medios de gran porte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos: API nivel intermedio (Medios socios de ADEPA (resto))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos: panel de tendencias y API intermedia (Verificadores)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos: acceso histórico (Universidades y observatorios)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos: API nivel superior (Agencias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos: reportes de monitoreo electoral, organismos y ONG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresos totales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costos por rubro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo: recursos humanos (desarrollador semi senior)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo: infraestructura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo: hosting del modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo: marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo: dominio, Chrome Web Store, marca y asesoría legal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo variable: análisis de usuarios gratuitos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo variable: consultas de la API B2B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costos totales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flujo de caja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flujo neto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factor de descuento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flujo descontado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flujo neto acumulado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flujo descontado acumulado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recupero simple: a + b/c en el año del cruce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recupero descontado: a + b/c en el año del cruce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicadores</t>
+  </si>
+  <si>
     <t xml:space="preserve">Escenario neutral (USD nominales; todo lo derivado es fórmula)</t>
   </si>
   <si>
-    <t xml:space="preserve">Columna de escenario en Supuestos (1 = optimista, 2 = neutral, 3 = pesimista)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Año calendario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Año electoral (1 = sí)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventas B2B habilitadas (1 = sí)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usuarios activos mensuales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios de gran porte: activos al inicio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios de gran porte: bajas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios de gran porte: altas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios de gran porte: activos al cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios de gran porte: promedio del año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios socios de ADEPA (resto): activos al inicio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios socios de ADEPA (resto): bajas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios socios de ADEPA (resto): altas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios socios de ADEPA (resto): activos al cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medios socios de ADEPA (resto): promedio del año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificadores: activos al inicio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificadores: bajas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificadores: altas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificadores: activos al cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificadores: promedio del año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universidades y observatorios: activos al inicio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universidades y observatorios: bajas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universidades y observatorios: altas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universidades y observatorios: activos al cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universidades y observatorios: promedio del año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agencias: activos al inicio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agencias: bajas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agencias: altas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agencias: activos al cierre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agencias: promedio del año</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Organismos y ONG: contratos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clientes B2B (promedio del año, con contratos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos por producto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos: API nivel superior (Medios de gran porte)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos: API nivel intermedio (Medios socios de ADEPA (resto))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos: panel de tendencias y API intermedia (Verificadores)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos: acceso histórico (Universidades y observatorios)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos: API nivel superior (Agencias)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos: reportes de monitoreo electoral, organismos y ONG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresos totales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costos por rubro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo: recursos humanos (desarrollador semi senior)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo: infraestructura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo: hosting del modelo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo: marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo: dominio, Chrome Web Store, marca y asesoría legal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo variable: análisis de usuarios gratuitos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costo variable: consultas de la API B2B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Costos totales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flujo de caja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flujo neto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Factor de descuento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flujo descontado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flujo neto acumulado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flujo descontado acumulado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recupero simple: a + b/c en el año del cruce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recupero descontado: a + b/c en el año del cruce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicadores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VAN (USD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Payback simple (años)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Payback descontado (años)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingreso medio por cliente B2B en el año 5 (USD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Punto de equilibrio (clientes B2B)</t>
+    <t xml:space="preserve">Escenario pesimista (USD nominales; todo lo derivado es fórmula)</t>
   </si>
 </sst>
 </file>
@@ -3029,6 +3050,144 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <f aca="false">Optimista!B67</f>
+        <v>1101468.41536853</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <f aca="false">Neutral!B67</f>
+        <v>1862.37728290133</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <f aca="false">Pesimista!B67</f>
+        <v>-153462.061591211</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <f aca="false">Optimista!B68</f>
+        <v>10.3696253055461</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <f aca="false">Neutral!B68</f>
+        <v>0.26328384883344</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <f aca="false">Pesimista!B68</f>
+        <v>no definida</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <f aca="false">Optimista!B69</f>
+        <v>0.103947535807236</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">Neutral!B69</f>
+        <v>3.31706526291709</v>
+      </c>
+      <c r="D4" s="0" t="str">
+        <f aca="false">Pesimista!B69</f>
+        <v>no se recupera</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">Optimista!B70</f>
+        <v>0.129934419759044</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <f aca="false">Neutral!B70</f>
+        <v>4.89511209324086</v>
+      </c>
+      <c r="D5" s="0" t="str">
+        <f aca="false">Pesimista!B70</f>
+        <v>no se recupera</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <f aca="false">Optimista!B72</f>
+        <v>40</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <f aca="false">Neutral!B72</f>
+        <v>36</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <f aca="false">Pesimista!B72</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <f aca="false">Optimista!B71</f>
+        <v>10781.4432989691</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">Neutral!B71</f>
+        <v>8901.20481927711</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <f aca="false">Pesimista!B71</f>
+        <v>5600</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3037,20 +3196,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B2" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -3079,7 +3238,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -3108,7 +3267,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -3137,7 +3296,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -3145,7 +3304,7 @@
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">IF(C$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">IF(D$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -3166,7 +3325,1507 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
+        <v>5000</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,D$3,$B$2)</f>
+        <v>20000</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,E$3,$B$2)</f>
+        <v>50000</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,F$3,$B$2)</f>
+        <v>100000</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,G$3,$B$2)</f>
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <f aca="false">N(B13)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <f aca="false">N(C13)</f>
+        <v>2</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <f aca="false">N(D13)</f>
+        <v>4</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <f aca="false">N(E13)</f>
+        <v>5</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <f aca="false">N(F13)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*D10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*E10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*F10,0)</f>
+        <v>1</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*G10,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>240</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-C10),0)</f>
+        <v>2</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-D10),0)</f>
+        <v>2</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-E10),0)</f>
+        <v>1</v>
+      </c>
+      <c r="F12" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-F10),0)</f>
+        <v>1</v>
+      </c>
+      <c r="G12" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-G10),0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <f aca="false">C10+C12-C11</f>
+        <v>2</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <f aca="false">D10+D12-D11</f>
+        <v>4</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <f aca="false">E10+E12-E11</f>
+        <v>5</v>
+      </c>
+      <c r="F13" s="0" t="n">
+        <f aca="false">F10+F12-F11</f>
+        <v>5</v>
+      </c>
+      <c r="G13" s="0" t="n">
+        <f aca="false">G10+G12-G11</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>242</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <f aca="false">(C10+C13)/2</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <f aca="false">(D10+D13)/2</f>
+        <v>3</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <f aca="false">(E10+E13)/2</f>
+        <v>4.5</v>
+      </c>
+      <c r="F14" s="0" t="n">
+        <f aca="false">(F10+F13)/2</f>
+        <v>5</v>
+      </c>
+      <c r="G14" s="0" t="n">
+        <f aca="false">(G10+G13)/2</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <f aca="false">N(B18)</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <f aca="false">N(C18)</f>
+        <v>9</v>
+      </c>
+      <c r="E15" s="0" t="n">
+        <f aca="false">N(D18)</f>
+        <v>16</v>
+      </c>
+      <c r="F15" s="0" t="n">
+        <f aca="false">N(E18)</f>
+        <v>22</v>
+      </c>
+      <c r="G15" s="0" t="n">
+        <f aca="false">N(F18)</f>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*D15,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*E15,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*F15,0)</f>
+        <v>3</v>
+      </c>
+      <c r="G16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*G15,0)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-C15),0)</f>
+        <v>9</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-D15),0)</f>
+        <v>8</v>
+      </c>
+      <c r="E17" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-E15),0)</f>
+        <v>8</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-F15),0)</f>
+        <v>7</v>
+      </c>
+      <c r="G17" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-G15),0)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <f aca="false">C15+C17-C16</f>
+        <v>9</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <f aca="false">D15+D17-D16</f>
+        <v>16</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <f aca="false">E15+E17-E16</f>
+        <v>22</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <f aca="false">F15+F17-F16</f>
+        <v>26</v>
+      </c>
+      <c r="G18" s="0" t="n">
+        <f aca="false">G15+G17-G16</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <f aca="false">(C15+C18)/2</f>
+        <v>4.5</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <f aca="false">(D15+D18)/2</f>
+        <v>12.5</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <f aca="false">(E15+E18)/2</f>
+        <v>19</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <f aca="false">(F15+F18)/2</f>
+        <v>24</v>
+      </c>
+      <c r="G19" s="0" t="n">
+        <f aca="false">(G15+G18)/2</f>
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <f aca="false">N(B23)</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <f aca="false">N(C23)</f>
+        <v>1</v>
+      </c>
+      <c r="E20" s="0" t="n">
+        <f aca="false">N(D23)</f>
+        <v>2</v>
+      </c>
+      <c r="F20" s="0" t="n">
+        <f aca="false">N(E23)</f>
+        <v>2</v>
+      </c>
+      <c r="G20" s="0" t="n">
+        <f aca="false">N(F23)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*D20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*E20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*F20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*G20,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>250</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-C20),0)</f>
+        <v>1</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-D20),0)</f>
+        <v>1</v>
+      </c>
+      <c r="E22" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-E20),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-F20),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-G20),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <f aca="false">C20+C22-C21</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <f aca="false">D20+D22-D21</f>
+        <v>2</v>
+      </c>
+      <c r="E23" s="0" t="n">
+        <f aca="false">E20+E22-E21</f>
+        <v>2</v>
+      </c>
+      <c r="F23" s="0" t="n">
+        <f aca="false">F20+F22-F21</f>
+        <v>2</v>
+      </c>
+      <c r="G23" s="0" t="n">
+        <f aca="false">G20+G22-G21</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <f aca="false">(C20+C23)/2</f>
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <f aca="false">(D20+D23)/2</f>
+        <v>1.5</v>
+      </c>
+      <c r="E24" s="0" t="n">
+        <f aca="false">(E20+E23)/2</f>
+        <v>2</v>
+      </c>
+      <c r="F24" s="0" t="n">
+        <f aca="false">(F20+F23)/2</f>
+        <v>2</v>
+      </c>
+      <c r="G24" s="0" t="n">
+        <f aca="false">(G20+G23)/2</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <f aca="false">N(B28)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <f aca="false">N(C28)</f>
+        <v>12</v>
+      </c>
+      <c r="E25" s="0" t="n">
+        <f aca="false">N(D28)</f>
+        <v>22</v>
+      </c>
+      <c r="F25" s="0" t="n">
+        <f aca="false">N(E28)</f>
+        <v>31</v>
+      </c>
+      <c r="G25" s="0" t="n">
+        <f aca="false">N(F28)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="C26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*D25,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*E25,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*F25,0)</f>
+        <v>2</v>
+      </c>
+      <c r="G26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*G25,0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="C27" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-C25),0)</f>
+        <v>12</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-D25),0)</f>
+        <v>11</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-E25),0)</f>
+        <v>10</v>
+      </c>
+      <c r="F27" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-F25),0)</f>
+        <v>9</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-G25),0)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <f aca="false">C25+C27-C26</f>
+        <v>12</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <f aca="false">D25+D27-D26</f>
+        <v>22</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <f aca="false">E25+E27-E26</f>
+        <v>31</v>
+      </c>
+      <c r="F28" s="0" t="n">
+        <f aca="false">F25+F27-F26</f>
+        <v>38</v>
+      </c>
+      <c r="G28" s="0" t="n">
+        <f aca="false">G25+G27-G26</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="C29" s="0" t="n">
+        <f aca="false">(C25+C28)/2</f>
+        <v>6</v>
+      </c>
+      <c r="D29" s="0" t="n">
+        <f aca="false">(D25+D28)/2</f>
+        <v>17</v>
+      </c>
+      <c r="E29" s="0" t="n">
+        <f aca="false">(E25+E28)/2</f>
+        <v>26.5</v>
+      </c>
+      <c r="F29" s="0" t="n">
+        <f aca="false">(F25+F28)/2</f>
+        <v>34.5</v>
+      </c>
+      <c r="G29" s="0" t="n">
+        <f aca="false">(G25+G28)/2</f>
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <f aca="false">N(B33)</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="0" t="n">
+        <f aca="false">N(C33)</f>
+        <v>6</v>
+      </c>
+      <c r="E30" s="0" t="n">
+        <f aca="false">N(D33)</f>
+        <v>11</v>
+      </c>
+      <c r="F30" s="0" t="n">
+        <f aca="false">N(E33)</f>
+        <v>14</v>
+      </c>
+      <c r="G30" s="0" t="n">
+        <f aca="false">N(F33)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*D30,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*E30,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*F30,0)</f>
+        <v>2</v>
+      </c>
+      <c r="G31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*G30,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="C32" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-C30),0)</f>
+        <v>6</v>
+      </c>
+      <c r="D32" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-D30),0)</f>
+        <v>6</v>
+      </c>
+      <c r="E32" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-E30),0)</f>
+        <v>5</v>
+      </c>
+      <c r="F32" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-F30),0)</f>
+        <v>5</v>
+      </c>
+      <c r="G32" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-G30),0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="C33" s="0" t="n">
+        <f aca="false">C30+C32-C31</f>
+        <v>6</v>
+      </c>
+      <c r="D33" s="0" t="n">
+        <f aca="false">D30+D32-D31</f>
+        <v>11</v>
+      </c>
+      <c r="E33" s="0" t="n">
+        <f aca="false">E30+E32-E31</f>
+        <v>14</v>
+      </c>
+      <c r="F33" s="0" t="n">
+        <f aca="false">F30+F32-F31</f>
+        <v>17</v>
+      </c>
+      <c r="G33" s="0" t="n">
+        <f aca="false">G30+G32-G31</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="C34" s="0" t="n">
+        <f aca="false">(C30+C33)/2</f>
+        <v>3</v>
+      </c>
+      <c r="D34" s="0" t="n">
+        <f aca="false">(D30+D33)/2</f>
+        <v>8.5</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <f aca="false">(E30+E33)/2</f>
+        <v>12.5</v>
+      </c>
+      <c r="F34" s="0" t="n">
+        <f aca="false">(F30+F33)/2</f>
+        <v>15.5</v>
+      </c>
+      <c r="G34" s="0" t="n">
+        <f aca="false">(G30+G33)/2</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="C35" s="0" t="n">
+        <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>3</v>
+      </c>
+      <c r="D35" s="0" t="n">
+        <f aca="false">D5*D6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="0" t="n">
+        <f aca="false">E5*E6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>3</v>
+      </c>
+      <c r="F35" s="0" t="n">
+        <f aca="false">F5*F6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="0" t="n">
+        <f aca="false">G5*G6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="C36" s="0" t="n">
+        <f aca="false">C14+C19+C24+C29+C34+C35</f>
+        <v>18</v>
+      </c>
+      <c r="D36" s="0" t="n">
+        <f aca="false">D14+D19+D24+D29+D34+D35</f>
+        <v>42.5</v>
+      </c>
+      <c r="E36" s="0" t="n">
+        <f aca="false">E14+E19+E24+E29+E34+E35</f>
+        <v>67.5</v>
+      </c>
+      <c r="F36" s="0" t="n">
+        <f aca="false">F14+F19+F24+F29+F34+F35</f>
+        <v>81</v>
+      </c>
+      <c r="G36" s="0" t="n">
+        <f aca="false">G14+G19+G24+G29+G34+G35</f>
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C39" s="0" t="n">
+        <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>36000</v>
+      </c>
+      <c r="D39" s="0" t="n">
+        <f aca="false">D14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>108000</v>
+      </c>
+      <c r="E39" s="0" t="n">
+        <f aca="false">E14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>162000</v>
+      </c>
+      <c r="F39" s="0" t="n">
+        <f aca="false">F14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>180000</v>
+      </c>
+      <c r="G39" s="0" t="n">
+        <f aca="false">G14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>180000</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="C40" s="0" t="n">
+        <f aca="false">C19*precio_medios_chicos*meses_anio</f>
+        <v>10800</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <f aca="false">D19*precio_medios_chicos*meses_anio</f>
+        <v>30000</v>
+      </c>
+      <c r="E40" s="0" t="n">
+        <f aca="false">E19*precio_medios_chicos*meses_anio</f>
+        <v>45600</v>
+      </c>
+      <c r="F40" s="0" t="n">
+        <f aca="false">F19*precio_medios_chicos*meses_anio</f>
+        <v>57600</v>
+      </c>
+      <c r="G40" s="0" t="n">
+        <f aca="false">G19*precio_medios_chicos*meses_anio</f>
+        <v>66000</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="C41" s="0" t="n">
+        <f aca="false">C24*precio_verificadores*meses_anio</f>
+        <v>3000</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <f aca="false">D24*precio_verificadores*meses_anio</f>
+        <v>9000</v>
+      </c>
+      <c r="E41" s="0" t="n">
+        <f aca="false">E24*precio_verificadores*meses_anio</f>
+        <v>12000</v>
+      </c>
+      <c r="F41" s="0" t="n">
+        <f aca="false">F24*precio_verificadores*meses_anio</f>
+        <v>12000</v>
+      </c>
+      <c r="G41" s="0" t="n">
+        <f aca="false">G24*precio_verificadores*meses_anio</f>
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="C42" s="0" t="n">
+        <f aca="false">C29*precio_universidades*meses_anio</f>
+        <v>7200</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <f aca="false">D29*precio_universidades*meses_anio</f>
+        <v>20400</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <f aca="false">E29*precio_universidades*meses_anio</f>
+        <v>31800</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <f aca="false">F29*precio_universidades*meses_anio</f>
+        <v>41400</v>
+      </c>
+      <c r="G42" s="0" t="n">
+        <f aca="false">G29*precio_universidades*meses_anio</f>
+        <v>49800</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="C43" s="0" t="n">
+        <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>108000</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <f aca="false">D34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>306000</v>
+      </c>
+      <c r="E43" s="0" t="n">
+        <f aca="false">E34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>450000</v>
+      </c>
+      <c r="F43" s="0" t="n">
+        <f aca="false">F34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>558000</v>
+      </c>
+      <c r="G43" s="0" t="n">
+        <f aca="false">G34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>648000</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C44" s="0" t="n">
+        <f aca="false">C35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>90000</v>
+      </c>
+      <c r="D44" s="0" t="n">
+        <f aca="false">D35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="0" t="n">
+        <f aca="false">E35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>90000</v>
+      </c>
+      <c r="F44" s="0" t="n">
+        <f aca="false">F35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="0" t="n">
+        <f aca="false">G35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="B45" s="0" t="n">
+        <f aca="false">SUM(B39:B44)</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <f aca="false">SUM(C39:C44)</f>
+        <v>255000</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <f aca="false">SUM(D39:D44)</f>
+        <v>473400</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <f aca="false">SUM(E39:E44)</f>
+        <v>791400</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <f aca="false">SUM(F39:F44)</f>
+        <v>849000</v>
+      </c>
+      <c r="G45" s="0" t="n">
+        <f aca="false">SUM(G39:G44)</f>
+        <v>1045800</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="B48" s="0" t="n">
+        <f aca="false">meses_anio_0*sueldo_usd*sueldos_por_anio/meses_anio</f>
+        <v>19391.6666666667</v>
+      </c>
+      <c r="C48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^C$3</f>
+        <v>24433.5</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^D$3</f>
+        <v>25655.175</v>
+      </c>
+      <c r="E48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^E$3</f>
+        <v>26937.93375</v>
+      </c>
+      <c r="F48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^F$3</f>
+        <v>28284.8304375</v>
+      </c>
+      <c r="G48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^G$3</f>
+        <v>29699.071959375</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="B49" s="0" t="n">
+        <f aca="false">inv_infraestructura_0</f>
+        <v>168</v>
+      </c>
+      <c r="C49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*C7/ua_escalado)+dominio_anual</f>
+        <v>663</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*D7/ua_escalado)+dominio_anual</f>
+        <v>843</v>
+      </c>
+      <c r="E49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*E7/ua_escalado)+dominio_anual</f>
+        <v>1203</v>
+      </c>
+      <c r="F49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*F7/ua_escalado)+dominio_anual</f>
+        <v>1803</v>
+      </c>
+      <c r="G49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*G7/ua_escalado)+dominio_anual</f>
+        <v>2403</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="s">
+        <v>276</v>
+      </c>
+      <c r="C50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>262.8</v>
+      </c>
+      <c r="D50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,D$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>4380</v>
+      </c>
+      <c r="E50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,E$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>4380</v>
+      </c>
+      <c r="F50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,F$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>4380</v>
+      </c>
+      <c r="G50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,G$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>4380</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="s">
+        <v>277</v>
+      </c>
+      <c r="C51" s="0" t="n">
+        <f aca="false">INDEX(marketing,C$3,$B$2)</f>
+        <v>6000</v>
+      </c>
+      <c r="D51" s="0" t="n">
+        <f aca="false">INDEX(marketing,D$3,$B$2)</f>
+        <v>9000</v>
+      </c>
+      <c r="E51" s="0" t="n">
+        <f aca="false">INDEX(marketing,E$3,$B$2)</f>
+        <v>12000</v>
+      </c>
+      <c r="F51" s="0" t="n">
+        <f aca="false">INDEX(marketing,F$3,$B$2)</f>
+        <v>15000</v>
+      </c>
+      <c r="G51" s="0" t="n">
+        <f aca="false">INDEX(marketing,G$3,$B$2)</f>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="B52" s="0" t="n">
+        <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
+        <v>1573</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="C53" s="0" t="n">
+        <f aca="false">C7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>10704.96</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <f aca="false">D7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>42819.84</v>
+      </c>
+      <c r="E53" s="0" t="n">
+        <f aca="false">E7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>107049.6</v>
+      </c>
+      <c r="F53" s="0" t="n">
+        <f aca="false">F7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>214099.2</v>
+      </c>
+      <c r="G53" s="0" t="n">
+        <f aca="false">G7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>321148.8</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="C54" s="0" t="n">
+        <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>9634.464</v>
+      </c>
+      <c r="D54" s="0" t="n">
+        <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>27618.7968</v>
+      </c>
+      <c r="E54" s="0" t="n">
+        <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>40892.9472</v>
+      </c>
+      <c r="F54" s="0" t="n">
+        <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>49456.9152</v>
+      </c>
+      <c r="G54" s="0" t="n">
+        <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>55558.7424</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="s">
+        <v>281</v>
+      </c>
+      <c r="B55" s="0" t="n">
+        <f aca="false">SUM(B48:B54)</f>
+        <v>21132.6666666667</v>
+      </c>
+      <c r="C55" s="0" t="n">
+        <f aca="false">SUM(C48:C54)</f>
+        <v>51698.724</v>
+      </c>
+      <c r="D55" s="0" t="n">
+        <f aca="false">SUM(D48:D54)</f>
+        <v>110316.8118</v>
+      </c>
+      <c r="E55" s="0" t="n">
+        <f aca="false">SUM(E48:E54)</f>
+        <v>192463.48095</v>
+      </c>
+      <c r="F55" s="0" t="n">
+        <f aca="false">SUM(F48:F54)</f>
+        <v>313023.9456375</v>
+      </c>
+      <c r="G55" s="0" t="n">
+        <f aca="false">SUM(G48:G54)</f>
+        <v>431189.614359375</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="s">
+        <v>283</v>
+      </c>
+      <c r="B58" s="0" t="n">
+        <f aca="false">B45-B55</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C58" s="0" t="n">
+        <f aca="false">C45-C55</f>
+        <v>203301.276</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <f aca="false">D45-D55</f>
+        <v>363083.1882</v>
+      </c>
+      <c r="E58" s="0" t="n">
+        <f aca="false">E45-E55</f>
+        <v>598936.51905</v>
+      </c>
+      <c r="F58" s="0" t="n">
+        <f aca="false">F45-F55</f>
+        <v>535976.0543625</v>
+      </c>
+      <c r="G58" s="0" t="n">
+        <f aca="false">G45-G55</f>
+        <v>614610.385640625</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="s">
+        <v>284</v>
+      </c>
+      <c r="B59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^B$3</f>
+        <v>1</v>
+      </c>
+      <c r="C59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^C$3</f>
+        <v>0.8</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^D$3</f>
+        <v>0.64</v>
+      </c>
+      <c r="E59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^E$3</f>
+        <v>0.512</v>
+      </c>
+      <c r="F59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^F$3</f>
+        <v>0.4096</v>
+      </c>
+      <c r="G59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^G$3</f>
+        <v>0.32768</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="s">
+        <v>285</v>
+      </c>
+      <c r="B60" s="0" t="n">
+        <f aca="false">B58*B59</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C60" s="0" t="n">
+        <f aca="false">C58*C59</f>
+        <v>162641.0208</v>
+      </c>
+      <c r="D60" s="0" t="n">
+        <f aca="false">D58*D59</f>
+        <v>232373.240448</v>
+      </c>
+      <c r="E60" s="0" t="n">
+        <f aca="false">E58*E59</f>
+        <v>306655.4977536</v>
+      </c>
+      <c r="F60" s="0" t="n">
+        <f aca="false">F58*F59</f>
+        <v>219535.79186688</v>
+      </c>
+      <c r="G60" s="0" t="n">
+        <f aca="false">G58*G59</f>
+        <v>201395.53116672</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="s">
+        <v>286</v>
+      </c>
+      <c r="B61" s="0" t="n">
+        <f aca="false">B58</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C61" s="0" t="n">
+        <f aca="false">B61+C58</f>
+        <v>182168.609333333</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <f aca="false">C61+D58</f>
+        <v>545251.797533333</v>
+      </c>
+      <c r="E61" s="0" t="n">
+        <f aca="false">D61+E58</f>
+        <v>1144188.31658333</v>
+      </c>
+      <c r="F61" s="0" t="n">
+        <f aca="false">E61+F58</f>
+        <v>1680164.37094583</v>
+      </c>
+      <c r="G61" s="0" t="n">
+        <f aca="false">F61+G58</f>
+        <v>2294774.75658646</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="s">
+        <v>287</v>
+      </c>
+      <c r="B62" s="0" t="n">
+        <f aca="false">B60</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C62" s="0" t="n">
+        <f aca="false">B62+C60</f>
+        <v>141508.354133333</v>
+      </c>
+      <c r="D62" s="0" t="n">
+        <f aca="false">C62+D60</f>
+        <v>373881.594581333</v>
+      </c>
+      <c r="E62" s="0" t="n">
+        <f aca="false">D62+E60</f>
+        <v>680537.092334933</v>
+      </c>
+      <c r="F62" s="0" t="n">
+        <f aca="false">E62+F60</f>
+        <v>900072.884201813</v>
+      </c>
+      <c r="G62" s="0" t="n">
+        <f aca="false">F62+G60</f>
+        <v>1101468.41536853</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="C63" s="0" t="n">
+        <f aca="false">IF(AND(B61&lt;0,C61&gt;=0),C$3-1+(-B61)/C58,"")</f>
+        <v>0.103947535807236</v>
+      </c>
+      <c r="D63" s="0" t="str">
+        <f aca="false">IF(AND(C61&lt;0,D61&gt;=0),D$3-1+(-C61)/D58,"")</f>
+        <v/>
+      </c>
+      <c r="E63" s="0" t="str">
+        <f aca="false">IF(AND(D61&lt;0,E61&gt;=0),E$3-1+(-D61)/E58,"")</f>
+        <v/>
+      </c>
+      <c r="F63" s="0" t="str">
+        <f aca="false">IF(AND(E61&lt;0,F61&gt;=0),F$3-1+(-E61)/F58,"")</f>
+        <v/>
+      </c>
+      <c r="G63" s="0" t="str">
+        <f aca="false">IF(AND(F61&lt;0,G61&gt;=0),G$3-1+(-F61)/G58,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>289</v>
+      </c>
+      <c r="C64" s="0" t="n">
+        <f aca="false">IF(AND(B62&lt;0,C62&gt;=0),C$3-1+(-B62)/C60,"")</f>
+        <v>0.129934419759044</v>
+      </c>
+      <c r="D64" s="0" t="str">
+        <f aca="false">IF(AND(C62&lt;0,D62&gt;=0),D$3-1+(-C62)/D60,"")</f>
+        <v/>
+      </c>
+      <c r="E64" s="0" t="str">
+        <f aca="false">IF(AND(D62&lt;0,E62&gt;=0),E$3-1+(-D62)/E60,"")</f>
+        <v/>
+      </c>
+      <c r="F64" s="0" t="str">
+        <f aca="false">IF(AND(E62&lt;0,F62&gt;=0),F$3-1+(-E62)/F60,"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="0" t="str">
+        <f aca="false">IF(AND(F62&lt;0,G62&gt;=0),G$3-1+(-F62)/G60,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="B67" s="0" t="n">
+        <f aca="false">SUM(B60:G60)</f>
+        <v>1101468.41536853</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="B68" s="2" t="n">
+        <f aca="false">IFERROR(IRR(B58:G58),"no definida")</f>
+        <v>10.3696253055461</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="s">
         <v>227</v>
+      </c>
+      <c r="B69" s="0" t="n">
+        <f aca="false">IF(COUNT(C63:G63)=0,"no se recupera",MIN(C63:G63))</f>
+        <v>0.103947535807236</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="B70" s="0" t="n">
+        <f aca="false">IF(COUNT(C64:G64)=0,"no se recupera",MIN(C64:G64))</f>
+        <v>0.129934419759044</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="B71" s="0" t="n">
+        <f aca="false">IFERROR(G45/G36,"no definido")</f>
+        <v>10781.4432989691</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="B72" s="0" t="n">
+        <f aca="false">IFERROR(ROUNDUP(G55/B71,0),"no definido")</f>
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>0</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>2</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>3</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>4</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <f aca="false">anio_0+B$3</f>
+        <v>2026</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">anio_0+C$3</f>
+        <v>2027</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <f aca="false">anio_0+D$3</f>
+        <v>2028</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <f aca="false">anio_0+E$3</f>
+        <v>2029</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <f aca="false">anio_0+F$3</f>
+        <v>2030</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <f aca="false">anio_0+G$3</f>
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,B$3+1)</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,C$3+1)</f>
+        <v>1</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,D$3+1)</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,E$3+1)</f>
+        <v>1</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,F$3+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,G$3+1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <f aca="false">IF(C$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <f aca="false">IF(D$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <f aca="false">IF(E$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <f aca="false">IF(F$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <f aca="false">IF(G$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>237</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -3196,7 +4855,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -3221,7 +4880,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -3246,7 +4905,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-C10),0)</f>
@@ -3271,7 +4930,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -3296,7 +4955,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -3321,7 +4980,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -3346,7 +5005,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -3371,7 +5030,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-C15),0)</f>
@@ -3396,7 +5055,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -3421,7 +5080,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -3446,7 +5105,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -3471,7 +5130,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -3496,7 +5155,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-C20),0)</f>
@@ -3521,7 +5180,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -3546,7 +5205,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -3571,7 +5230,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -3596,7 +5255,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -3621,7 +5280,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-C25),0)</f>
@@ -3646,7 +5305,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -3671,7 +5330,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -3696,7 +5355,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -3721,7 +5380,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -3746,7 +5405,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-C30),0)</f>
@@ -3771,7 +5430,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -3796,7 +5455,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -3821,7 +5480,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
@@ -3846,7 +5505,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -3871,12 +5530,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
@@ -3901,7 +5560,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*meses_anio</f>
@@ -3926,7 +5585,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*meses_anio</f>
@@ -3951,7 +5610,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*meses_anio</f>
@@ -3976,7 +5635,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
@@ -4001,7 +5660,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)</f>
@@ -4026,7 +5685,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -4055,12 +5714,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="B48" s="0" t="n">
         <f aca="false">meses_anio_0*sueldo_usd*sueldos_por_anio/meses_anio</f>
@@ -4089,7 +5748,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -4118,7 +5777,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -4143,7 +5802,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -4168,7 +5827,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -4177,7 +5836,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="C53" s="0" t="n">
         <f aca="false">C7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
@@ -4202,7 +5861,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
@@ -4227,7 +5886,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -4256,12 +5915,12 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -4290,7 +5949,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -4319,7 +5978,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">B58*B59</f>
@@ -4348,7 +6007,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B58</f>
@@ -4377,7 +6036,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B60</f>
@@ -4406,7 +6065,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="C63" s="0" t="str">
         <f aca="false">IF(AND(B61&lt;0,C61&gt;=0),C$3-1+(-B61)/C58,"")</f>
@@ -4431,7 +6090,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="C64" s="0" t="str">
         <f aca="false">IF(AND(B62&lt;0,C62&gt;=0),C$3-1+(-B62)/C60,"")</f>
@@ -4456,12 +6115,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>281</v>
+        <v>225</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">SUM(B60:G60)</f>
@@ -4470,7 +6129,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>282</v>
+        <v>226</v>
       </c>
       <c r="B68" s="2" t="n">
         <f aca="false">IFERROR(IRR(B58:G58),"no definida")</f>
@@ -4479,7 +6138,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>283</v>
+        <v>227</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">IF(COUNT(C63:G63)=0,"no se recupera",MIN(C63:G63))</f>
@@ -4488,7 +6147,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>284</v>
+        <v>228</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">IF(COUNT(C64:G64)=0,"no se recupera",MIN(C64:G64))</f>
@@ -4497,7 +6156,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>285</v>
+        <v>230</v>
       </c>
       <c r="B71" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -4506,11 +6165,1511 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>286</v>
+        <v>229</v>
       </c>
       <c r="B72" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B71,0),"no definido")</f>
         <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>0</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>2</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>3</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>4</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <f aca="false">COLUMN()-2</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <f aca="false">anio_0+B$3</f>
+        <v>2026</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <f aca="false">anio_0+C$3</f>
+        <v>2027</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <f aca="false">anio_0+D$3</f>
+        <v>2028</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <f aca="false">anio_0+E$3</f>
+        <v>2029</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <f aca="false">anio_0+F$3</f>
+        <v>2030</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <f aca="false">anio_0+G$3</f>
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>235</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,B$3+1)</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,C$3+1)</f>
+        <v>1</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,D$3+1)</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,E$3+1)</f>
+        <v>1</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,F$3+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <f aca="false">INDEX(anio_electoral,G$3+1)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <f aca="false">IF(C$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <f aca="false">IF(D$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <f aca="false">IF(E$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <f aca="false">IF(F$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <f aca="false">IF(G$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
+        <v>500</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,D$3,$B$2)</f>
+        <v>2000</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,E$3,$B$2)</f>
+        <v>5000</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,F$3,$B$2)</f>
+        <v>8000</v>
+      </c>
+      <c r="G7" s="0" t="n">
+        <f aca="false">INDEX(usuarios_activos,G$3,$B$2)</f>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <f aca="false">N(B13)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <f aca="false">N(C13)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <f aca="false">N(D13)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <f aca="false">N(E13)</f>
+        <v>1</v>
+      </c>
+      <c r="G10" s="0" t="n">
+        <f aca="false">N(F13)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*D10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*E10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*F10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*G10,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>240</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-C10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-D10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-E10),0)</f>
+        <v>1</v>
+      </c>
+      <c r="F12" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-F10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-G10),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <f aca="false">C10+C12-C11</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <f aca="false">D10+D12-D11</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <f aca="false">E10+E12-E11</f>
+        <v>1</v>
+      </c>
+      <c r="F13" s="0" t="n">
+        <f aca="false">F10+F12-F11</f>
+        <v>1</v>
+      </c>
+      <c r="G13" s="0" t="n">
+        <f aca="false">G10+G12-G11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>242</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <f aca="false">(C10+C13)/2</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <f aca="false">(D10+D13)/2</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <f aca="false">(E10+E13)/2</f>
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="0" t="n">
+        <f aca="false">(F10+F13)/2</f>
+        <v>1</v>
+      </c>
+      <c r="G14" s="0" t="n">
+        <f aca="false">(G10+G13)/2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <f aca="false">N(B18)</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <f aca="false">N(C18)</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="0" t="n">
+        <f aca="false">N(D18)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="0" t="n">
+        <f aca="false">N(E18)</f>
+        <v>2</v>
+      </c>
+      <c r="G15" s="0" t="n">
+        <f aca="false">N(F18)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*D15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*E15,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*F15,0)</f>
+        <v>1</v>
+      </c>
+      <c r="G16" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*G15,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-C15),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-D15),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-E15),0)</f>
+        <v>2</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-F15),0)</f>
+        <v>2</v>
+      </c>
+      <c r="G17" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-G15),0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <f aca="false">C15+C17-C16</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <f aca="false">D15+D17-D16</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <f aca="false">E15+E17-E16</f>
+        <v>2</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <f aca="false">F15+F17-F16</f>
+        <v>3</v>
+      </c>
+      <c r="G18" s="0" t="n">
+        <f aca="false">G15+G17-G16</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <f aca="false">(C15+C18)/2</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <f aca="false">(D15+D18)/2</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <f aca="false">(E15+E18)/2</f>
+        <v>1</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <f aca="false">(F15+F18)/2</f>
+        <v>2.5</v>
+      </c>
+      <c r="G19" s="0" t="n">
+        <f aca="false">(G15+G18)/2</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <f aca="false">N(B23)</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <f aca="false">N(C23)</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="0" t="n">
+        <f aca="false">N(D23)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="0" t="n">
+        <f aca="false">N(E23)</f>
+        <v>1</v>
+      </c>
+      <c r="G20" s="0" t="n">
+        <f aca="false">N(F23)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>249</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*D20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*E20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*F20,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*G20,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>250</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-C20),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-D20),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-E20),0)</f>
+        <v>1</v>
+      </c>
+      <c r="F22" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-F20),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-G20),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <f aca="false">C20+C22-C21</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <f aca="false">D20+D22-D21</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="0" t="n">
+        <f aca="false">E20+E22-E21</f>
+        <v>1</v>
+      </c>
+      <c r="F23" s="0" t="n">
+        <f aca="false">F20+F22-F21</f>
+        <v>1</v>
+      </c>
+      <c r="G23" s="0" t="n">
+        <f aca="false">G20+G22-G21</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <f aca="false">(C20+C23)/2</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <f aca="false">(D20+D23)/2</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="0" t="n">
+        <f aca="false">(E20+E23)/2</f>
+        <v>0.5</v>
+      </c>
+      <c r="F24" s="0" t="n">
+        <f aca="false">(F20+F23)/2</f>
+        <v>1</v>
+      </c>
+      <c r="G24" s="0" t="n">
+        <f aca="false">(G20+G23)/2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <f aca="false">N(B28)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <f aca="false">N(C28)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="0" t="n">
+        <f aca="false">N(D28)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="0" t="n">
+        <f aca="false">N(E28)</f>
+        <v>3</v>
+      </c>
+      <c r="G25" s="0" t="n">
+        <f aca="false">N(F28)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="C26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*D25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*E25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*F25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*G25,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>255</v>
+      </c>
+      <c r="C27" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-C25),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-D25),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-E25),0)</f>
+        <v>3</v>
+      </c>
+      <c r="F27" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-F25),0)</f>
+        <v>3</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-G25),0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <f aca="false">C25+C27-C26</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <f aca="false">D25+D27-D26</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <f aca="false">E25+E27-E26</f>
+        <v>3</v>
+      </c>
+      <c r="F28" s="0" t="n">
+        <f aca="false">F25+F27-F26</f>
+        <v>6</v>
+      </c>
+      <c r="G28" s="0" t="n">
+        <f aca="false">G25+G27-G26</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="C29" s="0" t="n">
+        <f aca="false">(C25+C28)/2</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="0" t="n">
+        <f aca="false">(D25+D28)/2</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="0" t="n">
+        <f aca="false">(E25+E28)/2</f>
+        <v>1.5</v>
+      </c>
+      <c r="F29" s="0" t="n">
+        <f aca="false">(F25+F28)/2</f>
+        <v>4.5</v>
+      </c>
+      <c r="G29" s="0" t="n">
+        <f aca="false">(G25+G28)/2</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <f aca="false">N(B33)</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="0" t="n">
+        <f aca="false">N(C33)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="0" t="n">
+        <f aca="false">N(D33)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="0" t="n">
+        <f aca="false">N(E33)</f>
+        <v>1</v>
+      </c>
+      <c r="G30" s="0" t="n">
+        <f aca="false">N(F33)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*D30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*E30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*F30,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="0" t="n">
+        <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*G30,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="C32" s="0" t="n">
+        <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-C30),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="0" t="n">
+        <f aca="false">D6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-D30),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="0" t="n">
+        <f aca="false">E6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-E30),0)</f>
+        <v>1</v>
+      </c>
+      <c r="F32" s="0" t="n">
+        <f aca="false">F6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-F30),0)</f>
+        <v>1</v>
+      </c>
+      <c r="G32" s="0" t="n">
+        <f aca="false">G6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-G30),0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="C33" s="0" t="n">
+        <f aca="false">C30+C32-C31</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="0" t="n">
+        <f aca="false">D30+D32-D31</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="0" t="n">
+        <f aca="false">E30+E32-E31</f>
+        <v>1</v>
+      </c>
+      <c r="F33" s="0" t="n">
+        <f aca="false">F30+F32-F31</f>
+        <v>2</v>
+      </c>
+      <c r="G33" s="0" t="n">
+        <f aca="false">G30+G32-G31</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="C34" s="0" t="n">
+        <f aca="false">(C30+C33)/2</f>
+        <v>0</v>
+      </c>
+      <c r="D34" s="0" t="n">
+        <f aca="false">(D30+D33)/2</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <f aca="false">(E30+E33)/2</f>
+        <v>0.5</v>
+      </c>
+      <c r="F34" s="0" t="n">
+        <f aca="false">(F30+F33)/2</f>
+        <v>1.5</v>
+      </c>
+      <c r="G34" s="0" t="n">
+        <f aca="false">(G30+G33)/2</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="C35" s="0" t="n">
+        <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D35" s="0" t="n">
+        <f aca="false">D5*D6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="0" t="n">
+        <f aca="false">E5*E6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F35" s="0" t="n">
+        <f aca="false">F5*F6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="0" t="n">
+        <f aca="false">G5*G6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="C36" s="0" t="n">
+        <f aca="false">C14+C19+C24+C29+C34+C35</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="0" t="n">
+        <f aca="false">D14+D19+D24+D29+D34+D35</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="0" t="n">
+        <f aca="false">E14+E19+E24+E29+E34+E35</f>
+        <v>5</v>
+      </c>
+      <c r="F36" s="0" t="n">
+        <f aca="false">F14+F19+F24+F29+F34+F35</f>
+        <v>10.5</v>
+      </c>
+      <c r="G36" s="0" t="n">
+        <f aca="false">G14+G19+G24+G29+G34+G35</f>
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="C39" s="0" t="n">
+        <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="0" t="n">
+        <f aca="false">D14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="0" t="n">
+        <f aca="false">E14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>9000</v>
+      </c>
+      <c r="F39" s="0" t="n">
+        <f aca="false">F14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>18000</v>
+      </c>
+      <c r="G39" s="0" t="n">
+        <f aca="false">G14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="C40" s="0" t="n">
+        <f aca="false">C19*precio_medios_chicos*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <f aca="false">D19*precio_medios_chicos*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="0" t="n">
+        <f aca="false">E19*precio_medios_chicos*meses_anio</f>
+        <v>2400</v>
+      </c>
+      <c r="F40" s="0" t="n">
+        <f aca="false">F19*precio_medios_chicos*meses_anio</f>
+        <v>6000</v>
+      </c>
+      <c r="G40" s="0" t="n">
+        <f aca="false">G19*precio_medios_chicos*meses_anio</f>
+        <v>8400</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="C41" s="0" t="n">
+        <f aca="false">C24*precio_verificadores*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <f aca="false">D24*precio_verificadores*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="0" t="n">
+        <f aca="false">E24*precio_verificadores*meses_anio</f>
+        <v>3000</v>
+      </c>
+      <c r="F41" s="0" t="n">
+        <f aca="false">F24*precio_verificadores*meses_anio</f>
+        <v>6000</v>
+      </c>
+      <c r="G41" s="0" t="n">
+        <f aca="false">G24*precio_verificadores*meses_anio</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="C42" s="0" t="n">
+        <f aca="false">C29*precio_universidades*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <f aca="false">D29*precio_universidades*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <f aca="false">E29*precio_universidades*meses_anio</f>
+        <v>1800</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <f aca="false">F29*precio_universidades*meses_anio</f>
+        <v>5400</v>
+      </c>
+      <c r="G42" s="0" t="n">
+        <f aca="false">G29*precio_universidades*meses_anio</f>
+        <v>8400</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="C43" s="0" t="n">
+        <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <f aca="false">D34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="0" t="n">
+        <f aca="false">E34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>9000</v>
+      </c>
+      <c r="F43" s="0" t="n">
+        <f aca="false">F34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>27000</v>
+      </c>
+      <c r="G43" s="0" t="n">
+        <f aca="false">G34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="C44" s="0" t="n">
+        <f aca="false">C35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="D44" s="0" t="n">
+        <f aca="false">D35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="0" t="n">
+        <f aca="false">E35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>10000</v>
+      </c>
+      <c r="F44" s="0" t="n">
+        <f aca="false">F35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="0" t="n">
+        <f aca="false">G35*INDEX(precio_organismos,1,$B$2)</f>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="B45" s="0" t="n">
+        <f aca="false">SUM(B39:B44)</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <f aca="false">SUM(C39:C44)</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <f aca="false">SUM(D39:D44)</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <f aca="false">SUM(E39:E44)</f>
+        <v>35200</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <f aca="false">SUM(F39:F44)</f>
+        <v>62400</v>
+      </c>
+      <c r="G45" s="0" t="n">
+        <f aca="false">SUM(G39:G44)</f>
+        <v>86800</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="B48" s="0" t="n">
+        <f aca="false">meses_anio_0*sueldo_usd*sueldos_por_anio/meses_anio</f>
+        <v>19391.6666666667</v>
+      </c>
+      <c r="C48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^C$3</f>
+        <v>24433.5</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^D$3</f>
+        <v>25655.175</v>
+      </c>
+      <c r="E48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^E$3</f>
+        <v>26937.93375</v>
+      </c>
+      <c r="F48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^F$3</f>
+        <v>28284.8304375</v>
+      </c>
+      <c r="G48" s="0" t="n">
+        <f aca="false">sueldo_usd*sueldos_por_anio*(1+ajuste_sueldo)^G$3</f>
+        <v>29699.071959375</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="B49" s="0" t="n">
+        <f aca="false">inv_infraestructura_0</f>
+        <v>168</v>
+      </c>
+      <c r="C49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*C7/ua_escalado)+dominio_anual</f>
+        <v>609</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*D7/ua_escalado)+dominio_anual</f>
+        <v>627</v>
+      </c>
+      <c r="E49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*E7/ua_escalado)+dominio_anual</f>
+        <v>663</v>
+      </c>
+      <c r="F49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*F7/ua_escalado)+dominio_anual</f>
+        <v>699</v>
+      </c>
+      <c r="G49" s="0" t="n">
+        <f aca="false">meses_anio*(infra_base+infra_escalado*G7/ua_escalado)+dominio_anual</f>
+        <v>723</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="s">
+        <v>276</v>
+      </c>
+      <c r="C50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>262.8</v>
+      </c>
+      <c r="D50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,D$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>262.8</v>
+      </c>
+      <c r="E50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,E$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>262.8</v>
+      </c>
+      <c r="F50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,F$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>262.8</v>
+      </c>
+      <c r="G50" s="0" t="n">
+        <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,G$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
+        <v>262.8</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="s">
+        <v>277</v>
+      </c>
+      <c r="C51" s="0" t="n">
+        <f aca="false">INDEX(marketing,C$3,$B$2)</f>
+        <v>2000</v>
+      </c>
+      <c r="D51" s="0" t="n">
+        <f aca="false">INDEX(marketing,D$3,$B$2)</f>
+        <v>3000</v>
+      </c>
+      <c r="E51" s="0" t="n">
+        <f aca="false">INDEX(marketing,E$3,$B$2)</f>
+        <v>4000</v>
+      </c>
+      <c r="F51" s="0" t="n">
+        <f aca="false">INDEX(marketing,F$3,$B$2)</f>
+        <v>5000</v>
+      </c>
+      <c r="G51" s="0" t="n">
+        <f aca="false">INDEX(marketing,G$3,$B$2)</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="B52" s="0" t="n">
+        <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
+        <v>1573</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="C53" s="0" t="n">
+        <f aca="false">C7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>1230.0336</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <f aca="false">D7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>4920.1344</v>
+      </c>
+      <c r="E53" s="0" t="n">
+        <f aca="false">E7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>12300.336</v>
+      </c>
+      <c r="F53" s="0" t="n">
+        <f aca="false">F7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>19680.5376</v>
+      </c>
+      <c r="G53" s="0" t="n">
+        <f aca="false">G7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>24600.672</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="C54" s="0" t="n">
+        <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="0" t="n">
+        <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>0</v>
+      </c>
+      <c r="E54" s="0" t="n">
+        <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>37721.0304</v>
+      </c>
+      <c r="F54" s="0" t="n">
+        <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>93482.5536</v>
+      </c>
+      <c r="G54" s="0" t="n">
+        <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <v>113163.0912</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="s">
+        <v>281</v>
+      </c>
+      <c r="B55" s="0" t="n">
+        <f aca="false">SUM(B48:B54)</f>
+        <v>21132.6666666667</v>
+      </c>
+      <c r="C55" s="0" t="n">
+        <f aca="false">SUM(C48:C54)</f>
+        <v>28535.3336</v>
+      </c>
+      <c r="D55" s="0" t="n">
+        <f aca="false">SUM(D48:D54)</f>
+        <v>34465.1094</v>
+      </c>
+      <c r="E55" s="0" t="n">
+        <f aca="false">SUM(E48:E54)</f>
+        <v>81885.10015</v>
+      </c>
+      <c r="F55" s="0" t="n">
+        <f aca="false">SUM(F48:F54)</f>
+        <v>147409.7216375</v>
+      </c>
+      <c r="G55" s="0" t="n">
+        <f aca="false">SUM(G48:G54)</f>
+        <v>174448.635159375</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="s">
+        <v>283</v>
+      </c>
+      <c r="B58" s="0" t="n">
+        <f aca="false">B45-B55</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C58" s="0" t="n">
+        <f aca="false">C45-C55</f>
+        <v>-28535.3336</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <f aca="false">D45-D55</f>
+        <v>-34465.1094</v>
+      </c>
+      <c r="E58" s="0" t="n">
+        <f aca="false">E45-E55</f>
+        <v>-46685.10015</v>
+      </c>
+      <c r="F58" s="0" t="n">
+        <f aca="false">F45-F55</f>
+        <v>-85009.7216375</v>
+      </c>
+      <c r="G58" s="0" t="n">
+        <f aca="false">G45-G55</f>
+        <v>-87648.635159375</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="s">
+        <v>284</v>
+      </c>
+      <c r="B59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^B$3</f>
+        <v>1</v>
+      </c>
+      <c r="C59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^C$3</f>
+        <v>0.8</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^D$3</f>
+        <v>0.64</v>
+      </c>
+      <c r="E59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^E$3</f>
+        <v>0.512</v>
+      </c>
+      <c r="F59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^F$3</f>
+        <v>0.4096</v>
+      </c>
+      <c r="G59" s="0" t="n">
+        <f aca="false">1/(1+tasa_descuento)^G$3</f>
+        <v>0.32768</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0" t="s">
+        <v>285</v>
+      </c>
+      <c r="B60" s="0" t="n">
+        <f aca="false">B58*B59</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C60" s="0" t="n">
+        <f aca="false">C58*C59</f>
+        <v>-22828.26688</v>
+      </c>
+      <c r="D60" s="0" t="n">
+        <f aca="false">D58*D59</f>
+        <v>-22057.670016</v>
+      </c>
+      <c r="E60" s="0" t="n">
+        <f aca="false">E58*E59</f>
+        <v>-23902.7712768</v>
+      </c>
+      <c r="F60" s="0" t="n">
+        <f aca="false">F58*F59</f>
+        <v>-34819.98198272</v>
+      </c>
+      <c r="G60" s="0" t="n">
+        <f aca="false">G58*G59</f>
+        <v>-28720.704769024</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0" t="s">
+        <v>286</v>
+      </c>
+      <c r="B61" s="0" t="n">
+        <f aca="false">B58</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C61" s="0" t="n">
+        <f aca="false">B61+C58</f>
+        <v>-49668.0002666667</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <f aca="false">C61+D58</f>
+        <v>-84133.1096666667</v>
+      </c>
+      <c r="E61" s="0" t="n">
+        <f aca="false">D61+E58</f>
+        <v>-130818.209816667</v>
+      </c>
+      <c r="F61" s="0" t="n">
+        <f aca="false">E61+F58</f>
+        <v>-215827.931454167</v>
+      </c>
+      <c r="G61" s="0" t="n">
+        <f aca="false">F61+G58</f>
+        <v>-303476.566613542</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0" t="s">
+        <v>287</v>
+      </c>
+      <c r="B62" s="0" t="n">
+        <f aca="false">B60</f>
+        <v>-21132.6666666667</v>
+      </c>
+      <c r="C62" s="0" t="n">
+        <f aca="false">B62+C60</f>
+        <v>-43960.9335466667</v>
+      </c>
+      <c r="D62" s="0" t="n">
+        <f aca="false">C62+D60</f>
+        <v>-66018.6035626667</v>
+      </c>
+      <c r="E62" s="0" t="n">
+        <f aca="false">D62+E60</f>
+        <v>-89921.3748394667</v>
+      </c>
+      <c r="F62" s="0" t="n">
+        <f aca="false">E62+F60</f>
+        <v>-124741.356822187</v>
+      </c>
+      <c r="G62" s="0" t="n">
+        <f aca="false">F62+G60</f>
+        <v>-153462.061591211</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="C63" s="0" t="str">
+        <f aca="false">IF(AND(B61&lt;0,C61&gt;=0),C$3-1+(-B61)/C58,"")</f>
+        <v/>
+      </c>
+      <c r="D63" s="0" t="str">
+        <f aca="false">IF(AND(C61&lt;0,D61&gt;=0),D$3-1+(-C61)/D58,"")</f>
+        <v/>
+      </c>
+      <c r="E63" s="0" t="str">
+        <f aca="false">IF(AND(D61&lt;0,E61&gt;=0),E$3-1+(-D61)/E58,"")</f>
+        <v/>
+      </c>
+      <c r="F63" s="0" t="str">
+        <f aca="false">IF(AND(E61&lt;0,F61&gt;=0),F$3-1+(-E61)/F58,"")</f>
+        <v/>
+      </c>
+      <c r="G63" s="0" t="str">
+        <f aca="false">IF(AND(F61&lt;0,G61&gt;=0),G$3-1+(-F61)/G58,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="0" t="s">
+        <v>289</v>
+      </c>
+      <c r="C64" s="0" t="str">
+        <f aca="false">IF(AND(B62&lt;0,C62&gt;=0),C$3-1+(-B62)/C60,"")</f>
+        <v/>
+      </c>
+      <c r="D64" s="0" t="str">
+        <f aca="false">IF(AND(C62&lt;0,D62&gt;=0),D$3-1+(-C62)/D60,"")</f>
+        <v/>
+      </c>
+      <c r="E64" s="0" t="str">
+        <f aca="false">IF(AND(D62&lt;0,E62&gt;=0),E$3-1+(-D62)/E60,"")</f>
+        <v/>
+      </c>
+      <c r="F64" s="0" t="str">
+        <f aca="false">IF(AND(E62&lt;0,F62&gt;=0),F$3-1+(-E62)/F60,"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="0" t="str">
+        <f aca="false">IF(AND(F62&lt;0,G62&gt;=0),G$3-1+(-F62)/G60,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="B67" s="0" t="n">
+        <f aca="false">SUM(B60:G60)</f>
+        <v>-153462.061591211</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="B68" s="2" t="str">
+        <f aca="false">IFERROR(IRR(B58:G58),"no definida")</f>
+        <v>no definida</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="B69" s="0" t="str">
+        <f aca="false">IF(COUNT(C63:G63)=0,"no se recupera",MIN(C63:G63))</f>
+        <v>no se recupera</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="B70" s="0" t="str">
+        <f aca="false">IF(COUNT(C64:G64)=0,"no se recupera",MIN(C64:G64))</f>
+        <v>no se recupera</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="B71" s="0" t="n">
+        <f aca="false">IFERROR(G45/G36,"no definido")</f>
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="B72" s="0" t="n">
+        <f aca="false">IFERROR(ROUNDUP(G55/B71,0),"no definido")</f>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aplicar el tope diario al costo variable y validar los argumentos del script
- El costo variable de los usuarios gratuitos usa
  MIN(analisis_por_ua_mes, tope_diario × dias_mes); con los supuestos
  actuales el tope no restringe y los resultados no cambian.
- validar_modelo_financiero.py parsea con argparse: --help y los flags
  desconocidos ya no corren la validación ni reescriben tablas, y
  --planilla sin valor no termina en IndexError. Test nuevo.

Refs #51, #53

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -19,22 +19,23 @@
     <definedName function="false" hidden="false" name="analisis_por_ua_mes" vbProcedure="false">Supuestos!$E$70:$G$70</definedName>
     <definedName function="false" hidden="false" name="anio_0" vbProcedure="false">Supuestos!$D$6</definedName>
     <definedName function="false" hidden="false" name="anio_electoral" vbProcedure="false">Supuestos!$D$8:$D$13</definedName>
-    <definedName function="false" hidden="false" name="anio_inicio_b2b" vbProcedure="false">Supuestos!$E$89:$G$89</definedName>
+    <definedName function="false" hidden="false" name="anio_inicio_b2b" vbProcedure="false">Supuestos!$E$90:$G$90</definedName>
     <definedName function="false" hidden="false" name="busquedas" vbProcedure="false">Supuestos!$E$63:$G$63</definedName>
-    <definedName function="false" hidden="false" name="capt_agencias" vbProcedure="false">Supuestos!$E$95:$G$95</definedName>
-    <definedName function="false" hidden="false" name="capt_medios_chicos" vbProcedure="false">Supuestos!$E$91:$G$91</definedName>
-    <definedName function="false" hidden="false" name="capt_medios_grandes" vbProcedure="false">Supuestos!$E$90:$G$90</definedName>
-    <definedName function="false" hidden="false" name="capt_organismos" vbProcedure="false">Supuestos!$E$94:$G$94</definedName>
-    <definedName function="false" hidden="false" name="capt_universidades" vbProcedure="false">Supuestos!$E$93:$G$93</definedName>
-    <definedName function="false" hidden="false" name="capt_verificadores" vbProcedure="false">Supuestos!$E$92:$G$92</definedName>
-    <definedName function="false" hidden="false" name="churn_agencias" vbProcedure="false">Supuestos!$E$100:$G$100</definedName>
-    <definedName function="false" hidden="false" name="churn_medios_chicos" vbProcedure="false">Supuestos!$E$97:$G$97</definedName>
-    <definedName function="false" hidden="false" name="churn_medios_grandes" vbProcedure="false">Supuestos!$E$96:$G$96</definedName>
-    <definedName function="false" hidden="false" name="churn_universidades" vbProcedure="false">Supuestos!$E$99:$G$99</definedName>
-    <definedName function="false" hidden="false" name="churn_verificadores" vbProcedure="false">Supuestos!$E$98:$G$98</definedName>
-    <definedName function="false" hidden="false" name="consultas_ent_mes" vbProcedure="false">Supuestos!$E$74:$G$74</definedName>
-    <definedName function="false" hidden="false" name="consultas_pro_mes" vbProcedure="false">Supuestos!$E$73:$G$73</definedName>
+    <definedName function="false" hidden="false" name="capt_agencias" vbProcedure="false">Supuestos!$E$96:$G$96</definedName>
+    <definedName function="false" hidden="false" name="capt_medios_chicos" vbProcedure="false">Supuestos!$E$92:$G$92</definedName>
+    <definedName function="false" hidden="false" name="capt_medios_grandes" vbProcedure="false">Supuestos!$E$91:$G$91</definedName>
+    <definedName function="false" hidden="false" name="capt_organismos" vbProcedure="false">Supuestos!$E$95:$G$95</definedName>
+    <definedName function="false" hidden="false" name="capt_universidades" vbProcedure="false">Supuestos!$E$94:$G$94</definedName>
+    <definedName function="false" hidden="false" name="capt_verificadores" vbProcedure="false">Supuestos!$E$93:$G$93</definedName>
+    <definedName function="false" hidden="false" name="churn_agencias" vbProcedure="false">Supuestos!$E$101:$G$101</definedName>
+    <definedName function="false" hidden="false" name="churn_medios_chicos" vbProcedure="false">Supuestos!$E$98:$G$98</definedName>
+    <definedName function="false" hidden="false" name="churn_medios_grandes" vbProcedure="false">Supuestos!$E$97:$G$97</definedName>
+    <definedName function="false" hidden="false" name="churn_universidades" vbProcedure="false">Supuestos!$E$100:$G$100</definedName>
+    <definedName function="false" hidden="false" name="churn_verificadores" vbProcedure="false">Supuestos!$E$99:$G$99</definedName>
+    <definedName function="false" hidden="false" name="consultas_ent_mes" vbProcedure="false">Supuestos!$E$75:$G$75</definedName>
+    <definedName function="false" hidden="false" name="consultas_pro_mes" vbProcedure="false">Supuestos!$E$74:$G$74</definedName>
     <definedName function="false" hidden="false" name="costo_analisis" vbProcedure="false">Supuestos!$E$64:$G$64</definedName>
+    <definedName function="false" hidden="false" name="dias_mes" vbProcedure="false">Supuestos!$D$72</definedName>
     <definedName function="false" hidden="false" name="dominio_anual" vbProcedure="false">Supuestos!$D$41</definedName>
     <definedName function="false" hidden="false" name="horas_anio" vbProcedure="false">Supuestos!$D$44</definedName>
     <definedName function="false" hidden="false" name="horizonte" vbProcedure="false">Supuestos!$D$5</definedName>
@@ -54,15 +55,15 @@
     <definedName function="false" hidden="false" name="marketing" vbProcedure="false">Supuestos!$E$50:$G$54</definedName>
     <definedName function="false" hidden="false" name="meses_anio" vbProcedure="false">Supuestos!$D$7</definedName>
     <definedName function="false" hidden="false" name="meses_anio_0" vbProcedure="false">Supuestos!$D$25</definedName>
-    <definedName function="false" hidden="false" name="precio_agencias" vbProcedure="false">Supuestos!$E$88:$G$88</definedName>
+    <definedName function="false" hidden="false" name="precio_agencias" vbProcedure="false">Supuestos!$E$89:$G$89</definedName>
     <definedName function="false" hidden="false" name="precio_busqueda" vbProcedure="false">Supuestos!$D$59</definedName>
     <definedName function="false" hidden="false" name="precio_entrada" vbProcedure="false">Supuestos!$D$57</definedName>
-    <definedName function="false" hidden="false" name="precio_medios_chicos" vbProcedure="false">Supuestos!$D$84</definedName>
-    <definedName function="false" hidden="false" name="precio_medios_grandes" vbProcedure="false">Supuestos!$E$83:$G$83</definedName>
-    <definedName function="false" hidden="false" name="precio_organismos" vbProcedure="false">Supuestos!$E$87:$G$87</definedName>
+    <definedName function="false" hidden="false" name="precio_medios_chicos" vbProcedure="false">Supuestos!$D$85</definedName>
+    <definedName function="false" hidden="false" name="precio_medios_grandes" vbProcedure="false">Supuestos!$E$84:$G$84</definedName>
+    <definedName function="false" hidden="false" name="precio_organismos" vbProcedure="false">Supuestos!$E$88:$G$88</definedName>
     <definedName function="false" hidden="false" name="precio_salida" vbProcedure="false">Supuestos!$D$58</definedName>
-    <definedName function="false" hidden="false" name="precio_universidades" vbProcedure="false">Supuestos!$D$86</definedName>
-    <definedName function="false" hidden="false" name="precio_verificadores" vbProcedure="false">Supuestos!$D$85</definedName>
+    <definedName function="false" hidden="false" name="precio_universidades" vbProcedure="false">Supuestos!$D$87</definedName>
+    <definedName function="false" hidden="false" name="precio_verificadores" vbProcedure="false">Supuestos!$D$86</definedName>
     <definedName function="false" hidden="false" name="prima_proyecto" vbProcedure="false">Supuestos!$D$16</definedName>
     <definedName function="false" hidden="false" name="riesgo_pais" vbProcedure="false">Supuestos!$D$15</definedName>
     <definedName function="false" hidden="false" name="sueldos_por_anio" vbProcedure="false">Supuestos!$D$23</definedName>
@@ -70,7 +71,7 @@
     <definedName function="false" hidden="false" name="sueldo_usd" vbProcedure="false">Supuestos!$D$22</definedName>
     <definedName function="false" hidden="false" name="tasa_descuento" vbProcedure="false">Supuestos!$D$17</definedName>
     <definedName function="false" hidden="false" name="tasa_libre_riesgo" vbProcedure="false">Supuestos!$D$14</definedName>
-    <definedName function="false" hidden="false" name="tasa_reuso" vbProcedure="false">Supuestos!$E$72:$G$72</definedName>
+    <definedName function="false" hidden="false" name="tasa_reuso" vbProcedure="false">Supuestos!$E$73:$G$73</definedName>
     <definedName function="false" hidden="false" name="tc_encuesta" vbProcedure="false">Supuestos!$D$21</definedName>
     <definedName function="false" hidden="false" name="tokens_entrada" vbProcedure="false">Supuestos!$E$61:$G$61</definedName>
     <definedName function="false" hidden="false" name="tokens_por_millon" vbProcedure="false">Supuestos!$D$60</definedName>
@@ -78,12 +79,12 @@
     <definedName function="false" hidden="false" name="tope_diario" vbProcedure="false">Supuestos!$D$71</definedName>
     <definedName function="false" hidden="false" name="ua_escalado" vbProcedure="false">Supuestos!$D$40</definedName>
     <definedName function="false" hidden="false" name="usuarios_activos" vbProcedure="false">Supuestos!$E$65:$G$69</definedName>
-    <definedName function="false" hidden="false" name="u_agencias" vbProcedure="false">Supuestos!$D$82</definedName>
-    <definedName function="false" hidden="false" name="u_medios_chicos" vbProcedure="false">Supuestos!$D$78</definedName>
-    <definedName function="false" hidden="false" name="u_medios_grandes" vbProcedure="false">Supuestos!$D$77</definedName>
-    <definedName function="false" hidden="false" name="u_organismos" vbProcedure="false">Supuestos!$D$81</definedName>
-    <definedName function="false" hidden="false" name="u_universidades" vbProcedure="false">Supuestos!$D$80</definedName>
-    <definedName function="false" hidden="false" name="u_verificadores" vbProcedure="false">Supuestos!$D$79</definedName>
+    <definedName function="false" hidden="false" name="u_agencias" vbProcedure="false">Supuestos!$D$83</definedName>
+    <definedName function="false" hidden="false" name="u_medios_chicos" vbProcedure="false">Supuestos!$D$79</definedName>
+    <definedName function="false" hidden="false" name="u_medios_grandes" vbProcedure="false">Supuestos!$D$78</definedName>
+    <definedName function="false" hidden="false" name="u_organismos" vbProcedure="false">Supuestos!$D$82</definedName>
+    <definedName function="false" hidden="false" name="u_universidades" vbProcedure="false">Supuestos!$D$81</definedName>
+    <definedName function="false" hidden="false" name="u_verificadores" vbProcedure="false">Supuestos!$D$80</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -95,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="296">
   <si>
     <t xml:space="preserve">clave</t>
   </si>
@@ -562,7 +563,16 @@
     <t xml:space="preserve">tope_diario</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope de análisis por usuario gratuito por día (no restrictivo)</t>
+    <t xml:space="preserve">Tope de análisis por usuario gratuito por día</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dias_mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días por mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">días</t>
   </si>
   <si>
     <t xml:space="preserve">tasa_reuso</t>
@@ -1320,7 +1330,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -2470,39 +2480,33 @@
         <v>157</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="E72" s="0" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F72" s="0" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G72" s="0" t="n">
-        <v>0.1</v>
+        <v>158</v>
+      </c>
+      <c r="D72" s="0" t="n">
+        <v>30</v>
       </c>
       <c r="H72" s="0" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>160</v>
+        <v>33</v>
       </c>
       <c r="E73" s="0" t="n">
-        <v>2000</v>
+        <v>0.3</v>
       </c>
       <c r="F73" s="0" t="n">
-        <v>4000</v>
+        <v>0.2</v>
       </c>
       <c r="G73" s="0" t="n">
-        <v>8000</v>
+        <v>0.1</v>
       </c>
       <c r="H73" s="0" t="s">
         <v>17</v>
@@ -2516,55 +2520,61 @@
         <v>162</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E74" s="0" t="n">
-        <v>20000</v>
+        <v>2000</v>
       </c>
       <c r="F74" s="0" t="n">
-        <v>40000</v>
+        <v>4000</v>
       </c>
       <c r="G74" s="0" t="n">
-        <v>80000</v>
+        <v>8000</v>
       </c>
       <c r="H74" s="0" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="1" t="s">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="B75" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="C75" s="0" t="s">
         <v>163</v>
       </c>
+      <c r="E75" s="0" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F75" s="0" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G75" s="0" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H75" s="0" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0" t="s">
-        <v>164</v>
-      </c>
-      <c r="B77" s="0" t="s">
-        <v>165</v>
-      </c>
-      <c r="C77" s="0" t="s">
+      <c r="A77" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="D77" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="H77" s="0" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="B78" s="0" t="s">
         <v>168</v>
       </c>
-      <c r="B78" s="0" t="s">
+      <c r="C78" s="0" t="s">
         <v>169</v>
       </c>
-      <c r="C78" s="0" t="s">
-        <v>166</v>
-      </c>
       <c r="D78" s="0" t="n">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="H78" s="0" t="s">
         <v>170</v>
@@ -2578,10 +2588,10 @@
         <v>172</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>3</v>
+        <v>93</v>
       </c>
       <c r="H79" s="0" t="s">
         <v>173</v>
@@ -2595,10 +2605,10 @@
         <v>175</v>
       </c>
       <c r="C80" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>149</v>
+        <v>3</v>
       </c>
       <c r="H80" s="0" t="s">
         <v>176</v>
@@ -2612,10 +2622,10 @@
         <v>178</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>32</v>
+        <v>149</v>
       </c>
       <c r="H81" s="0" t="s">
         <v>179</v>
@@ -2629,10 +2639,10 @@
         <v>181</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="H82" s="0" t="s">
         <v>182</v>
@@ -2646,16 +2656,10 @@
         <v>184</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="E83" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F83" s="0" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G83" s="0" t="n">
-        <v>1500</v>
+        <v>169</v>
+      </c>
+      <c r="D83" s="0" t="n">
+        <v>120</v>
       </c>
       <c r="H83" s="0" t="s">
         <v>185</v>
@@ -2671,68 +2675,68 @@
       <c r="C84" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="D84" s="0" t="n">
-        <v>200</v>
+      <c r="E84" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F84" s="0" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G84" s="0" t="n">
+        <v>1500</v>
       </c>
       <c r="H84" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C85" s="0" t="s">
         <v>54</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="H85" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C86" s="0" t="s">
         <v>54</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="H86" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B87" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C87" s="0" t="s">
-        <v>194</v>
-      </c>
-      <c r="E87" s="0" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F87" s="0" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G87" s="0" t="n">
-        <v>10000</v>
+        <v>54</v>
+      </c>
+      <c r="D87" s="0" t="n">
+        <v>100</v>
       </c>
       <c r="H87" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2743,62 +2747,62 @@
         <v>196</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>54</v>
+        <v>197</v>
       </c>
       <c r="E88" s="0" t="n">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="F88" s="0" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
       <c r="G88" s="0" t="n">
-        <v>1500</v>
+        <v>10000</v>
       </c>
       <c r="H88" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E89" s="0" t="n">
-        <v>1</v>
+        <v>3000</v>
       </c>
       <c r="F89" s="0" t="n">
-        <v>2</v>
+        <v>2500</v>
       </c>
       <c r="G89" s="0" t="n">
-        <v>3</v>
+        <v>1500</v>
       </c>
       <c r="H89" s="0" t="s">
-        <v>17</v>
+        <v>188</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E90" s="0" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="F90" s="0" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="G90" s="0" t="n">
-        <v>0.05</v>
+        <v>3</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>17</v>
@@ -2806,22 +2810,22 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C91" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E91" s="0" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F91" s="0" t="n">
         <v>0.1</v>
       </c>
-      <c r="F91" s="0" t="n">
+      <c r="G91" s="0" t="n">
         <v>0.05</v>
-      </c>
-      <c r="G91" s="0" t="n">
-        <v>0.02</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>17</v>
@@ -2829,22 +2833,22 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C92" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E92" s="0" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="F92" s="0" t="n">
-        <v>0.3</v>
+        <v>0.05</v>
       </c>
       <c r="G92" s="0" t="n">
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>17</v>
@@ -2852,22 +2856,22 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C93" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E93" s="0" t="n">
-        <v>0.08</v>
+        <v>0.4</v>
       </c>
       <c r="F93" s="0" t="n">
-        <v>0.04</v>
+        <v>0.3</v>
       </c>
       <c r="G93" s="0" t="n">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>17</v>
@@ -2875,22 +2879,22 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C94" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E94" s="0" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F94" s="0" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="G94" s="0" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="H94" s="0" t="s">
         <v>17</v>
@@ -2898,22 +2902,22 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C95" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E95" s="0" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F95" s="0" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="G95" s="0" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="H95" s="0" t="s">
         <v>17</v>
@@ -2921,22 +2925,22 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C96" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E96" s="0" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F96" s="0" t="n">
-        <v>0.15</v>
+        <v>0.02</v>
       </c>
       <c r="G96" s="0" t="n">
-        <v>0.25</v>
+        <v>0.01</v>
       </c>
       <c r="H96" s="0" t="s">
         <v>17</v>
@@ -2944,22 +2948,22 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C97" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E97" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F97" s="0" t="n">
         <v>0.15</v>
       </c>
-      <c r="F97" s="0" t="n">
-        <v>0.2</v>
-      </c>
       <c r="G97" s="0" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="H97" s="0" t="s">
         <v>17</v>
@@ -2967,22 +2971,22 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C98" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E98" s="0" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="F98" s="0" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G98" s="0" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H98" s="0" t="s">
         <v>17</v>
@@ -2990,22 +2994,22 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B99" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C99" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E99" s="0" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F99" s="0" t="n">
         <v>0.1</v>
       </c>
       <c r="G99" s="0" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="H99" s="0" t="s">
         <v>17</v>
@@ -3013,24 +3017,47 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B100" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C100" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E100" s="0" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F100" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G100" s="0" t="n">
         <v>0.15</v>
       </c>
-      <c r="F100" s="0" t="n">
+      <c r="H100" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="B101" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="C101" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E101" s="0" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F101" s="0" t="n">
         <v>0.2</v>
       </c>
-      <c r="G100" s="0" t="n">
+      <c r="G101" s="0" t="n">
         <v>0.3</v>
       </c>
-      <c r="H100" s="0" t="s">
+      <c r="H101" s="0" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3058,21 +3085,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B2" s="0" t="n">
         <f aca="false">Optimista!B67</f>
@@ -3089,7 +3116,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B3" s="2" t="n">
         <f aca="false">Optimista!B68</f>
@@ -3106,7 +3133,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">Optimista!B69</f>
@@ -3123,7 +3150,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">Optimista!B70</f>
@@ -3140,7 +3167,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">Optimista!B72</f>
@@ -3157,7 +3184,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B7" s="0" t="n">
         <f aca="false">Optimista!B71</f>
@@ -3196,12 +3223,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>1</v>
@@ -3209,7 +3236,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -3238,7 +3265,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -3267,7 +3294,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -3296,7 +3323,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -3325,7 +3352,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -3350,12 +3377,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -3380,7 +3407,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -3405,7 +3432,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-C10),0)</f>
@@ -3430,7 +3457,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -3455,7 +3482,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -3480,7 +3507,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -3505,7 +3532,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -3530,7 +3557,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-C15),0)</f>
@@ -3555,7 +3582,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -3580,7 +3607,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -3605,7 +3632,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -3630,7 +3657,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -3655,7 +3682,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-C20),0)</f>
@@ -3680,7 +3707,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -3705,7 +3732,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -3730,7 +3757,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -3755,7 +3782,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -3780,7 +3807,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-C25),0)</f>
@@ -3805,7 +3832,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -3830,7 +3857,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -3855,7 +3882,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -3880,7 +3907,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -3905,7 +3932,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-C30),0)</f>
@@ -3930,7 +3957,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -3955,7 +3982,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -3980,7 +4007,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
@@ -4005,7 +4032,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -4030,12 +4057,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
@@ -4060,7 +4087,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*meses_anio</f>
@@ -4085,7 +4112,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*meses_anio</f>
@@ -4110,7 +4137,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*meses_anio</f>
@@ -4135,7 +4162,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
@@ -4160,7 +4187,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)</f>
@@ -4185,7 +4212,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -4214,12 +4241,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B48" s="0" t="n">
         <f aca="false">meses_anio_0*sueldo_usd*sueldos_por_anio/meses_anio</f>
@@ -4248,7 +4275,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -4277,7 +4304,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -4302,7 +4329,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -4327,7 +4354,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -4336,32 +4363,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">C7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>10704.96</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">D7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>42819.84</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">E7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>107049.6</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">F7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>214099.2</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">G7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>321148.8</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
@@ -4386,7 +4413,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -4415,12 +4442,12 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -4449,7 +4476,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -4478,7 +4505,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">B58*B59</f>
@@ -4507,7 +4534,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B58</f>
@@ -4536,7 +4563,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B60</f>
@@ -4565,7 +4592,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C63" s="0" t="n">
         <f aca="false">IF(AND(B61&lt;0,C61&gt;=0),C$3-1+(-B61)/C58,"")</f>
@@ -4590,7 +4617,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C64" s="0" t="n">
         <f aca="false">IF(AND(B62&lt;0,C62&gt;=0),C$3-1+(-B62)/C60,"")</f>
@@ -4615,12 +4642,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">SUM(B60:G60)</f>
@@ -4629,7 +4656,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B68" s="2" t="n">
         <f aca="false">IFERROR(IRR(B58:G58),"no definida")</f>
@@ -4638,7 +4665,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">IF(COUNT(C63:G63)=0,"no se recupera",MIN(C63:G63))</f>
@@ -4647,7 +4674,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">IF(COUNT(C64:G64)=0,"no se recupera",MIN(C64:G64))</f>
@@ -4656,7 +4683,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B71" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -4665,7 +4692,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B72" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B71,0),"no definido")</f>
@@ -4696,12 +4723,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>2</v>
@@ -4709,7 +4736,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -4738,7 +4765,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -4767,7 +4794,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -4796,7 +4823,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -4825,7 +4852,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -4850,12 +4877,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -4880,7 +4907,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -4905,7 +4932,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-C10),0)</f>
@@ -4930,7 +4957,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -4955,7 +4982,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -4980,7 +5007,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -5005,7 +5032,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -5030,7 +5057,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-C15),0)</f>
@@ -5055,7 +5082,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -5080,7 +5107,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -5105,7 +5132,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -5130,7 +5157,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -5155,7 +5182,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-C20),0)</f>
@@ -5180,7 +5207,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -5205,7 +5232,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -5230,7 +5257,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -5255,7 +5282,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -5280,7 +5307,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-C25),0)</f>
@@ -5305,7 +5332,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -5330,7 +5357,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -5355,7 +5382,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -5380,7 +5407,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -5405,7 +5432,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-C30),0)</f>
@@ -5430,7 +5457,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -5455,7 +5482,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -5480,7 +5507,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
@@ -5505,7 +5532,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -5530,12 +5557,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
@@ -5560,7 +5587,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*meses_anio</f>
@@ -5585,7 +5612,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*meses_anio</f>
@@ -5610,7 +5637,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*meses_anio</f>
@@ -5635,7 +5662,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
@@ -5660,7 +5687,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)</f>
@@ -5685,7 +5712,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -5714,12 +5741,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B48" s="0" t="n">
         <f aca="false">meses_anio_0*sueldo_usd*sueldos_por_anio/meses_anio</f>
@@ -5748,7 +5775,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -5777,7 +5804,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -5802,7 +5829,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -5827,7 +5854,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -5836,32 +5863,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">C7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>5677.9776</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">D7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>22711.9104</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">E7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>56779.776</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">F7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>113559.552</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">G7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>170339.328</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
@@ -5886,7 +5913,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -5915,12 +5942,12 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -5949,7 +5976,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -5978,7 +6005,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">B58*B59</f>
@@ -6007,7 +6034,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B58</f>
@@ -6036,7 +6063,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B60</f>
@@ -6065,7 +6092,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C63" s="0" t="str">
         <f aca="false">IF(AND(B61&lt;0,C61&gt;=0),C$3-1+(-B61)/C58,"")</f>
@@ -6090,7 +6117,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C64" s="0" t="str">
         <f aca="false">IF(AND(B62&lt;0,C62&gt;=0),C$3-1+(-B62)/C60,"")</f>
@@ -6115,12 +6142,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">SUM(B60:G60)</f>
@@ -6129,7 +6156,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B68" s="2" t="n">
         <f aca="false">IFERROR(IRR(B58:G58),"no definida")</f>
@@ -6138,7 +6165,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">IF(COUNT(C63:G63)=0,"no se recupera",MIN(C63:G63))</f>
@@ -6147,7 +6174,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">IF(COUNT(C64:G64)=0,"no se recupera",MIN(C64:G64))</f>
@@ -6156,7 +6183,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B71" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -6165,7 +6192,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B72" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B71,0),"no definido")</f>
@@ -6196,12 +6223,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>3</v>
@@ -6209,7 +6236,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -6238,7 +6265,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -6267,7 +6294,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -6296,7 +6323,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -6325,7 +6352,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -6350,12 +6377,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -6380,7 +6407,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -6405,7 +6432,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*(u_medios_grandes-C10),0)</f>
@@ -6430,7 +6457,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -6455,7 +6482,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -6480,7 +6507,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -6505,7 +6532,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -6530,7 +6557,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*(u_medios_chicos-C15),0)</f>
@@ -6555,7 +6582,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -6580,7 +6607,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -6605,7 +6632,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -6630,7 +6657,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -6655,7 +6682,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*(u_verificadores-C20),0)</f>
@@ -6680,7 +6707,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -6705,7 +6732,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -6730,7 +6757,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -6755,7 +6782,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -6780,7 +6807,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*(u_universidades-C25),0)</f>
@@ -6805,7 +6832,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -6830,7 +6857,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -6855,7 +6882,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -6880,7 +6907,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -6905,7 +6932,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*(u_agencias-C30),0)</f>
@@ -6930,7 +6957,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -6955,7 +6982,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -6980,7 +7007,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*u_organismos,0)</f>
@@ -7005,7 +7032,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -7030,12 +7057,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*meses_anio</f>
@@ -7060,7 +7087,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*meses_anio</f>
@@ -7085,7 +7112,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*meses_anio</f>
@@ -7110,7 +7137,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*meses_anio</f>
@@ -7135,7 +7162,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*meses_anio</f>
@@ -7160,7 +7187,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)</f>
@@ -7185,7 +7212,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -7214,12 +7241,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B48" s="0" t="n">
         <f aca="false">meses_anio_0*sueldo_usd*sueldos_por_anio/meses_anio</f>
@@ -7248,7 +7275,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -7277,7 +7304,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -7302,7 +7329,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -7327,7 +7354,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -7336,32 +7363,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">C7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>1230.0336</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">D7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>4920.1344</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">E7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>12300.336</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">F7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>19680.5376</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">G7*INDEX(analisis_por_ua_mes,1,$B$2)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
+        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
         <v>24600.672</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)</f>
@@ -7386,7 +7413,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -7415,12 +7442,12 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -7449,7 +7476,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -7478,7 +7505,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">B58*B59</f>
@@ -7507,7 +7534,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B58</f>
@@ -7536,7 +7563,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B60</f>
@@ -7565,7 +7592,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C63" s="0" t="str">
         <f aca="false">IF(AND(B61&lt;0,C61&gt;=0),C$3-1+(-B61)/C58,"")</f>
@@ -7590,7 +7617,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C64" s="0" t="str">
         <f aca="false">IF(AND(B62&lt;0,C62&gt;=0),C$3-1+(-B62)/C60,"")</f>
@@ -7615,12 +7642,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">SUM(B60:G60)</f>
@@ -7629,7 +7656,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B68" s="2" t="str">
         <f aca="false">IFERROR(IRR(B58:G58),"no definida")</f>
@@ -7638,7 +7665,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B69" s="0" t="str">
         <f aca="false">IF(COUNT(C63:G63)=0,"no se recupera",MIN(C63:G63))</f>
@@ -7647,7 +7674,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B70" s="0" t="str">
         <f aca="false">IF(COUNT(C64:G64)=0,"no se recupera",MIN(C64:G64))</f>
@@ -7656,7 +7683,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B71" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -7665,7 +7692,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B72" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B71,0),"no definido")</f>

</xml_diff>

<commit_message>
Tope gratuito de 5 análisis por mes y caché del 30 % en el modelo financiero
Decisión de producto para que el escenario neutral sea viable: la versión
gratuita admite 5 análisis nuevos por usuario por mes (reemplaza el tope
diario) y la caché, que sirve los tuits virales ya analizados, sube a
40/30/20 %. Neutral: VAN 59.396, TIR 68,99 %, payback 3,00 / 3,58 años.
Cap. 3, conclusión, wiki y bitácora reescritos con las cifras nuevas.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -20,26 +20,25 @@
     <definedName function="false" hidden="false" name="analisis_por_ua_mes" vbProcedure="false">Supuestos!$E$79:$G$79</definedName>
     <definedName function="false" hidden="false" name="anio_0" vbProcedure="false">Supuestos!$D$6</definedName>
     <definedName function="false" hidden="false" name="anio_electoral" vbProcedure="false">Supuestos!$D$8:$D$13</definedName>
-    <definedName function="false" hidden="false" name="anio_inicio_b2b" vbProcedure="false">Supuestos!$E$100:$G$100</definedName>
+    <definedName function="false" hidden="false" name="anio_inicio_b2b" vbProcedure="false">Supuestos!$E$99:$G$99</definedName>
     <definedName function="false" hidden="false" name="busquedas" vbProcedure="false">Supuestos!$E$72:$G$72</definedName>
-    <definedName function="false" hidden="false" name="capt_agencias" vbProcedure="false">Supuestos!$E$106:$G$106</definedName>
-    <definedName function="false" hidden="false" name="capt_medios_chicos" vbProcedure="false">Supuestos!$E$102:$G$102</definedName>
-    <definedName function="false" hidden="false" name="capt_medios_grandes" vbProcedure="false">Supuestos!$E$101:$G$101</definedName>
-    <definedName function="false" hidden="false" name="capt_organismos" vbProcedure="false">Supuestos!$E$105:$G$105</definedName>
-    <definedName function="false" hidden="false" name="capt_universidades" vbProcedure="false">Supuestos!$E$104:$G$104</definedName>
-    <definedName function="false" hidden="false" name="capt_verificadores" vbProcedure="false">Supuestos!$E$103:$G$103</definedName>
+    <definedName function="false" hidden="false" name="capt_agencias" vbProcedure="false">Supuestos!$E$105:$G$105</definedName>
+    <definedName function="false" hidden="false" name="capt_medios_chicos" vbProcedure="false">Supuestos!$E$101:$G$101</definedName>
+    <definedName function="false" hidden="false" name="capt_medios_grandes" vbProcedure="false">Supuestos!$E$100:$G$100</definedName>
+    <definedName function="false" hidden="false" name="capt_organismos" vbProcedure="false">Supuestos!$E$104:$G$104</definedName>
+    <definedName function="false" hidden="false" name="capt_universidades" vbProcedure="false">Supuestos!$E$103:$G$103</definedName>
+    <definedName function="false" hidden="false" name="capt_verificadores" vbProcedure="false">Supuestos!$E$102:$G$102</definedName>
     <definedName function="false" hidden="false" name="cargas_sociales" vbProcedure="false">Supuestos!$D$29</definedName>
-    <definedName function="false" hidden="false" name="churn_agencias" vbProcedure="false">Supuestos!$E$111:$G$111</definedName>
-    <definedName function="false" hidden="false" name="churn_medios_chicos" vbProcedure="false">Supuestos!$E$108:$G$108</definedName>
-    <definedName function="false" hidden="false" name="churn_medios_grandes" vbProcedure="false">Supuestos!$E$107:$G$107</definedName>
-    <definedName function="false" hidden="false" name="churn_universidades" vbProcedure="false">Supuestos!$E$110:$G$110</definedName>
-    <definedName function="false" hidden="false" name="churn_verificadores" vbProcedure="false">Supuestos!$E$109:$G$109</definedName>
-    <definedName function="false" hidden="false" name="consultas_ent_mes" vbProcedure="false">Supuestos!$E$84:$G$84</definedName>
-    <definedName function="false" hidden="false" name="consultas_pro_mes" vbProcedure="false">Supuestos!$E$83:$G$83</definedName>
+    <definedName function="false" hidden="false" name="churn_agencias" vbProcedure="false">Supuestos!$E$110:$G$110</definedName>
+    <definedName function="false" hidden="false" name="churn_medios_chicos" vbProcedure="false">Supuestos!$E$107:$G$107</definedName>
+    <definedName function="false" hidden="false" name="churn_medios_grandes" vbProcedure="false">Supuestos!$E$106:$G$106</definedName>
+    <definedName function="false" hidden="false" name="churn_universidades" vbProcedure="false">Supuestos!$E$109:$G$109</definedName>
+    <definedName function="false" hidden="false" name="churn_verificadores" vbProcedure="false">Supuestos!$E$108:$G$108</definedName>
+    <definedName function="false" hidden="false" name="consultas_ent_mes" vbProcedure="false">Supuestos!$E$83:$G$83</definedName>
+    <definedName function="false" hidden="false" name="consultas_pro_mes" vbProcedure="false">Supuestos!$E$82:$G$82</definedName>
     <definedName function="false" hidden="false" name="costo_analisis" vbProcedure="false">Supuestos!$E$73:$G$73</definedName>
     <definedName function="false" hidden="false" name="crecimiento_perpetuo" vbProcedure="false">Supuestos!$D$21</definedName>
     <definedName function="false" hidden="false" name="crp_argentina" vbProcedure="false">Supuestos!$D$19</definedName>
-    <definedName function="false" hidden="false" name="dias_mes" vbProcedure="false">Supuestos!$D$81</definedName>
     <definedName function="false" hidden="false" name="dominio_anual" vbProcedure="false">Supuestos!$D$50</definedName>
     <definedName function="false" hidden="false" name="erp_maduro" vbProcedure="false">Supuestos!$D$18</definedName>
     <definedName function="false" hidden="false" name="horas_anio" vbProcedure="false">Supuestos!$D$53</definedName>
@@ -61,41 +60,41 @@
     <definedName function="false" hidden="false" name="meses_anio" vbProcedure="false">Supuestos!$D$7</definedName>
     <definedName function="false" hidden="false" name="meses_anio_0" vbProcedure="false">Supuestos!$D$30</definedName>
     <definedName function="false" hidden="false" name="meses_cobro" vbProcedure="false">Supuestos!$D$34</definedName>
-    <definedName function="false" hidden="false" name="precio_agencias" vbProcedure="false">Supuestos!$E$99:$G$99</definedName>
+    <definedName function="false" hidden="false" name="precio_agencias" vbProcedure="false">Supuestos!$E$98:$G$98</definedName>
     <definedName function="false" hidden="false" name="precio_busqueda" vbProcedure="false">Supuestos!$D$68</definedName>
     <definedName function="false" hidden="false" name="precio_entrada" vbProcedure="false">Supuestos!$D$66</definedName>
-    <definedName function="false" hidden="false" name="precio_medios_chicos" vbProcedure="false">Supuestos!$D$95</definedName>
-    <definedName function="false" hidden="false" name="precio_medios_grandes" vbProcedure="false">Supuestos!$E$94:$G$94</definedName>
-    <definedName function="false" hidden="false" name="precio_organismos" vbProcedure="false">Supuestos!$E$98:$G$98</definedName>
+    <definedName function="false" hidden="false" name="precio_medios_chicos" vbProcedure="false">Supuestos!$D$94</definedName>
+    <definedName function="false" hidden="false" name="precio_medios_grandes" vbProcedure="false">Supuestos!$E$93:$G$93</definedName>
+    <definedName function="false" hidden="false" name="precio_organismos" vbProcedure="false">Supuestos!$E$97:$G$97</definedName>
     <definedName function="false" hidden="false" name="precio_salida" vbProcedure="false">Supuestos!$D$67</definedName>
-    <definedName function="false" hidden="false" name="precio_universidades" vbProcedure="false">Supuestos!$D$97</definedName>
-    <definedName function="false" hidden="false" name="precio_verificadores" vbProcedure="false">Supuestos!$D$96</definedName>
+    <definedName function="false" hidden="false" name="precio_universidades" vbProcedure="false">Supuestos!$D$96</definedName>
+    <definedName function="false" hidden="false" name="precio_verificadores" vbProcedure="false">Supuestos!$D$95</definedName>
     <definedName function="false" hidden="false" name="prima_proyecto" vbProcedure="false">Supuestos!$D$16</definedName>
     <definedName function="false" hidden="false" name="riesgo_pais" vbProcedure="false">Supuestos!$D$15</definedName>
-    <definedName function="false" hidden="false" name="sens_captacion" vbProcedure="false">Supuestos!$D$116</definedName>
-    <definedName function="false" hidden="false" name="sens_costo_analisis" vbProcedure="false">Supuestos!$D$114</definedName>
-    <definedName function="false" hidden="false" name="sens_precios" vbProcedure="false">Supuestos!$D$115</definedName>
+    <definedName function="false" hidden="false" name="sens_captacion" vbProcedure="false">Supuestos!$D$115</definedName>
+    <definedName function="false" hidden="false" name="sens_costo_analisis" vbProcedure="false">Supuestos!$D$113</definedName>
+    <definedName function="false" hidden="false" name="sens_precios" vbProcedure="false">Supuestos!$D$114</definedName>
     <definedName function="false" hidden="false" name="sueldos_por_anio" vbProcedure="false">Supuestos!$D$27</definedName>
     <definedName function="false" hidden="false" name="sueldo_ars" vbProcedure="false">Supuestos!$D$24</definedName>
     <definedName function="false" hidden="false" name="sueldo_usd" vbProcedure="false">Supuestos!$D$26</definedName>
     <definedName function="false" hidden="false" name="tasa_capm" vbProcedure="false">Supuestos!$D$20</definedName>
     <definedName function="false" hidden="false" name="tasa_descuento" vbProcedure="false">Supuestos!$D$17</definedName>
     <definedName function="false" hidden="false" name="tasa_libre_riesgo" vbProcedure="false">Supuestos!$D$14</definedName>
-    <definedName function="false" hidden="false" name="tasa_reuso" vbProcedure="false">Supuestos!$E$82:$G$82</definedName>
+    <definedName function="false" hidden="false" name="tasa_reuso" vbProcedure="false">Supuestos!$E$81:$G$81</definedName>
     <definedName function="false" hidden="false" name="tc_encuesta" vbProcedure="false">Supuestos!$D$25</definedName>
     <definedName function="false" hidden="false" name="tokens_entrada" vbProcedure="false">Supuestos!$E$70:$G$70</definedName>
     <definedName function="false" hidden="false" name="tokens_por_millon" vbProcedure="false">Supuestos!$D$69</definedName>
     <definedName function="false" hidden="false" name="tokens_salida" vbProcedure="false">Supuestos!$E$71:$G$71</definedName>
-    <definedName function="false" hidden="false" name="tope_diario" vbProcedure="false">Supuestos!$D$80</definedName>
+    <definedName function="false" hidden="false" name="tope_mensual" vbProcedure="false">Supuestos!$D$80</definedName>
     <definedName function="false" hidden="false" name="ua_escalado" vbProcedure="false">Supuestos!$D$49</definedName>
     <definedName function="false" hidden="false" name="usuarios_activos" vbProcedure="false">Supuestos!$E$74:$G$78</definedName>
-    <definedName function="false" hidden="false" name="u_agencias" vbProcedure="false">Supuestos!$D$93</definedName>
-    <definedName function="false" hidden="false" name="u_medios_chicos" vbProcedure="false">Supuestos!$D$89</definedName>
-    <definedName function="false" hidden="false" name="u_medios_grandes" vbProcedure="false">Supuestos!$D$88</definedName>
-    <definedName function="false" hidden="false" name="u_medios_total" vbProcedure="false">Supuestos!$D$87</definedName>
-    <definedName function="false" hidden="false" name="u_organismos" vbProcedure="false">Supuestos!$D$92</definedName>
-    <definedName function="false" hidden="false" name="u_universidades" vbProcedure="false">Supuestos!$D$91</definedName>
-    <definedName function="false" hidden="false" name="u_verificadores" vbProcedure="false">Supuestos!$D$90</definedName>
+    <definedName function="false" hidden="false" name="u_agencias" vbProcedure="false">Supuestos!$D$92</definedName>
+    <definedName function="false" hidden="false" name="u_medios_chicos" vbProcedure="false">Supuestos!$D$88</definedName>
+    <definedName function="false" hidden="false" name="u_medios_grandes" vbProcedure="false">Supuestos!$D$87</definedName>
+    <definedName function="false" hidden="false" name="u_medios_total" vbProcedure="false">Supuestos!$D$86</definedName>
+    <definedName function="false" hidden="false" name="u_organismos" vbProcedure="false">Supuestos!$D$91</definedName>
+    <definedName function="false" hidden="false" name="u_universidades" vbProcedure="false">Supuestos!$D$90</definedName>
+    <definedName function="false" hidden="false" name="u_verificadores" vbProcedure="false">Supuestos!$D$89</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -107,7 +106,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="338">
   <si>
     <t xml:space="preserve">clave</t>
   </si>
@@ -628,25 +627,19 @@
     <t xml:space="preserve">análisis</t>
   </si>
   <si>
-    <t xml:space="preserve">tope_diario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tope de análisis por usuario gratuito por día</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dias_mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Días por mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">días</t>
+    <t xml:space="preserve">tope_mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope de análisis gratuitos por usuario por mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decisión de producto</t>
   </si>
   <si>
     <t xml:space="preserve">tasa_reuso</t>
   </si>
   <si>
-    <t xml:space="preserve">Análisis servidos desde la caché</t>
+    <t xml:space="preserve">Análisis servidos desde la caché (los tuits virales concentran la demanda)</t>
   </si>
   <si>
     <t xml:space="preserve">consultas_pro_mes</t>
@@ -1473,7 +1466,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -2734,27 +2727,33 @@
         <v>172</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H80" s="0" t="s">
-        <v>17</v>
+        <v>175</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C81" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D81" s="0" t="n">
-        <v>30</v>
+        <v>33</v>
+      </c>
+      <c r="E81" s="0" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F81" s="0" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G81" s="0" t="n">
+        <v>0.2</v>
       </c>
       <c r="H81" s="0" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2765,16 +2764,16 @@
         <v>179</v>
       </c>
       <c r="C82" s="0" t="s">
-        <v>33</v>
+        <v>180</v>
       </c>
       <c r="E82" s="0" t="n">
-        <v>0.3</v>
+        <v>2000</v>
       </c>
       <c r="F82" s="0" t="n">
-        <v>0.2</v>
+        <v>4000</v>
       </c>
       <c r="G82" s="0" t="n">
-        <v>0.1</v>
+        <v>8000</v>
       </c>
       <c r="H82" s="0" t="s">
         <v>17</v>
@@ -2782,87 +2781,81 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="B83" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="C83" s="0" t="s">
         <v>180</v>
       </c>
-      <c r="B83" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="C83" s="0" t="s">
-        <v>182</v>
-      </c>
       <c r="E83" s="0" t="n">
-        <v>2000</v>
+        <v>20000</v>
       </c>
       <c r="F83" s="0" t="n">
-        <v>4000</v>
+        <v>40000</v>
       </c>
       <c r="G83" s="0" t="n">
-        <v>8000</v>
+        <v>80000</v>
       </c>
       <c r="H83" s="0" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="0" t="s">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B84" s="0" t="s">
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="0" t="s">
         <v>184</v>
       </c>
-      <c r="C84" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="E84" s="0" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F84" s="0" t="n">
-        <v>40000</v>
-      </c>
-      <c r="G84" s="0" t="n">
-        <v>80000</v>
-      </c>
-      <c r="H84" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="1" t="s">
+      <c r="B86" s="0" t="s">
         <v>185</v>
+      </c>
+      <c r="C86" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="D86" s="0" t="n">
+        <v>130</v>
+      </c>
+      <c r="H86" s="0" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="B87" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="C87" s="0" t="s">
         <v>186</v>
       </c>
-      <c r="B87" s="0" t="s">
-        <v>187</v>
-      </c>
-      <c r="C87" s="0" t="s">
-        <v>188</v>
-      </c>
       <c r="D87" s="0" t="n">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="H87" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>10</v>
+        <v>93</v>
       </c>
       <c r="H88" s="0" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2873,104 +2866,104 @@
         <v>194</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>93</v>
+        <v>3</v>
       </c>
       <c r="H89" s="0" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>3</v>
+        <v>149</v>
       </c>
       <c r="H90" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C91" s="0" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>149</v>
+        <v>32</v>
       </c>
       <c r="H91" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="H92" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C93" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="D93" s="0" t="n">
-        <v>120</v>
+        <v>65</v>
+      </c>
+      <c r="E93" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F93" s="0" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G93" s="0" t="n">
+        <v>1500</v>
       </c>
       <c r="H93" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C94" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="E94" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F94" s="0" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G94" s="0" t="n">
-        <v>1500</v>
+      <c r="D94" s="0" t="n">
+        <v>200</v>
       </c>
       <c r="H94" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2984,10 +2977,10 @@
         <v>65</v>
       </c>
       <c r="D95" s="0" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="H95" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3001,10 +2994,10 @@
         <v>65</v>
       </c>
       <c r="D96" s="0" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="H96" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3015,36 +3008,42 @@
         <v>215</v>
       </c>
       <c r="C97" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="D97" s="0" t="n">
-        <v>100</v>
+        <v>216</v>
+      </c>
+      <c r="E97" s="0" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F97" s="0" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G97" s="0" t="n">
+        <v>10000</v>
       </c>
       <c r="H97" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C98" s="0" t="s">
-        <v>218</v>
+        <v>65</v>
       </c>
       <c r="E98" s="0" t="n">
-        <v>30000</v>
+        <v>3000</v>
       </c>
       <c r="F98" s="0" t="n">
-        <v>20000</v>
+        <v>2500</v>
       </c>
       <c r="G98" s="0" t="n">
-        <v>10000</v>
+        <v>1500</v>
       </c>
       <c r="H98" s="0" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3055,19 +3054,19 @@
         <v>220</v>
       </c>
       <c r="C99" s="0" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="E99" s="0" t="n">
-        <v>3000</v>
+        <v>1</v>
       </c>
       <c r="F99" s="0" t="n">
-        <v>2500</v>
+        <v>2</v>
       </c>
       <c r="G99" s="0" t="n">
-        <v>1500</v>
+        <v>3</v>
       </c>
       <c r="H99" s="0" t="s">
-        <v>209</v>
+        <v>17</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3078,16 +3077,16 @@
         <v>222</v>
       </c>
       <c r="C100" s="0" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E100" s="0" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="F100" s="0" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="G100" s="0" t="n">
-        <v>3</v>
+        <v>0.05</v>
       </c>
       <c r="H100" s="0" t="s">
         <v>17</v>
@@ -3104,13 +3103,13 @@
         <v>33</v>
       </c>
       <c r="E101" s="0" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F101" s="0" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G101" s="0" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="H101" s="0" t="s">
         <v>17</v>
@@ -3127,13 +3126,13 @@
         <v>33</v>
       </c>
       <c r="E102" s="0" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="F102" s="0" t="n">
-        <v>0.05</v>
+        <v>0.3</v>
       </c>
       <c r="G102" s="0" t="n">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="H102" s="0" t="s">
         <v>17</v>
@@ -3150,13 +3149,13 @@
         <v>33</v>
       </c>
       <c r="E103" s="0" t="n">
-        <v>0.4</v>
+        <v>0.08</v>
       </c>
       <c r="F103" s="0" t="n">
-        <v>0.3</v>
+        <v>0.04</v>
       </c>
       <c r="G103" s="0" t="n">
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="H103" s="0" t="s">
         <v>17</v>
@@ -3173,13 +3172,13 @@
         <v>33</v>
       </c>
       <c r="E104" s="0" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="F104" s="0" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="G104" s="0" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="H104" s="0" t="s">
         <v>17</v>
@@ -3196,13 +3195,13 @@
         <v>33</v>
       </c>
       <c r="E105" s="0" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F105" s="0" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="G105" s="0" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="H105" s="0" t="s">
         <v>17</v>
@@ -3219,13 +3218,13 @@
         <v>33</v>
       </c>
       <c r="E106" s="0" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F106" s="0" t="n">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
       <c r="G106" s="0" t="n">
-        <v>0.01</v>
+        <v>0.25</v>
       </c>
       <c r="H106" s="0" t="s">
         <v>17</v>
@@ -3242,13 +3241,13 @@
         <v>33</v>
       </c>
       <c r="E107" s="0" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F107" s="0" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G107" s="0" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="H107" s="0" t="s">
         <v>17</v>
@@ -3265,13 +3264,13 @@
         <v>33</v>
       </c>
       <c r="E108" s="0" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="F108" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G108" s="0" t="n">
         <v>0.2</v>
-      </c>
-      <c r="G108" s="0" t="n">
-        <v>0.3</v>
       </c>
       <c r="H108" s="0" t="s">
         <v>17</v>
@@ -3288,13 +3287,13 @@
         <v>33</v>
       </c>
       <c r="E109" s="0" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F109" s="0" t="n">
         <v>0.1</v>
       </c>
       <c r="G109" s="0" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="H109" s="0" t="s">
         <v>17</v>
@@ -3311,55 +3310,49 @@
         <v>33</v>
       </c>
       <c r="E110" s="0" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F110" s="0" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G110" s="0" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="H110" s="0" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="0" t="s">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B111" s="0" t="s">
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="0" t="s">
         <v>244</v>
       </c>
-      <c r="C111" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="E111" s="0" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F111" s="0" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G111" s="0" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H111" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="1" t="s">
+      <c r="B113" s="0" t="s">
         <v>245</v>
+      </c>
+      <c r="C113" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="D113" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H113" s="0" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="B114" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="C114" s="0" t="s">
         <v>246</v>
-      </c>
-      <c r="B114" s="0" t="s">
-        <v>247</v>
-      </c>
-      <c r="C114" s="0" t="s">
-        <v>248</v>
       </c>
       <c r="D114" s="0" t="n">
         <v>1</v>
@@ -3376,29 +3369,12 @@
         <v>250</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D115" s="0" t="n">
         <v>1</v>
       </c>
       <c r="H115" s="0" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="0" t="s">
-        <v>251</v>
-      </c>
-      <c r="B116" s="0" t="s">
-        <v>252</v>
-      </c>
-      <c r="C116" s="0" t="s">
-        <v>248</v>
-      </c>
-      <c r="D116" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H116" s="0" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3426,46 +3402,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>254</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B2" s="0" t="n">
         <f aca="false">Optimista!B75</f>
-        <v>674427.968185843</v>
+        <v>827194.037742681</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">Neutral!B75</f>
-        <v>-12295.6221440048</v>
+        <v>59396.0929553104</v>
       </c>
       <c r="D2" s="0" t="n">
         <f aca="false">Pesimista!B75</f>
-        <v>-154002.763648191</v>
+        <v>-136598.112572607</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B3" s="2" t="n">
         <f aca="false">Optimista!B76</f>
-        <v>50.7108739159507</v>
+        <v>54.4725888516988</v>
       </c>
       <c r="C3" s="2" t="n">
         <f aca="false">Neutral!B76</f>
-        <v>0.14478841787379</v>
+        <v>0.689916456530632</v>
       </c>
       <c r="D3" s="2" t="str">
         <f aca="false">Pesimista!B76</f>
@@ -3474,15 +3450,15 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">Optimista!B77</f>
-        <v>0.0202145886215281</v>
+        <v>0.0188241201012943</v>
       </c>
       <c r="C4" s="0" t="n">
         <f aca="false">Neutral!B77</f>
-        <v>4.50369272722782</v>
+        <v>3.00121464151533</v>
       </c>
       <c r="D4" s="0" t="str">
         <f aca="false">Pesimista!B77</f>
@@ -3491,15 +3467,15 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">Optimista!B78</f>
-        <v>0.0252682357769101</v>
-      </c>
-      <c r="C5" s="0" t="str">
+        <v>0.0235301501266178</v>
+      </c>
+      <c r="C5" s="0" t="n">
         <f aca="false">Neutral!B78</f>
-        <v>no se recupera</v>
+        <v>3.5847846276075</v>
       </c>
       <c r="D5" s="0" t="str">
         <f aca="false">Pesimista!B78</f>
@@ -3508,24 +3484,24 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">Optimista!B81</f>
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">Neutral!B81</f>
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">Pesimista!B81</f>
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B7" s="0" t="n">
         <f aca="false">Optimista!B80</f>
@@ -3542,29 +3518,29 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">Optimista!B79</f>
-        <v>1200014.0933853</v>
+        <v>1598622.49924048</v>
       </c>
       <c r="C8" s="0" t="n">
         <f aca="false">Neutral!B79</f>
-        <v>5048.94149861585</v>
+        <v>190486.580559725</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">Pesimista!B79</f>
-        <v>-154002.763648191</v>
+        <v>-136598.112572607</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">meses_anio*(u_medios_grandes*INDEX(precio_medios_grandes,1,2)+(u_medios_total-u_medios_grandes)*precio_medios_chicos+u_verificadores*precio_verificadores+u_universidades*precio_universidades+u_agencias*INDEX(precio_agencias,1,2))+u_organismos*INDEX(precio_organismos,1,2)</f>
@@ -3573,7 +3549,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">meses_anio*(u_medios_grandes*INDEX(precio_medios_grandes,1,2)+u_medios_chicos*precio_medios_chicos+u_verificadores*precio_verificadores+u_universidades*precio_universidades+u_agencias*INDEX(precio_agencias,1,2))+u_organismos*INDEX(precio_organismos,1,2)</f>
@@ -3582,7 +3558,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B13" s="0" t="n">
         <f aca="false">Neutral!G45</f>
@@ -3591,12 +3567,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">meses_anio_0*sueldo_usd*(1+cargas_sociales)*sueldos_por_anio/meses_anio</f>
@@ -3605,7 +3581,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">tasa_capm</f>
@@ -3636,12 +3612,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>1</v>
@@ -3649,7 +3625,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -3678,7 +3654,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -3707,7 +3683,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -3736,7 +3712,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -3765,7 +3741,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -3790,12 +3766,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -3820,7 +3796,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -3845,7 +3821,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*sens_captacion*(u_medios_grandes-C10),0)</f>
@@ -3870,7 +3846,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -3895,7 +3871,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -3920,7 +3896,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -3945,7 +3921,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -3970,7 +3946,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*sens_captacion*(u_medios_chicos-C15),0)</f>
@@ -3995,7 +3971,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -4020,7 +3996,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -4045,7 +4021,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -4070,7 +4046,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -4095,7 +4071,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*sens_captacion*(u_verificadores-C20),0)</f>
@@ -4120,7 +4096,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -4145,7 +4121,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -4170,7 +4146,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -4195,7 +4171,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -4220,7 +4196,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*sens_captacion*(u_universidades-C25),0)</f>
@@ -4245,7 +4221,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -4270,7 +4246,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -4295,7 +4271,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -4320,7 +4296,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -4345,7 +4321,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*sens_captacion*(u_agencias-C30),0)</f>
@@ -4370,7 +4346,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -4395,7 +4371,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -4420,7 +4396,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*sens_captacion*u_organismos,0)</f>
@@ -4445,7 +4421,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -4470,12 +4446,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*sens_precios*meses_anio</f>
@@ -4500,7 +4476,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*sens_precios*meses_anio</f>
@@ -4525,7 +4501,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*sens_precios*meses_anio</f>
@@ -4550,7 +4526,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*sens_precios*meses_anio</f>
@@ -4575,7 +4551,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*sens_precios*meses_anio</f>
@@ -4600,7 +4576,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)*sens_precios</f>
@@ -4625,7 +4601,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -4654,12 +4630,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C48" s="0" t="n">
         <f aca="false">sueldo_usd*sueldos_por_anio*(1+cargas_sociales)*(1+ajuste_sueldo)^C$3</f>
@@ -4684,7 +4660,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -4713,7 +4689,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -4738,7 +4714,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -4763,7 +4739,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -4772,57 +4748,57 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>10704.96</v>
+        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>2293.92</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>42819.84</v>
+        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>9175.68</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>107049.6</v>
+        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>22939.2</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>214099.2</v>
+        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>45878.4</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>321148.8</v>
+        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>68817.6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>9634.464</v>
+        <v>8258.112</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>27618.7968</v>
+        <v>23673.2544</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>40892.9472</v>
+        <v>35051.0976</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>49456.9152</v>
+        <v>42391.6416</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>55558.7424</v>
+        <v>47621.7792</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -4830,33 +4806,33 @@
       </c>
       <c r="C55" s="0" t="n">
         <f aca="false">SUM(C48:C54)</f>
-        <v>58051.434</v>
+        <v>48264.042</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">SUM(D48:D54)</f>
-        <v>116987.1573</v>
+        <v>79397.4549</v>
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">SUM(E48:E54)</f>
-        <v>199467.343725</v>
+        <v>109515.094125</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">SUM(F48:F54)</f>
-        <v>320378.00155125</v>
+        <v>145091.92795125</v>
       </c>
       <c r="G55" s="0" t="n">
         <f aca="false">SUM(G48:G54)</f>
-        <v>438911.373068813</v>
+        <v>178643.209868813</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -4864,28 +4840,28 @@
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">C45-C55</f>
-        <v>196948.566</v>
+        <v>206735.958</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">D45-D55</f>
-        <v>356412.8427</v>
+        <v>394002.5451</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">E45-E55</f>
-        <v>591932.656275</v>
+        <v>681884.905875</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">F45-F55</f>
-        <v>528621.99844875</v>
+        <v>703908.07204875</v>
       </c>
       <c r="G58" s="0" t="n">
         <f aca="false">G45-G55</f>
-        <v>606888.626931188</v>
+        <v>867156.790131188</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">MIN(0,B58)</f>
@@ -4914,7 +4890,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B58)</f>
@@ -4922,28 +4898,28 @@
       </c>
       <c r="C60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B59+C58)</f>
-        <v>68322.6481</v>
+        <v>71748.2353</v>
       </c>
       <c r="D60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,C59+D58)</f>
-        <v>124744.494945</v>
+        <v>137900.890785</v>
       </c>
       <c r="E60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,D59+E58)</f>
-        <v>207176.42969625</v>
+        <v>238659.71705625</v>
       </c>
       <c r="F60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,E59+F58)</f>
-        <v>185017.699457063</v>
+        <v>246367.825217063</v>
       </c>
       <c r="G60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,F59+G58)</f>
-        <v>212411.019425916</v>
+        <v>303504.876545916</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">meses_cobro/meses_anio*B45</f>
@@ -4972,7 +4948,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B61</f>
@@ -5001,7 +4977,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G63" s="0" t="n">
         <f aca="false">G61</f>
@@ -5010,12 +4986,12 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">B58-B60-B62+N(B63)</f>
@@ -5023,28 +4999,28 @@
       </c>
       <c r="C66" s="0" t="n">
         <f aca="false">C58-C60-C62+N(C63)</f>
-        <v>86125.9179</v>
+        <v>92487.7227</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">D58-D60-D62+N(D63)</f>
-        <v>195268.347755</v>
+        <v>219701.654315</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">E58-E60-E62+N(E63)</f>
-        <v>331756.22657875</v>
+        <v>390225.18881875</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">F58-F60-F62+N(F63)</f>
-        <v>334004.298991688</v>
+        <v>447940.246831688</v>
       </c>
       <c r="G66" s="0" t="n">
         <f aca="false">G58-G60-G62+N(G63)</f>
-        <v>535977.607505272</v>
+        <v>705151.913585272</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -5073,7 +5049,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B66*B67</f>
@@ -5081,28 +5057,28 @@
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">C66*C67</f>
-        <v>68900.73432</v>
+        <v>73990.17816</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">D66*D67</f>
-        <v>124971.7425632</v>
+        <v>140609.0587616</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">E66*E67</f>
-        <v>169859.18800832</v>
+        <v>199795.2966752</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">F66*F67</f>
-        <v>136808.160866995</v>
+        <v>183476.325102259</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">G66*G67</f>
-        <v>175629.142427328</v>
+        <v>231064.179043622</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B66</f>
@@ -5110,28 +5086,28 @@
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">B69+C66</f>
-        <v>84384.9179</v>
+        <v>90746.7227</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">C69+D66</f>
-        <v>279653.265655</v>
+        <v>310448.377015</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E66</f>
-        <v>611409.49223375</v>
+        <v>700673.56583375</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F66</f>
-        <v>945413.791225437</v>
+        <v>1148613.81266544</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G66</f>
-        <v>1481391.39873071</v>
+        <v>1853765.72625071</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">B68</f>
@@ -5139,32 +5115,32 @@
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">B70+C68</f>
-        <v>67159.73432</v>
+        <v>72249.17816</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">C70+D68</f>
-        <v>192131.4768832</v>
+        <v>212858.2369216</v>
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">D70+E68</f>
-        <v>361990.66489152</v>
+        <v>412653.5335968</v>
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">E70+F68</f>
-        <v>498798.825758515</v>
+        <v>596129.858699059</v>
       </c>
       <c r="G70" s="0" t="n">
         <f aca="false">F70+G68</f>
-        <v>674427.968185843</v>
+        <v>827194.037742681</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C71" s="0" t="n">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C66,"")</f>
-        <v>0.0202145886215281</v>
+        <v>0.0188241201012943</v>
       </c>
       <c r="D71" s="0" t="str">
         <f aca="false">IF(AND(C69&lt;0,D69&gt;=0),D$3-1+(-C69)/D66,"")</f>
@@ -5185,11 +5161,11 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C72" s="0" t="n">
         <f aca="false">IF(AND(B70&lt;0,C70&gt;=0),C$3-1+(-B70)/C68,"")</f>
-        <v>0.0252682357769101</v>
+        <v>0.0235301501266178</v>
       </c>
       <c r="D72" s="0" t="str">
         <f aca="false">IF(AND(C70&lt;0,D70&gt;=0),D$3-1+(-C70)/D68,"")</f>
@@ -5210,57 +5186,57 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B75" s="0" t="n">
         <f aca="false">SUM(B68:G68)</f>
-        <v>674427.968185843</v>
+        <v>827194.037742681</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B76" s="2" t="n">
         <f aca="false">IFERROR(IRR(B66:G66),"no definida")</f>
-        <v>50.7108739159507</v>
+        <v>54.4725888516988</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
-        <v>0.0202145886215281</v>
+        <v>0.0188241201012943</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">IF(COUNT(C72:G72)=0,"no se recupera",MIN(C72:G72))</f>
-        <v>0.0252682357769101</v>
+        <v>0.0235301501266178</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">SUM(B68:G68)+MAX(0,G66-G63)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>1200014.0933853</v>
+        <v>1598622.49924048</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B80" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -5269,11 +5245,11 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B81" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B80,0),"no definido")</f>
-        <v>41</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -5300,12 +5276,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>2</v>
@@ -5313,7 +5289,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -5342,7 +5318,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -5371,7 +5347,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -5400,7 +5376,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -5429,7 +5405,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -5454,12 +5430,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -5484,7 +5460,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -5509,7 +5485,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*sens_captacion*(u_medios_grandes-C10),0)</f>
@@ -5534,7 +5510,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -5559,7 +5535,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -5584,7 +5560,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -5609,7 +5585,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -5634,7 +5610,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*sens_captacion*(u_medios_chicos-C15),0)</f>
@@ -5659,7 +5635,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -5684,7 +5660,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -5709,7 +5685,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -5734,7 +5710,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -5759,7 +5735,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*sens_captacion*(u_verificadores-C20),0)</f>
@@ -5784,7 +5760,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -5809,7 +5785,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -5834,7 +5810,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -5859,7 +5835,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -5884,7 +5860,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*sens_captacion*(u_universidades-C25),0)</f>
@@ -5909,7 +5885,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -5934,7 +5910,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -5959,7 +5935,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -5984,7 +5960,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -6009,7 +5985,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*sens_captacion*(u_agencias-C30),0)</f>
@@ -6034,7 +6010,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -6059,7 +6035,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -6084,7 +6060,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*sens_captacion*u_organismos,0)</f>
@@ -6109,7 +6085,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -6134,12 +6110,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*sens_precios*meses_anio</f>
@@ -6164,7 +6140,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*sens_precios*meses_anio</f>
@@ -6189,7 +6165,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*sens_precios*meses_anio</f>
@@ -6214,7 +6190,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*sens_precios*meses_anio</f>
@@ -6239,7 +6215,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*sens_precios*meses_anio</f>
@@ -6264,7 +6240,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)*sens_precios</f>
@@ -6289,7 +6265,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -6318,12 +6294,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C48" s="0" t="n">
         <f aca="false">sueldo_usd*sueldos_por_anio*(1+cargas_sociales)*(1+ajuste_sueldo)^C$3</f>
@@ -6348,7 +6324,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -6377,7 +6353,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -6402,7 +6378,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -6427,7 +6403,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -6436,32 +6412,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>5677.9776</v>
+        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>2070.096</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>22711.9104</v>
+        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>8280.384</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>56779.776</v>
+        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>20700.96</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>113559.552</v>
+        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>41401.92</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>170339.328</v>
+        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>62102.88</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
@@ -6469,24 +6445,24 @@
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>17033.9328</v>
+        <v>14904.6912</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>50155.4688</v>
+        <v>43886.0352</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>76652.6976</v>
+        <v>67071.1104</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>97471.9488</v>
+        <v>85287.9552</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -6494,33 +6470,33 @@
       </c>
       <c r="C55" s="0" t="n">
         <f aca="false">SUM(C48:C54)</f>
-        <v>41353.9876</v>
+        <v>37746.106</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">SUM(D48:D54)</f>
-        <v>79033.1637</v>
+        <v>62472.3957</v>
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">SUM(E48:E54)</f>
-        <v>154100.041325</v>
+        <v>111751.791725</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">SUM(F48:F54)</f>
-        <v>241314.13595125</v>
+        <v>159574.91675125</v>
       </c>
       <c r="G55" s="0" t="n">
         <f aca="false">SUM(G48:G54)</f>
-        <v>322935.107468813</v>
+        <v>202514.665868813</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -6528,28 +6504,28 @@
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">C45-C55</f>
-        <v>-41353.9876</v>
+        <v>-37746.106</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">D45-D55</f>
-        <v>-21433.1637</v>
+        <v>-4872.3957</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">E45-E55</f>
-        <v>55699.958675</v>
+        <v>98048.208275</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">F45-F55</f>
-        <v>18485.86404875</v>
+        <v>100225.08324875</v>
       </c>
       <c r="G58" s="0" t="n">
         <f aca="false">G45-G55</f>
-        <v>46464.8925311875</v>
+        <v>166885.334131188</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">MIN(0,B58)</f>
@@ -6557,15 +6533,15 @@
       </c>
       <c r="C59" s="0" t="n">
         <f aca="false">MIN(0,B59+C58)</f>
-        <v>-43094.9876</v>
+        <v>-39487.106</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">MIN(0,C59+D58)</f>
-        <v>-64528.1513</v>
+        <v>-44359.5017</v>
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">MIN(0,D59+E58)</f>
-        <v>-8828.192625</v>
+        <v>0</v>
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">MIN(0,E59+F58)</f>
@@ -6578,7 +6554,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B58)</f>
@@ -6594,20 +6570,20 @@
       </c>
       <c r="E60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,D59+E58)</f>
-        <v>0</v>
+        <v>18791.04730125</v>
       </c>
       <c r="F60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,E59+F58)</f>
-        <v>3380.1849983125</v>
+        <v>35078.7791370625</v>
       </c>
       <c r="G60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,F59+G58)</f>
-        <v>16262.7123859156</v>
+        <v>58409.8669459156</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">meses_cobro/meses_anio*B45</f>
@@ -6636,7 +6612,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B61</f>
@@ -6665,7 +6641,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G63" s="0" t="n">
         <f aca="false">G61</f>
@@ -6674,12 +6650,12 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">B58-B60-B62+N(B63)</f>
@@ -6687,28 +6663,28 @@
       </c>
       <c r="C66" s="0" t="n">
         <f aca="false">C58-C60-C62+N(C63)</f>
-        <v>-41353.9876</v>
+        <v>-37746.106</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">D58-D60-D62+N(D63)</f>
-        <v>-31033.1637</v>
+        <v>-14472.3957</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">E58-E60-E62+N(E63)</f>
-        <v>30333.2920083333</v>
+        <v>53890.4943070833</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">F58-F60-F62+N(F63)</f>
-        <v>6772.34571710416</v>
+        <v>56812.9707783542</v>
       </c>
       <c r="G66" s="0" t="n">
         <f aca="false">G58-G60-G62+N(G63)</f>
-        <v>73502.1801452719</v>
+        <v>151775.467185272</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -6737,7 +6713,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B66*B67</f>
@@ -6745,28 +6721,28 @@
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">C66*C67</f>
-        <v>-33083.19008</v>
+        <v>-30196.8848</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">D66*D67</f>
-        <v>-19861.224768</v>
+        <v>-9262.333248</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">E66*E67</f>
-        <v>15530.6455082667</v>
+        <v>27591.9330852267</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">F66*F67</f>
-        <v>2773.95280572587</v>
+        <v>23270.5928308139</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">G66*G67</f>
-        <v>24085.1943900027</v>
+        <v>49733.7850872699</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B66</f>
@@ -6774,28 +6750,28 @@
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">B69+C66</f>
-        <v>-43094.9876</v>
+        <v>-39487.106</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">C69+D66</f>
-        <v>-74128.1513</v>
+        <v>-53959.5017</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E66</f>
-        <v>-43794.8592916667</v>
+        <v>-69.0073929166683</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F66</f>
-        <v>-37022.5135745625</v>
+        <v>56743.9633854375</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G66</f>
-        <v>36479.6665707094</v>
+        <v>208519.430570709</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">B68</f>
@@ -6803,28 +6779,28 @@
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">B70+C68</f>
-        <v>-34824.19008</v>
+        <v>-31937.8848</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">C70+D68</f>
-        <v>-54685.414848</v>
+        <v>-41200.218048</v>
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">D70+E68</f>
-        <v>-39154.7693397333</v>
+        <v>-13608.2849627733</v>
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">E70+F68</f>
-        <v>-36380.8165340075</v>
+        <v>9662.30786804053</v>
       </c>
       <c r="G70" s="0" t="n">
         <f aca="false">F70+G68</f>
-        <v>-12295.6221440048</v>
+        <v>59396.0929553104</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C71" s="0" t="str">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C66,"")</f>
@@ -6838,18 +6814,18 @@
         <f aca="false">IF(AND(D69&lt;0,E69&gt;=0),E$3-1+(-D69)/E66,"")</f>
         <v/>
       </c>
-      <c r="F71" s="0" t="str">
+      <c r="F71" s="0" t="n">
         <f aca="false">IF(AND(E69&lt;0,F69&gt;=0),F$3-1+(-E69)/F66,"")</f>
+        <v>3.00121464151533</v>
+      </c>
+      <c r="G71" s="0" t="str">
+        <f aca="false">IF(AND(F69&lt;0,G69&gt;=0),G$3-1+(-F69)/G66,"")</f>
         <v/>
-      </c>
-      <c r="G71" s="0" t="n">
-        <f aca="false">IF(AND(F69&lt;0,G69&gt;=0),G$3-1+(-F69)/G66,"")</f>
-        <v>4.50369272722782</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C72" s="0" t="str">
         <f aca="false">IF(AND(B70&lt;0,C70&gt;=0),C$3-1+(-B70)/C68,"")</f>
@@ -6863,9 +6839,9 @@
         <f aca="false">IF(AND(D70&lt;0,E70&gt;=0),E$3-1+(-D70)/E68,"")</f>
         <v/>
       </c>
-      <c r="F72" s="0" t="str">
+      <c r="F72" s="0" t="n">
         <f aca="false">IF(AND(E70&lt;0,F70&gt;=0),F$3-1+(-E70)/F68,"")</f>
-        <v/>
+        <v>3.5847846276075</v>
       </c>
       <c r="G72" s="0" t="str">
         <f aca="false">IF(AND(F70&lt;0,G70&gt;=0),G$3-1+(-F70)/G68,"")</f>
@@ -6874,57 +6850,57 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B75" s="0" t="n">
         <f aca="false">SUM(B68:G68)</f>
-        <v>-12295.6221440048</v>
+        <v>59396.0929553104</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B76" s="2" t="n">
         <f aca="false">IFERROR(IRR(B66:G66),"no definida")</f>
-        <v>0.14478841787379</v>
+        <v>0.689916456530632</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
-        <v>4.50369272722782</v>
+        <v>3.00121464151533</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>260</v>
-      </c>
-      <c r="B78" s="0" t="str">
+        <v>258</v>
+      </c>
+      <c r="B78" s="0" t="n">
         <f aca="false">IF(COUNT(C72:G72)=0,"no se recupera",MIN(C72:G72))</f>
-        <v>no se recupera</v>
+        <v>3.5847846276075</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">SUM(B68:G68)+MAX(0,G66-G63)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>5048.94149861585</v>
+        <v>190486.580559725</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B80" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -6933,11 +6909,11 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B81" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B80,0),"no definido")</f>
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -6964,12 +6940,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>3</v>
@@ -6977,7 +6953,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -7006,7 +6982,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -7035,7 +7011,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -7064,7 +7040,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">IF(B$3&gt;=INDEX(anio_inicio_b2b,1,$B$2),1,0)</f>
@@ -7093,7 +7069,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -7118,12 +7094,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -7148,7 +7124,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -7173,7 +7149,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_grandes,1,$B$2)*sens_captacion*(u_medios_grandes-C10),0)</f>
@@ -7198,7 +7174,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -7223,7 +7199,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -7248,7 +7224,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -7273,7 +7249,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -7298,7 +7274,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_medios_chicos,1,$B$2)*sens_captacion*(u_medios_chicos-C15),0)</f>
@@ -7323,7 +7299,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -7348,7 +7324,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -7373,7 +7349,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -7398,7 +7374,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -7423,7 +7399,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_verificadores,1,$B$2)*sens_captacion*(u_verificadores-C20),0)</f>
@@ -7448,7 +7424,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -7473,7 +7449,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -7498,7 +7474,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -7523,7 +7499,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -7548,7 +7524,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_universidades,1,$B$2)*sens_captacion*(u_universidades-C25),0)</f>
@@ -7573,7 +7549,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -7598,7 +7574,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -7623,7 +7599,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -7648,7 +7624,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -7673,7 +7649,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C6*ROUND(INDEX(capt_agencias,1,$B$2)*sens_captacion*(u_agencias-C30),0)</f>
@@ -7698,7 +7674,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -7723,7 +7699,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -7748,7 +7724,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C6*ROUND(INDEX(capt_organismos,1,$B$2)*sens_captacion*u_organismos,0)</f>
@@ -7773,7 +7749,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -7798,12 +7774,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*sens_precios*meses_anio</f>
@@ -7828,7 +7804,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*sens_precios*meses_anio</f>
@@ -7853,7 +7829,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*sens_precios*meses_anio</f>
@@ -7878,7 +7854,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*sens_precios*meses_anio</f>
@@ -7903,7 +7879,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*sens_precios*meses_anio</f>
@@ -7928,7 +7904,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)*sens_precios</f>
@@ -7953,7 +7929,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -7982,12 +7958,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C48" s="0" t="n">
         <f aca="false">sueldo_usd*sueldos_por_anio*(1+cargas_sociales)*(1+ajuste_sueldo)^C$3</f>
@@ -8012,7 +7988,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -8041,7 +8017,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">horas_anio*IF(INDEX(hosting_gpu_activo,C$3,$B$2)=1,hosting_gpu,hosting_cpu)</f>
@@ -8066,7 +8042,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C51" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -8091,7 +8067,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B52" s="0" t="n">
         <f aca="false">inv_dominio+inv_chrome_web_store+inv_marca_inpi+inv_legal</f>
@@ -8100,32 +8076,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>1230.0336</v>
+        <f aca="false">C7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>911.136</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>4920.1344</v>
+        <f aca="false">D7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>3644.544</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>12300.336</v>
+        <f aca="false">E7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>9111.36</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>19680.5376</v>
+        <f aca="false">F7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>14578.176</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_diario*dias_mes)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>24600.672</v>
+        <f aca="false">G7*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>18222.72</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
@@ -8137,20 +8113,20 @@
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>37721.0304</v>
+        <v>33529.8048</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>93482.5536</v>
+        <v>83095.6032</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>113163.0912</v>
+        <v>100589.4144</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B55" s="0" t="n">
         <f aca="false">SUM(B48:B54)</f>
@@ -8158,33 +8134,33 @@
       </c>
       <c r="C55" s="0" t="n">
         <f aca="false">SUM(C48:C54)</f>
-        <v>34888.0436</v>
+        <v>34569.146</v>
       </c>
       <c r="D55" s="0" t="n">
         <f aca="false">SUM(D48:D54)</f>
-        <v>41135.4549</v>
+        <v>39859.8645</v>
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">SUM(E48:E54)</f>
-        <v>88888.962925</v>
+        <v>81508.761325</v>
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">SUM(F48:F54)</f>
-        <v>154763.77755125</v>
+        <v>139274.46555125</v>
       </c>
       <c r="G55" s="0" t="n">
         <f aca="false">SUM(G48:G54)</f>
-        <v>182170.393868813</v>
+        <v>163218.765068813</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">B45-B55</f>
@@ -8192,28 +8168,28 @@
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">C45-C55</f>
-        <v>-34888.0436</v>
+        <v>-34569.146</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">D45-D55</f>
-        <v>-41135.4549</v>
+        <v>-39859.8645</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">E45-E55</f>
-        <v>-53688.962925</v>
+        <v>-46308.761325</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">F45-F55</f>
-        <v>-92363.77755125</v>
+        <v>-76874.46555125</v>
       </c>
       <c r="G58" s="0" t="n">
         <f aca="false">G45-G55</f>
-        <v>-95370.3938688125</v>
+        <v>-76418.7650688125</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">MIN(0,B58)</f>
@@ -8221,28 +8197,28 @@
       </c>
       <c r="C59" s="0" t="n">
         <f aca="false">MIN(0,B59+C58)</f>
-        <v>-36629.0436</v>
+        <v>-36310.146</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">MIN(0,C59+D58)</f>
-        <v>-77764.4985</v>
+        <v>-76170.0105</v>
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">MIN(0,D59+E58)</f>
-        <v>-131453.461425</v>
+        <v>-122478.771825</v>
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">MIN(0,E59+F58)</f>
-        <v>-223817.23897625</v>
+        <v>-199353.23737625</v>
       </c>
       <c r="G59" s="0" t="n">
         <f aca="false">MIN(0,F59+G58)</f>
-        <v>-319187.632845063</v>
+        <v>-275772.002445063</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B58)</f>
@@ -8271,7 +8247,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">meses_cobro/meses_anio*B45</f>
@@ -8300,7 +8276,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B62" s="0" t="n">
         <f aca="false">B61</f>
@@ -8329,7 +8305,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G63" s="0" t="n">
         <f aca="false">G61</f>
@@ -8338,12 +8314,12 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">B58-B60-B62+N(B63)</f>
@@ -8351,28 +8327,28 @@
       </c>
       <c r="C66" s="0" t="n">
         <f aca="false">C58-C60-C62+N(C63)</f>
-        <v>-34888.0436</v>
+        <v>-34569.146</v>
       </c>
       <c r="D66" s="0" t="n">
         <f aca="false">D58-D60-D62+N(D63)</f>
-        <v>-41135.4549</v>
+        <v>-39859.8645</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">E58-E60-E62+N(E63)</f>
-        <v>-59555.6295916667</v>
+        <v>-52175.4279916667</v>
       </c>
       <c r="F66" s="0" t="n">
         <f aca="false">F58-F60-F62+N(F63)</f>
-        <v>-96897.1108845833</v>
+        <v>-81407.7988845833</v>
       </c>
       <c r="G66" s="0" t="n">
         <f aca="false">G58-G60-G62+N(G63)</f>
-        <v>-84970.3938688125</v>
+        <v>-66018.7650688125</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -8401,7 +8377,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B66*B67</f>
@@ -8409,28 +8385,28 @@
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">C66*C67</f>
-        <v>-27910.43488</v>
+        <v>-27655.3168</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">D66*D67</f>
-        <v>-26326.691136</v>
+        <v>-25510.31328</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">E66*E67</f>
-        <v>-30492.4823509333</v>
+        <v>-26713.8191317333</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">F66*F67</f>
-        <v>-39689.0566183253</v>
+        <v>-33344.6344231253</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">G66*G67</f>
-        <v>-27843.0986629325</v>
+        <v>-21633.0289377485</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B66</f>
@@ -8438,28 +8414,28 @@
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">B69+C66</f>
-        <v>-36629.0436</v>
+        <v>-36310.146</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">C69+D66</f>
-        <v>-77764.4985</v>
+        <v>-76170.0105</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E66</f>
-        <v>-137320.128091667</v>
+        <v>-128345.438491667</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F66</f>
-        <v>-234217.23897625</v>
+        <v>-209753.23737625</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G66</f>
-        <v>-319187.632845063</v>
+        <v>-275772.002445063</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B70" s="0" t="n">
         <f aca="false">B68</f>
@@ -8467,28 +8443,28 @@
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">B70+C68</f>
-        <v>-29651.43488</v>
+        <v>-29396.3168</v>
       </c>
       <c r="D70" s="0" t="n">
         <f aca="false">C70+D68</f>
-        <v>-55978.126016</v>
+        <v>-54906.63008</v>
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">D70+E68</f>
-        <v>-86470.6083669334</v>
+        <v>-81620.4492117333</v>
       </c>
       <c r="F70" s="0" t="n">
         <f aca="false">E70+F68</f>
-        <v>-126159.664985259</v>
+        <v>-114965.083634859</v>
       </c>
       <c r="G70" s="0" t="n">
         <f aca="false">F70+G68</f>
-        <v>-154002.763648191</v>
+        <v>-136598.112572607</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C71" s="0" t="str">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C66,"")</f>
@@ -8513,7 +8489,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="0" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C72" s="0" t="str">
         <f aca="false">IF(AND(B70&lt;0,C70&gt;=0),C$3-1+(-B70)/C68,"")</f>
@@ -8538,21 +8514,21 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B75" s="0" t="n">
         <f aca="false">SUM(B68:G68)</f>
-        <v>-154002.763648191</v>
+        <v>-136598.112572607</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B76" s="2" t="str">
         <f aca="false">IFERROR(IRR(B66:G66),"no definida")</f>
@@ -8561,7 +8537,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B77" s="0" t="str">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
@@ -8570,7 +8546,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B78" s="0" t="str">
         <f aca="false">IF(COUNT(C72:G72)=0,"no se recupera",MIN(C72:G72))</f>
@@ -8579,16 +8555,16 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">SUM(B68:G68)+MAX(0,G66-G63)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>-154002.763648191</v>
+        <v>-136598.112572607</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B80" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -8597,11 +8573,11 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B81" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G55/B80,0),"no definido")</f>
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustar las cuotas de la API y agregar CAC, LTV y el tope gratuito
La API intermedia pasa de 50.000 a 5.000 consultas por USD 200 y la
superior incluye 40.000, con excedente a USD 0,04 por consulta: el margen
a cuota llena queda positivo en los tres escenarios. El script costea
MIN(demanda, cuota), calcula el margen a cuota llena y el CAC/LTV del
escenario neutral, y el validador exporta la tabla y las macros. Neutral
y optimista no cambian; el pesimista mejora (VAN -134.903 -> -94.161).

Cap. 3: tabla de precios públicos de herramientas comparables como
validación por comparación de mercado, subsección de CAC y LTV y prosa
del escenario pesimista. Cap. 4: RF-17, tope de cinco análisis a demanda
nuevos por instalación, previsto y no implementado en el prototipo.
Parte de #87.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -21,23 +21,25 @@
     <definedName function="false" hidden="false" name="anio_0" vbProcedure="false">Supuestos!$D$6</definedName>
     <definedName function="false" hidden="false" name="anio_electoral" vbProcedure="false">Supuestos!$D$8:$D$13</definedName>
     <definedName function="false" hidden="false" name="busquedas" vbProcedure="false">Supuestos!$E$60:$G$60</definedName>
-    <definedName function="false" hidden="false" name="capt_agencias" vbProcedure="false">Supuestos!$E$93:$G$93</definedName>
-    <definedName function="false" hidden="false" name="capt_medios_chicos" vbProcedure="false">Supuestos!$E$89:$G$89</definedName>
-    <definedName function="false" hidden="false" name="capt_medios_grandes" vbProcedure="false">Supuestos!$E$88:$G$88</definedName>
-    <definedName function="false" hidden="false" name="capt_organismos" vbProcedure="false">Supuestos!$E$92:$G$92</definedName>
-    <definedName function="false" hidden="false" name="capt_universidades" vbProcedure="false">Supuestos!$E$91:$G$91</definedName>
-    <definedName function="false" hidden="false" name="capt_verificadores" vbProcedure="false">Supuestos!$E$90:$G$90</definedName>
+    <definedName function="false" hidden="false" name="capt_agencias" vbProcedure="false">Supuestos!$E$96:$G$96</definedName>
+    <definedName function="false" hidden="false" name="capt_medios_chicos" vbProcedure="false">Supuestos!$E$92:$G$92</definedName>
+    <definedName function="false" hidden="false" name="capt_medios_grandes" vbProcedure="false">Supuestos!$E$91:$G$91</definedName>
+    <definedName function="false" hidden="false" name="capt_organismos" vbProcedure="false">Supuestos!$E$95:$G$95</definedName>
+    <definedName function="false" hidden="false" name="capt_universidades" vbProcedure="false">Supuestos!$E$94:$G$94</definedName>
+    <definedName function="false" hidden="false" name="capt_verificadores" vbProcedure="false">Supuestos!$E$93:$G$93</definedName>
     <definedName function="false" hidden="false" name="cargas_sociales" vbProcedure="false">Supuestos!$D$29</definedName>
-    <definedName function="false" hidden="false" name="churn_agencias" vbProcedure="false">Supuestos!$E$98:$G$98</definedName>
-    <definedName function="false" hidden="false" name="churn_medios_chicos" vbProcedure="false">Supuestos!$E$95:$G$95</definedName>
-    <definedName function="false" hidden="false" name="churn_medios_grandes" vbProcedure="false">Supuestos!$E$94:$G$94</definedName>
-    <definedName function="false" hidden="false" name="churn_universidades" vbProcedure="false">Supuestos!$E$97:$G$97</definedName>
-    <definedName function="false" hidden="false" name="churn_verificadores" vbProcedure="false">Supuestos!$E$96:$G$96</definedName>
+    <definedName function="false" hidden="false" name="churn_agencias" vbProcedure="false">Supuestos!$E$101:$G$101</definedName>
+    <definedName function="false" hidden="false" name="churn_medios_chicos" vbProcedure="false">Supuestos!$E$98:$G$98</definedName>
+    <definedName function="false" hidden="false" name="churn_medios_grandes" vbProcedure="false">Supuestos!$E$97:$G$97</definedName>
+    <definedName function="false" hidden="false" name="churn_universidades" vbProcedure="false">Supuestos!$E$100:$G$100</definedName>
+    <definedName function="false" hidden="false" name="churn_verificadores" vbProcedure="false">Supuestos!$E$99:$G$99</definedName>
     <definedName function="false" hidden="false" name="consultas_ent_mes" vbProcedure="false">Supuestos!$E$71:$G$71</definedName>
     <definedName function="false" hidden="false" name="consultas_pro_mes" vbProcedure="false">Supuestos!$E$70:$G$70</definedName>
     <definedName function="false" hidden="false" name="costo_analisis" vbProcedure="false">Supuestos!$E$61:$G$61</definedName>
     <definedName function="false" hidden="false" name="crecimiento_perpetuo" vbProcedure="false">Supuestos!$D$21</definedName>
     <definedName function="false" hidden="false" name="crp_argentina" vbProcedure="false">Supuestos!$D$19</definedName>
+    <definedName function="false" hidden="false" name="cuota_intermedia" vbProcedure="false">Supuestos!$D$72</definedName>
+    <definedName function="false" hidden="false" name="cuota_superior" vbProcedure="false">Supuestos!$D$73</definedName>
     <definedName function="false" hidden="false" name="dominio_anual" vbProcedure="false">Supuestos!$D$46</definedName>
     <definedName function="false" hidden="false" name="erp_maduro" vbProcedure="false">Supuestos!$D$18</definedName>
     <definedName function="false" hidden="false" name="horizonte" vbProcedure="false">Supuestos!$D$5</definedName>
@@ -51,20 +53,21 @@
     <definedName function="false" hidden="false" name="meses_anio" vbProcedure="false">Supuestos!$D$7</definedName>
     <definedName function="false" hidden="false" name="meses_anio_0" vbProcedure="false">Supuestos!$D$30</definedName>
     <definedName function="false" hidden="false" name="meses_cobro" vbProcedure="false">Supuestos!$D$34</definedName>
-    <definedName function="false" hidden="false" name="precio_agencias" vbProcedure="false">Supuestos!$E$86:$G$86</definedName>
+    <definedName function="false" hidden="false" name="precio_agencias" vbProcedure="false">Supuestos!$E$89:$G$89</definedName>
     <definedName function="false" hidden="false" name="precio_busqueda" vbProcedure="false">Supuestos!$D$56</definedName>
     <definedName function="false" hidden="false" name="precio_entrada" vbProcedure="false">Supuestos!$D$54</definedName>
-    <definedName function="false" hidden="false" name="precio_medios_chicos" vbProcedure="false">Supuestos!$D$82</definedName>
-    <definedName function="false" hidden="false" name="precio_medios_grandes" vbProcedure="false">Supuestos!$E$81:$G$81</definedName>
-    <definedName function="false" hidden="false" name="precio_organismos" vbProcedure="false">Supuestos!$E$85:$G$85</definedName>
+    <definedName function="false" hidden="false" name="precio_excedente" vbProcedure="false">Supuestos!$D$74</definedName>
+    <definedName function="false" hidden="false" name="precio_medios_chicos" vbProcedure="false">Supuestos!$D$85</definedName>
+    <definedName function="false" hidden="false" name="precio_medios_grandes" vbProcedure="false">Supuestos!$E$84:$G$84</definedName>
+    <definedName function="false" hidden="false" name="precio_organismos" vbProcedure="false">Supuestos!$E$88:$G$88</definedName>
     <definedName function="false" hidden="false" name="precio_salida" vbProcedure="false">Supuestos!$D$55</definedName>
-    <definedName function="false" hidden="false" name="precio_universidades" vbProcedure="false">Supuestos!$D$84</definedName>
-    <definedName function="false" hidden="false" name="precio_verificadores" vbProcedure="false">Supuestos!$D$83</definedName>
+    <definedName function="false" hidden="false" name="precio_universidades" vbProcedure="false">Supuestos!$D$87</definedName>
+    <definedName function="false" hidden="false" name="precio_verificadores" vbProcedure="false">Supuestos!$D$86</definedName>
     <definedName function="false" hidden="false" name="prima_proyecto" vbProcedure="false">Supuestos!$D$16</definedName>
     <definedName function="false" hidden="false" name="riesgo_pais" vbProcedure="false">Supuestos!$D$15</definedName>
-    <definedName function="false" hidden="false" name="sens_captacion" vbProcedure="false">Supuestos!$D$103</definedName>
-    <definedName function="false" hidden="false" name="sens_costo_analisis" vbProcedure="false">Supuestos!$D$101</definedName>
-    <definedName function="false" hidden="false" name="sens_precios" vbProcedure="false">Supuestos!$D$102</definedName>
+    <definedName function="false" hidden="false" name="sens_captacion" vbProcedure="false">Supuestos!$D$106</definedName>
+    <definedName function="false" hidden="false" name="sens_costo_analisis" vbProcedure="false">Supuestos!$D$104</definedName>
+    <definedName function="false" hidden="false" name="sens_precios" vbProcedure="false">Supuestos!$D$105</definedName>
     <definedName function="false" hidden="false" name="sueldos_por_anio" vbProcedure="false">Supuestos!$D$27</definedName>
     <definedName function="false" hidden="false" name="sueldo_ars" vbProcedure="false">Supuestos!$D$24</definedName>
     <definedName function="false" hidden="false" name="sueldo_usd" vbProcedure="false">Supuestos!$D$26</definedName>
@@ -78,15 +81,15 @@
     <definedName function="false" hidden="false" name="tokens_salida" vbProcedure="false">Supuestos!$E$59:$G$59</definedName>
     <definedName function="false" hidden="false" name="tope_mensual" vbProcedure="false">Supuestos!$D$68</definedName>
     <definedName function="false" hidden="false" name="ua_escalado" vbProcedure="false">Supuestos!$D$45</definedName>
-    <definedName function="false" hidden="false" name="ua_inicio_b2b" vbProcedure="false">Supuestos!$D$87</definedName>
+    <definedName function="false" hidden="false" name="ua_inicio_b2b" vbProcedure="false">Supuestos!$D$90</definedName>
     <definedName function="false" hidden="false" name="usuarios_activos" vbProcedure="false">Supuestos!$E$62:$G$66</definedName>
-    <definedName function="false" hidden="false" name="u_agencias" vbProcedure="false">Supuestos!$D$80</definedName>
-    <definedName function="false" hidden="false" name="u_medios_chicos" vbProcedure="false">Supuestos!$D$76</definedName>
-    <definedName function="false" hidden="false" name="u_medios_grandes" vbProcedure="false">Supuestos!$D$75</definedName>
-    <definedName function="false" hidden="false" name="u_medios_total" vbProcedure="false">Supuestos!$D$74</definedName>
-    <definedName function="false" hidden="false" name="u_organismos" vbProcedure="false">Supuestos!$D$79</definedName>
-    <definedName function="false" hidden="false" name="u_universidades" vbProcedure="false">Supuestos!$D$78</definedName>
-    <definedName function="false" hidden="false" name="u_verificadores" vbProcedure="false">Supuestos!$D$77</definedName>
+    <definedName function="false" hidden="false" name="u_agencias" vbProcedure="false">Supuestos!$D$83</definedName>
+    <definedName function="false" hidden="false" name="u_medios_chicos" vbProcedure="false">Supuestos!$D$79</definedName>
+    <definedName function="false" hidden="false" name="u_medios_grandes" vbProcedure="false">Supuestos!$D$78</definedName>
+    <definedName function="false" hidden="false" name="u_medios_total" vbProcedure="false">Supuestos!$D$77</definedName>
+    <definedName function="false" hidden="false" name="u_organismos" vbProcedure="false">Supuestos!$D$82</definedName>
+    <definedName function="false" hidden="false" name="u_universidades" vbProcedure="false">Supuestos!$D$81</definedName>
+    <definedName function="false" hidden="false" name="u_verificadores" vbProcedure="false">Supuestos!$D$80</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -98,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="337">
   <si>
     <t xml:space="preserve">clave</t>
   </si>
@@ -544,10 +547,10 @@
     <t xml:space="preserve">tope_mensual</t>
   </si>
   <si>
-    <t xml:space="preserve">Tope de análisis gratuitos por usuario por mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decisión de producto</t>
+    <t xml:space="preserve">Tope de análisis a demanda nuevos por instalación por mes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decisión de producto (RF-17)</t>
   </si>
   <si>
     <t xml:space="preserve">tasa_reuso</t>
@@ -559,7 +562,7 @@
     <t xml:space="preserve">consultas_pro_mes</t>
   </si>
   <si>
-    <t xml:space="preserve">Consultas por cliente API Pro por mes (uso parcial de la cuota)</t>
+    <t xml:space="preserve">Demanda de consultas por cliente de la API intermedia por mes (se costea hasta la cuota)</t>
   </si>
   <si>
     <t xml:space="preserve">consultas</t>
@@ -568,7 +571,31 @@
     <t xml:space="preserve">consultas_ent_mes</t>
   </si>
   <si>
-    <t xml:space="preserve">Consultas por cliente API Enterprise por mes</t>
+    <t xml:space="preserve">Demanda de consultas por cliente de la API superior por mes (se costea hasta la cuota)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuota_intermedia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuota mensual incluida en la API intermedia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap. 3, tab:pricing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cuota_superior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuota mensual incluida en la API superior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">precio_excedente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio por consulta excedente sobre la cuota (no se modela)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD/consulta</t>
   </si>
   <si>
     <t xml:space="preserve">Clientes B2B</t>
@@ -643,9 +670,6 @@
     <t xml:space="preserve">Precio: API nivel superior, medios de gran porte</t>
   </si>
   <si>
-    <t xml:space="preserve">Cap. 3, tab:pricing</t>
-  </si>
-  <si>
     <t xml:space="preserve">precio_medios_chicos</t>
   </si>
   <si>
@@ -827,6 +851,63 @@
   </si>
   <si>
     <t xml:space="preserve">Tasa CAPM de contraste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen mensual por cliente a cuota llena (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API intermedia: costo variable a cuota llena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API intermedia: margen a cuota llena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API superior: costo variable a cuota llena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API superior: margen a cuota llena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Economía unitaria, escenario neutral (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precio mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costo variable mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Margen mensual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Churn anual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTV/CAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payback del CAC (meses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAC (USD por alta de suscripción)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unitaria: Medios de gran porte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unitaria: Medios socios de ADEPA (resto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unitaria: Verificadores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unitaria: Universidades y observatorios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unitaria: Agencias</t>
   </si>
   <si>
     <t xml:space="preserve">Escenario optimista (USD nominales; todo lo derivado es fórmula)</t>
@@ -1377,7 +1458,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -2490,74 +2571,74 @@
         <v>17</v>
       </c>
     </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="B72" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="C72" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="D72" s="0" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H72" s="0" t="s">
+        <v>159</v>
+      </c>
+    </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="s">
-        <v>157</v>
+      <c r="A73" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="B73" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="C73" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="D73" s="0" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H73" s="0" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B74" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="C74" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="D74" s="0" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H74" s="0" t="s">
         <v>159</v>
       </c>
-      <c r="C74" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="D74" s="0" t="n">
-        <v>130</v>
-      </c>
-      <c r="H74" s="0" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="B75" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="C75" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="D75" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="H75" s="0" t="s">
-        <v>164</v>
-      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0" t="s">
+      <c r="A76" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B76" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="C76" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="D76" s="0" t="n">
-        <v>93</v>
-      </c>
-      <c r="H76" s="0" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="B77" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="B77" s="0" t="s">
+      <c r="C77" s="0" t="s">
         <v>168</v>
       </c>
-      <c r="C77" s="0" t="s">
-        <v>160</v>
-      </c>
       <c r="D77" s="0" t="n">
-        <v>3</v>
+        <v>130</v>
       </c>
       <c r="H77" s="0" t="s">
         <v>169</v>
@@ -2571,10 +2652,10 @@
         <v>171</v>
       </c>
       <c r="C78" s="0" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>149</v>
+        <v>10</v>
       </c>
       <c r="H78" s="0" t="s">
         <v>172</v>
@@ -2588,70 +2669,64 @@
         <v>174</v>
       </c>
       <c r="C79" s="0" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>32</v>
+        <v>93</v>
       </c>
       <c r="H79" s="0" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="B80" s="0" t="s">
         <v>176</v>
       </c>
-      <c r="B80" s="0" t="s">
+      <c r="C80" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="D80" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H80" s="0" t="s">
         <v>177</v>
-      </c>
-      <c r="C80" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="D80" s="0" t="n">
-        <v>120</v>
-      </c>
-      <c r="H80" s="0" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="B81" s="0" t="s">
         <v>179</v>
       </c>
-      <c r="B81" s="0" t="s">
+      <c r="C81" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="D81" s="0" t="n">
+        <v>149</v>
+      </c>
+      <c r="H81" s="0" t="s">
         <v>180</v>
-      </c>
-      <c r="C81" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="E81" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F81" s="0" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G81" s="0" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H81" s="0" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="B82" s="0" t="s">
         <v>182</v>
       </c>
-      <c r="B82" s="0" t="s">
+      <c r="C82" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="D82" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="H82" s="0" t="s">
         <v>183</v>
-      </c>
-      <c r="C82" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="D82" s="0" t="n">
-        <v>200</v>
-      </c>
-      <c r="H82" s="0" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2662,53 +2737,53 @@
         <v>185</v>
       </c>
       <c r="C83" s="0" t="s">
-        <v>65</v>
+        <v>168</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>500</v>
+        <v>120</v>
       </c>
       <c r="H83" s="0" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C84" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="D84" s="0" t="n">
-        <v>100</v>
+      <c r="E84" s="0" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F84" s="0" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G84" s="0" t="n">
+        <v>1500</v>
       </c>
       <c r="H84" s="0" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>190</v>
-      </c>
-      <c r="E85" s="0" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F85" s="0" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G85" s="0" t="n">
-        <v>10000</v>
+        <v>65</v>
+      </c>
+      <c r="D85" s="0" t="n">
+        <v>200</v>
       </c>
       <c r="H85" s="0" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2721,17 +2796,11 @@
       <c r="C86" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="E86" s="0" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F86" s="0" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G86" s="0" t="n">
-        <v>1500</v>
+      <c r="D86" s="0" t="n">
+        <v>500</v>
       </c>
       <c r="H86" s="0" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2742,13 +2811,13 @@
         <v>194</v>
       </c>
       <c r="C87" s="0" t="s">
-        <v>105</v>
+        <v>65</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>5000</v>
+        <v>100</v>
       </c>
       <c r="H87" s="0" t="s">
-        <v>17</v>
+        <v>159</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2759,62 +2828,56 @@
         <v>196</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>33</v>
+        <v>197</v>
       </c>
       <c r="E88" s="0" t="n">
-        <v>0.2</v>
+        <v>30000</v>
       </c>
       <c r="F88" s="0" t="n">
-        <v>0.1</v>
+        <v>20000</v>
       </c>
       <c r="G88" s="0" t="n">
-        <v>0.05</v>
+        <v>10000</v>
       </c>
       <c r="H88" s="0" t="s">
-        <v>17</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B89" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C89" s="0" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="E89" s="0" t="n">
-        <v>0.1</v>
+        <v>3000</v>
       </c>
       <c r="F89" s="0" t="n">
-        <v>0.05</v>
+        <v>2500</v>
       </c>
       <c r="G89" s="0" t="n">
-        <v>0.02</v>
+        <v>1500</v>
       </c>
       <c r="H89" s="0" t="s">
-        <v>17</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B90" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="E90" s="0" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F90" s="0" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G90" s="0" t="n">
-        <v>0.2</v>
+        <v>105</v>
+      </c>
+      <c r="D90" s="0" t="n">
+        <v>5000</v>
       </c>
       <c r="H90" s="0" t="s">
         <v>17</v>
@@ -2822,22 +2885,22 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B91" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C91" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E91" s="0" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="F91" s="0" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="G91" s="0" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="H91" s="0" t="s">
         <v>17</v>
@@ -2845,10 +2908,10 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C92" s="0" t="s">
         <v>33</v>
@@ -2857,10 +2920,10 @@
         <v>0.1</v>
       </c>
       <c r="F92" s="0" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="G92" s="0" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="H92" s="0" t="s">
         <v>17</v>
@@ -2868,22 +2931,22 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B93" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C93" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E93" s="0" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
       <c r="F93" s="0" t="n">
-        <v>0.02</v>
+        <v>0.3</v>
       </c>
       <c r="G93" s="0" t="n">
-        <v>0.01</v>
+        <v>0.2</v>
       </c>
       <c r="H93" s="0" t="s">
         <v>17</v>
@@ -2891,22 +2954,22 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B94" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C94" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E94" s="0" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F94" s="0" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="G94" s="0" t="n">
-        <v>0.25</v>
+        <v>0.02</v>
       </c>
       <c r="H94" s="0" t="s">
         <v>17</v>
@@ -2914,22 +2977,22 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C95" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E95" s="0" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F95" s="0" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="G95" s="0" t="n">
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="H95" s="0" t="s">
         <v>17</v>
@@ -2937,22 +3000,22 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B96" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C96" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E96" s="0" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="F96" s="0" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="G96" s="0" t="n">
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="H96" s="0" t="s">
         <v>17</v>
@@ -2960,22 +3023,22 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B97" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C97" s="0" t="s">
         <v>33</v>
       </c>
       <c r="E97" s="0" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F97" s="0" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="G97" s="0" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="H97" s="0" t="s">
         <v>17</v>
@@ -2983,10 +3046,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B98" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C98" s="0" t="s">
         <v>33</v>
@@ -3004,59 +3067,128 @@
         <v>17</v>
       </c>
     </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="0" t="s">
+        <v>218</v>
+      </c>
+      <c r="B99" s="0" t="s">
+        <v>219</v>
+      </c>
+      <c r="C99" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E99" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G99" s="0" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H99" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="1" t="s">
-        <v>217</v>
+      <c r="A100" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="B100" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="C100" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E100" s="0" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F100" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G100" s="0" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H100" s="0" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="0" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B101" s="0" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C101" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="D101" s="0" t="n">
-        <v>1</v>
+        <v>33</v>
+      </c>
+      <c r="E101" s="0" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F101" s="0" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G101" s="0" t="n">
+        <v>0.3</v>
       </c>
       <c r="H101" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="B104" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="C104" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="D104" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H104" s="0" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="0" t="s">
-        <v>221</v>
-      </c>
-      <c r="B102" s="0" t="s">
-        <v>222</v>
-      </c>
-      <c r="C102" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="D102" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H102" s="0" t="s">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="B105" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="C105" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="D105" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H105" s="0" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0" t="s">
-        <v>223</v>
-      </c>
-      <c r="B103" s="0" t="s">
-        <v>224</v>
-      </c>
-      <c r="C103" s="0" t="s">
-        <v>220</v>
-      </c>
-      <c r="D103" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H103" s="0" t="s">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="B106" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="C106" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="D106" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H106" s="0" t="s">
         <v>21</v>
       </c>
     </row>
@@ -3076,7 +3208,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -3084,21 +3216,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B2" s="0" t="n">
         <f aca="false">Optimista!B74</f>
@@ -3110,12 +3242,12 @@
       </c>
       <c r="D2" s="0" t="n">
         <f aca="false">Pesimista!B74</f>
-        <v>-134903.452188607</v>
+        <v>-94161.0656562552</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B3" s="2" t="n">
         <f aca="false">Optimista!B75</f>
@@ -3132,7 +3264,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">Optimista!B76</f>
@@ -3149,7 +3281,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">Optimista!B77</f>
@@ -3166,7 +3298,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B6" s="0" t="n">
         <f aca="false">Optimista!B80</f>
@@ -3178,12 +3310,12 @@
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">Pesimista!B80</f>
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B7" s="0" t="n">
         <f aca="false">Optimista!B79</f>
@@ -3200,7 +3332,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">Optimista!B78</f>
@@ -3212,17 +3344,17 @@
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">Pesimista!B78</f>
-        <v>-134903.452188607</v>
+        <v>-94161.0656562552</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">meses_anio*(u_medios_grandes*INDEX(precio_medios_grandes,1,2)+(u_medios_total-u_medios_grandes)*precio_medios_chicos+u_verificadores*precio_verificadores+u_universidades*precio_universidades+u_agencias*INDEX(precio_agencias,1,2))+u_organismos*INDEX(precio_organismos,1,2)</f>
@@ -3231,7 +3363,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">meses_anio*(u_medios_grandes*INDEX(precio_medios_grandes,1,2)+u_medios_chicos*precio_medios_chicos+u_verificadores*precio_verificadores+u_universidades*precio_universidades+u_agencias*INDEX(precio_agencias,1,2))+u_organismos*INDEX(precio_organismos,1,2)</f>
@@ -3240,7 +3372,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="B13" s="0" t="n">
         <f aca="false">Neutral!G45</f>
@@ -3249,12 +3381,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">meses_anio_0*sueldo_usd*(1+cargas_sociales)*sueldos_por_anio/meses_anio</f>
@@ -3263,11 +3395,293 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">tasa_capm</f>
         <v>0.1911</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>251</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <f aca="false">cuota_intermedia*(1-INDEX(tasa_reuso,1,1))*INDEX(costo_analisis,1,1)*sens_costo_analisis</f>
+        <v>38.232</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <f aca="false">cuota_intermedia*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>86.254</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <f aca="false">cuota_intermedia*(1-INDEX(tasa_reuso,1,3))*INDEX(costo_analisis,1,3)*sens_costo_analisis</f>
+        <v>151.856</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="B21" s="0" t="n">
+        <f aca="false">precio_medios_chicos*sens_precios-cuota_intermedia*(1-INDEX(tasa_reuso,1,1))*INDEX(costo_analisis,1,1)*sens_costo_analisis</f>
+        <v>161.768</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <f aca="false">precio_medios_chicos*sens_precios-cuota_intermedia*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>113.746</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <f aca="false">precio_medios_chicos*sens_precios-cuota_intermedia*(1-INDEX(tasa_reuso,1,3))*INDEX(costo_analisis,1,3)*sens_costo_analisis</f>
+        <v>48.144</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="B22" s="0" t="n">
+        <f aca="false">cuota_superior*(1-INDEX(tasa_reuso,1,1))*INDEX(costo_analisis,1,1)*sens_costo_analisis</f>
+        <v>305.856</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <f aca="false">cuota_superior*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>690.032</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <f aca="false">cuota_superior*(1-INDEX(tasa_reuso,1,3))*INDEX(costo_analisis,1,3)*sens_costo_analisis</f>
+        <v>1214.848</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="B23" s="0" t="n">
+        <f aca="false">INDEX(precio_medios_grandes,1,1)*sens_precios-cuota_superior*(1-INDEX(tasa_reuso,1,1))*INDEX(costo_analisis,1,1)*sens_costo_analisis</f>
+        <v>2694.144</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <f aca="false">INDEX(precio_medios_grandes,1,2)*sens_precios-cuota_superior*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>1809.968</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <f aca="false">INDEX(precio_medios_grandes,1,3)*sens_precios-cuota_superior*(1-INDEX(tasa_reuso,1,3))*INDEX(costo_analisis,1,3)*sens_costo_analisis</f>
+        <v>285.152</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="G25" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>263</v>
+      </c>
+      <c r="B26" s="0" t="n">
+        <f aca="false">SUM(Neutral!C50:G50)/(SUM(Neutral!C12:G12)+SUM(Neutral!C17:G17)+SUM(Neutral!C22:G22)+SUM(Neutral!C27:G27)+SUM(Neutral!C32:G32))</f>
+        <v>740.740740740741</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>264</v>
+      </c>
+      <c r="B27" s="0" t="n">
+        <f aca="false">INDEX(precio_medios_grandes,1,2)*sens_precios</f>
+        <v>2500</v>
+      </c>
+      <c r="C27" s="0" t="n">
+        <f aca="false">MIN(INDEX(consultas_ent_mes,1,2),cuota_superior)*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>690.032</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <f aca="false">B27-C27</f>
+        <v>1809.968</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <f aca="false">INDEX(churn_medios_grandes,1,2)</f>
+        <v>0.15</v>
+      </c>
+      <c r="F27" s="0" t="n">
+        <f aca="false">D27*meses_anio/E27</f>
+        <v>144797.44</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <f aca="false">F27/$B$26</f>
+        <v>195.476544</v>
+      </c>
+      <c r="H27" s="0" t="n">
+        <f aca="false">$B$26/D27</f>
+        <v>0.40925626350341</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="B28" s="0" t="n">
+        <f aca="false">precio_medios_chicos*sens_precios</f>
+        <v>200</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <f aca="false">MIN(INDEX(consultas_pro_mes,1,2),cuota_intermedia)*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>69.0032</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <f aca="false">B28-C28</f>
+        <v>130.9968</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <f aca="false">INDEX(churn_medios_chicos,1,2)</f>
+        <v>0.2</v>
+      </c>
+      <c r="F28" s="0" t="n">
+        <f aca="false">D28*meses_anio/E28</f>
+        <v>7859.808</v>
+      </c>
+      <c r="G28" s="0" t="n">
+        <f aca="false">F28/$B$26</f>
+        <v>10.6107408</v>
+      </c>
+      <c r="H28" s="0" t="n">
+        <f aca="false">$B$26/D28</f>
+        <v>5.6546476000997</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>266</v>
+      </c>
+      <c r="B29" s="0" t="n">
+        <f aca="false">precio_verificadores*sens_precios</f>
+        <v>500</v>
+      </c>
+      <c r="C29" s="0" t="n">
+        <f aca="false">MIN(INDEX(consultas_pro_mes,1,2),cuota_intermedia)*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>69.0032</v>
+      </c>
+      <c r="D29" s="0" t="n">
+        <f aca="false">B29-C29</f>
+        <v>430.9968</v>
+      </c>
+      <c r="E29" s="0" t="n">
+        <f aca="false">INDEX(churn_verificadores,1,2)</f>
+        <v>0.1</v>
+      </c>
+      <c r="F29" s="0" t="n">
+        <f aca="false">D29*meses_anio/E29</f>
+        <v>51719.616</v>
+      </c>
+      <c r="G29" s="0" t="n">
+        <f aca="false">F29/$B$26</f>
+        <v>69.8214816</v>
+      </c>
+      <c r="H29" s="0" t="n">
+        <f aca="false">$B$26/D29</f>
+        <v>1.71866877141719</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>267</v>
+      </c>
+      <c r="B30" s="0" t="n">
+        <f aca="false">precio_universidades*sens_precios</f>
+        <v>100</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <f aca="false">0*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="0" t="n">
+        <f aca="false">B30-C30</f>
+        <v>100</v>
+      </c>
+      <c r="E30" s="0" t="n">
+        <f aca="false">INDEX(churn_universidades,1,2)</f>
+        <v>0.1</v>
+      </c>
+      <c r="F30" s="0" t="n">
+        <f aca="false">D30*meses_anio/E30</f>
+        <v>12000</v>
+      </c>
+      <c r="G30" s="0" t="n">
+        <f aca="false">F30/$B$26</f>
+        <v>16.2</v>
+      </c>
+      <c r="H30" s="0" t="n">
+        <f aca="false">$B$26/D30</f>
+        <v>7.40740740740741</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>268</v>
+      </c>
+      <c r="B31" s="0" t="n">
+        <f aca="false">INDEX(precio_agencias,1,2)*sens_precios</f>
+        <v>2500</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <f aca="false">MIN(INDEX(consultas_ent_mes,1,2),cuota_superior)*(1-INDEX(tasa_reuso,1,2))*INDEX(costo_analisis,1,2)*sens_costo_analisis</f>
+        <v>690.032</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <f aca="false">B31-C31</f>
+        <v>1809.968</v>
+      </c>
+      <c r="E31" s="0" t="n">
+        <f aca="false">INDEX(churn_agencias,1,2)</f>
+        <v>0.2</v>
+      </c>
+      <c r="F31" s="0" t="n">
+        <f aca="false">D31*meses_anio/E31</f>
+        <v>108598.08</v>
+      </c>
+      <c r="G31" s="0" t="n">
+        <f aca="false">F31/$B$26</f>
+        <v>146.607408</v>
+      </c>
+      <c r="H31" s="0" t="n">
+        <f aca="false">$B$26/D31</f>
+        <v>0.40925626350341</v>
       </c>
     </row>
   </sheetData>
@@ -3294,12 +3708,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>243</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>1</v>
@@ -3307,7 +3721,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>245</v>
+        <v>271</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -3336,7 +3750,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -3365,7 +3779,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -3394,7 +3808,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>248</v>
+        <v>274</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -3419,7 +3833,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">IF(C6&gt;=ua_inicio_b2b,1,0)</f>
@@ -3444,12 +3858,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -3474,7 +3888,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -3499,7 +3913,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>252</v>
+        <v>278</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_medios_grandes,1,$B$2)*sens_captacion*(u_medios_grandes-C10),0)</f>
@@ -3524,7 +3938,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>253</v>
+        <v>279</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -3549,7 +3963,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>254</v>
+        <v>280</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -3574,7 +3988,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>255</v>
+        <v>281</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -3599,7 +4013,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>256</v>
+        <v>282</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -3624,7 +4038,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>257</v>
+        <v>283</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_medios_chicos,1,$B$2)*sens_captacion*(u_medios_chicos-C15),0)</f>
@@ -3649,7 +4063,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>258</v>
+        <v>284</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -3674,7 +4088,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>259</v>
+        <v>285</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -3699,7 +4113,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -3724,7 +4138,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -3749,7 +4163,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_verificadores,1,$B$2)*sens_captacion*(u_verificadores-C20),0)</f>
@@ -3774,7 +4188,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>263</v>
+        <v>289</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -3799,7 +4213,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>264</v>
+        <v>290</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -3824,7 +4238,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>265</v>
+        <v>291</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -3849,7 +4263,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>266</v>
+        <v>292</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -3874,7 +4288,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>267</v>
+        <v>293</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_universidades,1,$B$2)*sens_captacion*(u_universidades-C25),0)</f>
@@ -3899,7 +4313,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -3924,7 +4338,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>269</v>
+        <v>295</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -3949,7 +4363,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>270</v>
+        <v>296</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -3974,7 +4388,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>271</v>
+        <v>297</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -3999,7 +4413,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>272</v>
+        <v>298</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_agencias,1,$B$2)*sens_captacion*(u_agencias-C30),0)</f>
@@ -4024,7 +4438,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>273</v>
+        <v>299</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -4049,7 +4463,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -4074,7 +4488,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C7*ROUND(INDEX(capt_organismos,1,$B$2)*sens_captacion*u_organismos,0)</f>
@@ -4099,7 +4513,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -4124,12 +4538,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>277</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>278</v>
+        <v>304</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*sens_precios*meses_anio</f>
@@ -4154,7 +4568,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>279</v>
+        <v>305</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*sens_precios*meses_anio</f>
@@ -4179,7 +4593,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>280</v>
+        <v>306</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*sens_precios*meses_anio</f>
@@ -4204,7 +4618,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>281</v>
+        <v>307</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*sens_precios*meses_anio</f>
@@ -4229,7 +4643,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>282</v>
+        <v>308</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*sens_precios*meses_anio</f>
@@ -4254,7 +4668,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>283</v>
+        <v>309</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)*sens_precios</f>
@@ -4279,7 +4693,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>284</v>
+        <v>310</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -4308,12 +4722,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>285</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>286</v>
+        <v>312</v>
       </c>
       <c r="C48" s="0" t="n">
         <f aca="false">sueldo_usd*sueldos_por_anio*(1+cargas_sociales)*(1+ajuste_sueldo)^C$3</f>
@@ -4338,7 +4752,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -4367,7 +4781,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>288</v>
+        <v>314</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -4392,7 +4806,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="B51" s="0" t="n">
         <f aca="false">inv_dominio+inv_marca_inpi+inv_legal</f>
@@ -4401,7 +4815,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>290</v>
+        <v>316</v>
       </c>
       <c r="C52" s="0" t="n">
         <f aca="false">C6*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
@@ -4426,32 +4840,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>291</v>
+        <v>317</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((C19+C24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(C14+C34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>8258.112</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((D19+D24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(D14+D34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>23673.2544</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((E19+E24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(E14+E34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>35051.0976</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((F19+F24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(F14+F34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>42391.6416</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((G19+G24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(G14+G34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>47621.7792</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>292</v>
+        <v>318</v>
       </c>
       <c r="B54" s="0" t="n">
         <f aca="false">SUM(B48:B53)</f>
@@ -4480,12 +4894,12 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>293</v>
+        <v>319</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>294</v>
+        <v>320</v>
       </c>
       <c r="B57" s="0" t="n">
         <f aca="false">B45-B54</f>
@@ -4514,7 +4928,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>295</v>
+        <v>321</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">MIN(0,B57)</f>
@@ -4543,7 +4957,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>296</v>
+        <v>322</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B57)</f>
@@ -4572,7 +4986,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>297</v>
+        <v>323</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">meses_cobro/meses_anio*B45</f>
@@ -4601,7 +5015,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>298</v>
+        <v>324</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B60</f>
@@ -4630,7 +5044,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>299</v>
+        <v>325</v>
       </c>
       <c r="G62" s="0" t="n">
         <f aca="false">G60</f>
@@ -4639,12 +5053,12 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>300</v>
+        <v>326</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>301</v>
+        <v>327</v>
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">B57-B59-B61+N(B62)</f>
@@ -4673,7 +5087,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>302</v>
+        <v>328</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -4702,7 +5116,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>303</v>
+        <v>329</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">B65*B66</f>
@@ -4731,7 +5145,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>304</v>
+        <v>330</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B65</f>
@@ -4760,7 +5174,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>305</v>
+        <v>331</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B67</f>
@@ -4789,7 +5203,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>306</v>
+        <v>332</v>
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">IF(AND(B68&lt;0,C68&gt;=0),C$3-1+(-B68)/C65,"")</f>
@@ -4814,7 +5228,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>307</v>
+        <v>333</v>
       </c>
       <c r="C71" s="0" t="n">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C67,"")</f>
@@ -4839,12 +5253,12 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>308</v>
+        <v>334</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">SUM(B67:G67)</f>
@@ -4853,7 +5267,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B75" s="2" t="n">
         <f aca="false">IFERROR(IRR(B65:G65),"no definida")</f>
@@ -4862,7 +5276,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B76" s="0" t="n">
         <f aca="false">IF(COUNT(C70:G70)=0,"no se recupera",MIN(C70:G70))</f>
@@ -4871,7 +5285,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
@@ -4880,7 +5294,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">SUM(B67:G67)+MAX(0,G65-G62)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
@@ -4889,7 +5303,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -4898,7 +5312,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B80" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G54/B79,0),"no definido")</f>
@@ -4929,12 +5343,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>309</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>2</v>
@@ -4942,7 +5356,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>245</v>
+        <v>271</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -4971,7 +5385,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -5000,7 +5414,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -5029,7 +5443,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>248</v>
+        <v>274</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -5054,7 +5468,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">IF(C6&gt;=ua_inicio_b2b,1,0)</f>
@@ -5079,12 +5493,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -5109,7 +5523,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -5134,7 +5548,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>252</v>
+        <v>278</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_medios_grandes,1,$B$2)*sens_captacion*(u_medios_grandes-C10),0)</f>
@@ -5159,7 +5573,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>253</v>
+        <v>279</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -5184,7 +5598,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>254</v>
+        <v>280</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -5209,7 +5623,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>255</v>
+        <v>281</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -5234,7 +5648,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>256</v>
+        <v>282</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -5259,7 +5673,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>257</v>
+        <v>283</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_medios_chicos,1,$B$2)*sens_captacion*(u_medios_chicos-C15),0)</f>
@@ -5284,7 +5698,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>258</v>
+        <v>284</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -5309,7 +5723,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>259</v>
+        <v>285</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -5334,7 +5748,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -5359,7 +5773,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -5384,7 +5798,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_verificadores,1,$B$2)*sens_captacion*(u_verificadores-C20),0)</f>
@@ -5409,7 +5823,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>263</v>
+        <v>289</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -5434,7 +5848,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>264</v>
+        <v>290</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -5459,7 +5873,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>265</v>
+        <v>291</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -5484,7 +5898,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>266</v>
+        <v>292</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -5509,7 +5923,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>267</v>
+        <v>293</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_universidades,1,$B$2)*sens_captacion*(u_universidades-C25),0)</f>
@@ -5534,7 +5948,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -5559,7 +5973,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>269</v>
+        <v>295</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -5584,7 +5998,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>270</v>
+        <v>296</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -5609,7 +6023,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>271</v>
+        <v>297</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -5634,7 +6048,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>272</v>
+        <v>298</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_agencias,1,$B$2)*sens_captacion*(u_agencias-C30),0)</f>
@@ -5659,7 +6073,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>273</v>
+        <v>299</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -5684,7 +6098,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -5709,7 +6123,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C7*ROUND(INDEX(capt_organismos,1,$B$2)*sens_captacion*u_organismos,0)</f>
@@ -5734,7 +6148,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -5759,12 +6173,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>277</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>278</v>
+        <v>304</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*sens_precios*meses_anio</f>
@@ -5789,7 +6203,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>279</v>
+        <v>305</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*sens_precios*meses_anio</f>
@@ -5814,7 +6228,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>280</v>
+        <v>306</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*sens_precios*meses_anio</f>
@@ -5839,7 +6253,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>281</v>
+        <v>307</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*sens_precios*meses_anio</f>
@@ -5864,7 +6278,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>282</v>
+        <v>308</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*sens_precios*meses_anio</f>
@@ -5889,7 +6303,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>283</v>
+        <v>309</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)*sens_precios</f>
@@ -5914,7 +6328,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>284</v>
+        <v>310</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -5943,12 +6357,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>285</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>286</v>
+        <v>312</v>
       </c>
       <c r="C48" s="0" t="n">
         <f aca="false">sueldo_usd*sueldos_por_anio*(1+cargas_sociales)*(1+ajuste_sueldo)^C$3</f>
@@ -5973,7 +6387,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -6002,7 +6416,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>288</v>
+        <v>314</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -6027,7 +6441,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="B51" s="0" t="n">
         <f aca="false">inv_dominio+inv_marca_inpi+inv_legal</f>
@@ -6036,7 +6450,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>290</v>
+        <v>316</v>
       </c>
       <c r="C52" s="0" t="n">
         <f aca="false">C6*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
@@ -6061,32 +6475,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>291</v>
+        <v>317</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((C19+C24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(C14+C34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>0</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((D19+D24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(D14+D34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>14904.6912</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((E19+E24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(E14+E34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>43886.0352</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((F19+F24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(F14+F34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>67071.1104</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((G19+G24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(G14+G34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>85287.9552</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>292</v>
+        <v>318</v>
       </c>
       <c r="B54" s="0" t="n">
         <f aca="false">SUM(B48:B53)</f>
@@ -6115,12 +6529,12 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>293</v>
+        <v>319</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>294</v>
+        <v>320</v>
       </c>
       <c r="B57" s="0" t="n">
         <f aca="false">B45-B54</f>
@@ -6149,7 +6563,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>295</v>
+        <v>321</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">MIN(0,B57)</f>
@@ -6178,7 +6592,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>296</v>
+        <v>322</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B57)</f>
@@ -6207,7 +6621,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>297</v>
+        <v>323</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">meses_cobro/meses_anio*B45</f>
@@ -6236,7 +6650,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>298</v>
+        <v>324</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B60</f>
@@ -6265,7 +6679,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>299</v>
+        <v>325</v>
       </c>
       <c r="G62" s="0" t="n">
         <f aca="false">G60</f>
@@ -6274,12 +6688,12 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>300</v>
+        <v>326</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>301</v>
+        <v>327</v>
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">B57-B59-B61+N(B62)</f>
@@ -6308,7 +6722,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>302</v>
+        <v>328</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -6337,7 +6751,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>303</v>
+        <v>329</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">B65*B66</f>
@@ -6366,7 +6780,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>304</v>
+        <v>330</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B65</f>
@@ -6395,7 +6809,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>305</v>
+        <v>331</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B67</f>
@@ -6424,7 +6838,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>306</v>
+        <v>332</v>
       </c>
       <c r="C70" s="0" t="str">
         <f aca="false">IF(AND(B68&lt;0,C68&gt;=0),C$3-1+(-B68)/C65,"")</f>
@@ -6449,7 +6863,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>307</v>
+        <v>333</v>
       </c>
       <c r="C71" s="0" t="str">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C67,"")</f>
@@ -6474,12 +6888,12 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>308</v>
+        <v>334</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">SUM(B67:G67)</f>
@@ -6488,7 +6902,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B75" s="2" t="n">
         <f aca="false">IFERROR(IRR(B65:G65),"no definida")</f>
@@ -6497,7 +6911,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B76" s="0" t="n">
         <f aca="false">IF(COUNT(C70:G70)=0,"no se recupera",MIN(C70:G70))</f>
@@ -6506,7 +6920,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
@@ -6515,7 +6929,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">SUM(B67:G67)+MAX(0,G65-G62)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
@@ -6524,7 +6938,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -6533,7 +6947,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B80" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G54/B79,0),"no definido")</f>
@@ -6564,12 +6978,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>310</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>3</v>
@@ -6577,7 +6991,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>245</v>
+        <v>271</v>
       </c>
       <c r="B3" s="0" t="n">
         <f aca="false">COLUMN()-2</f>
@@ -6606,7 +7020,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">anio_0+B$3</f>
@@ -6635,7 +7049,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>247</v>
+        <v>273</v>
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">INDEX(anio_electoral,B$3+1)</f>
@@ -6664,7 +7078,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>248</v>
+        <v>274</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">INDEX(usuarios_activos,C$3,$B$2)</f>
@@ -6689,7 +7103,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="C7" s="0" t="n">
         <f aca="false">IF(C6&gt;=ua_inicio_b2b,1,0)</f>
@@ -6714,12 +7128,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">N(B13)</f>
@@ -6744,7 +7158,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_grandes,1,$B$2)*C10,0)</f>
@@ -6769,7 +7183,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>252</v>
+        <v>278</v>
       </c>
       <c r="C12" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_medios_grandes,1,$B$2)*sens_captacion*(u_medios_grandes-C10),0)</f>
@@ -6794,7 +7208,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>253</v>
+        <v>279</v>
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C10+C12-C11</f>
@@ -6819,7 +7233,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>254</v>
+        <v>280</v>
       </c>
       <c r="C14" s="0" t="n">
         <f aca="false">(C10+C13)/2</f>
@@ -6844,7 +7258,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>255</v>
+        <v>281</v>
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">N(B18)</f>
@@ -6869,7 +7283,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>256</v>
+        <v>282</v>
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_medios_chicos,1,$B$2)*C15,0)</f>
@@ -6894,7 +7308,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>257</v>
+        <v>283</v>
       </c>
       <c r="C17" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_medios_chicos,1,$B$2)*sens_captacion*(u_medios_chicos-C15),0)</f>
@@ -6919,7 +7333,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>258</v>
+        <v>284</v>
       </c>
       <c r="C18" s="0" t="n">
         <f aca="false">C15+C17-C16</f>
@@ -6944,7 +7358,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>259</v>
+        <v>285</v>
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">(C15+C18)/2</f>
@@ -6969,7 +7383,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>260</v>
+        <v>286</v>
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">N(B23)</f>
@@ -6994,7 +7408,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>261</v>
+        <v>287</v>
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_verificadores,1,$B$2)*C20,0)</f>
@@ -7019,7 +7433,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>262</v>
+        <v>288</v>
       </c>
       <c r="C22" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_verificadores,1,$B$2)*sens_captacion*(u_verificadores-C20),0)</f>
@@ -7044,7 +7458,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>263</v>
+        <v>289</v>
       </c>
       <c r="C23" s="0" t="n">
         <f aca="false">C20+C22-C21</f>
@@ -7069,7 +7483,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>264</v>
+        <v>290</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(C20+C23)/2</f>
@@ -7094,7 +7508,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>265</v>
+        <v>291</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">N(B28)</f>
@@ -7119,7 +7533,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>266</v>
+        <v>292</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_universidades,1,$B$2)*C25,0)</f>
@@ -7144,7 +7558,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>267</v>
+        <v>293</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_universidades,1,$B$2)*sens_captacion*(u_universidades-C25),0)</f>
@@ -7169,7 +7583,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">C25+C27-C26</f>
@@ -7194,7 +7608,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>269</v>
+        <v>295</v>
       </c>
       <c r="C29" s="0" t="n">
         <f aca="false">(C25+C28)/2</f>
@@ -7219,7 +7633,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>270</v>
+        <v>296</v>
       </c>
       <c r="C30" s="0" t="n">
         <f aca="false">N(B33)</f>
@@ -7244,7 +7658,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>271</v>
+        <v>297</v>
       </c>
       <c r="C31" s="0" t="n">
         <f aca="false">ROUND(INDEX(churn_agencias,1,$B$2)*C30,0)</f>
@@ -7269,7 +7683,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>272</v>
+        <v>298</v>
       </c>
       <c r="C32" s="0" t="n">
         <f aca="false">C7*ROUND(INDEX(capt_agencias,1,$B$2)*sens_captacion*(u_agencias-C30),0)</f>
@@ -7294,7 +7708,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>273</v>
+        <v>299</v>
       </c>
       <c r="C33" s="0" t="n">
         <f aca="false">C30+C32-C31</f>
@@ -7319,7 +7733,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>274</v>
+        <v>300</v>
       </c>
       <c r="C34" s="0" t="n">
         <f aca="false">(C30+C33)/2</f>
@@ -7344,7 +7758,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>275</v>
+        <v>301</v>
       </c>
       <c r="C35" s="0" t="n">
         <f aca="false">C5*C7*ROUND(INDEX(capt_organismos,1,$B$2)*sens_captacion*u_organismos,0)</f>
@@ -7369,7 +7783,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>276</v>
+        <v>302</v>
       </c>
       <c r="C36" s="0" t="n">
         <f aca="false">C14+C19+C24+C29+C34+C35</f>
@@ -7394,12 +7808,12 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>277</v>
+        <v>303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>278</v>
+        <v>304</v>
       </c>
       <c r="C39" s="0" t="n">
         <f aca="false">C14*INDEX(precio_medios_grandes,1,$B$2)*sens_precios*meses_anio</f>
@@ -7424,7 +7838,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>279</v>
+        <v>305</v>
       </c>
       <c r="C40" s="0" t="n">
         <f aca="false">C19*precio_medios_chicos*sens_precios*meses_anio</f>
@@ -7449,7 +7863,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>280</v>
+        <v>306</v>
       </c>
       <c r="C41" s="0" t="n">
         <f aca="false">C24*precio_verificadores*sens_precios*meses_anio</f>
@@ -7474,7 +7888,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>281</v>
+        <v>307</v>
       </c>
       <c r="C42" s="0" t="n">
         <f aca="false">C29*precio_universidades*sens_precios*meses_anio</f>
@@ -7499,7 +7913,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>282</v>
+        <v>308</v>
       </c>
       <c r="C43" s="0" t="n">
         <f aca="false">C34*INDEX(precio_agencias,1,$B$2)*sens_precios*meses_anio</f>
@@ -7524,7 +7938,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>283</v>
+        <v>309</v>
       </c>
       <c r="C44" s="0" t="n">
         <f aca="false">C35*INDEX(precio_organismos,1,$B$2)*sens_precios</f>
@@ -7549,7 +7963,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>284</v>
+        <v>310</v>
       </c>
       <c r="B45" s="0" t="n">
         <f aca="false">SUM(B39:B44)</f>
@@ -7578,12 +7992,12 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>285</v>
+        <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>286</v>
+        <v>312</v>
       </c>
       <c r="C48" s="0" t="n">
         <f aca="false">sueldo_usd*sueldos_por_anio*(1+cargas_sociales)*(1+ajuste_sueldo)^C$3</f>
@@ -7608,7 +8022,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="B49" s="0" t="n">
         <f aca="false">inv_infraestructura_0</f>
@@ -7637,7 +8051,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>288</v>
+        <v>314</v>
       </c>
       <c r="C50" s="0" t="n">
         <f aca="false">INDEX(marketing,C$3,$B$2)</f>
@@ -7662,7 +8076,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="B51" s="0" t="n">
         <f aca="false">inv_dominio+inv_marca_inpi+inv_legal</f>
@@ -7671,7 +8085,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>290</v>
+        <v>316</v>
       </c>
       <c r="C52" s="0" t="n">
         <f aca="false">C6*MIN(INDEX(analisis_por_ua_mes,1,$B$2),tope_mensual)*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
@@ -7696,32 +8110,32 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>291</v>
+        <v>317</v>
       </c>
       <c r="C53" s="0" t="n">
-        <f aca="false">((C19+C24)*INDEX(consultas_pro_mes,1,$B$2)+(C14+C34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((C19+C24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(C14+C34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>0</v>
       </c>
       <c r="D53" s="0" t="n">
-        <f aca="false">((D19+D24)*INDEX(consultas_pro_mes,1,$B$2)+(D14+D34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <f aca="false">((D19+D24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(D14+D34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
         <v>0</v>
       </c>
       <c r="E53" s="0" t="n">
-        <f aca="false">((E19+E24)*INDEX(consultas_pro_mes,1,$B$2)+(E14+E34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>33529.8048</v>
+        <f aca="false">((E19+E24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(E14+E34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>17311.584</v>
       </c>
       <c r="F53" s="0" t="n">
-        <f aca="false">((F19+F24)*INDEX(consultas_pro_mes,1,$B$2)+(F14+F34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>83095.6032</v>
+        <f aca="false">((F19+F24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(F14+F34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>42823.392</v>
       </c>
       <c r="G53" s="0" t="n">
-        <f aca="false">((G19+G24)*INDEX(consultas_pro_mes,1,$B$2)+(G14+G34)*INDEX(consultas_ent_mes,1,$B$2))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
-        <v>100589.4144</v>
+        <f aca="false">((G19+G24)*MIN(INDEX(consultas_pro_mes,1,$B$2),cuota_intermedia)+(G14+G34)*MIN(INDEX(consultas_ent_mes,1,$B$2),cuota_superior))*meses_anio*(1-INDEX(tasa_reuso,1,$B$2))*INDEX(costo_analisis,1,$B$2)*sens_costo_analisis</f>
+        <v>51934.752</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>292</v>
+        <v>318</v>
       </c>
       <c r="B54" s="0" t="n">
         <f aca="false">SUM(B48:B53)</f>
@@ -7737,25 +8151,25 @@
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">SUM(E48:E53)</f>
-        <v>80888.461325</v>
+        <v>64670.240525</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">SUM(F48:F53)</f>
-        <v>138654.16555125</v>
+        <v>98381.95435125</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">SUM(G48:G53)</f>
-        <v>162598.465068813</v>
+        <v>113943.802668813</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>293</v>
+        <v>319</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>294</v>
+        <v>320</v>
       </c>
       <c r="B57" s="0" t="n">
         <f aca="false">B45-B54</f>
@@ -7771,20 +8185,20 @@
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">E45-E54</f>
-        <v>-45688.461325</v>
+        <v>-29470.240525</v>
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">F45-F54</f>
-        <v>-76254.16555125</v>
+        <v>-35981.95435125</v>
       </c>
       <c r="G57" s="0" t="n">
         <f aca="false">G45-G54</f>
-        <v>-75798.4650688125</v>
+        <v>-27143.8026688125</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>295</v>
+        <v>321</v>
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">MIN(0,B57)</f>
@@ -7800,20 +8214,20 @@
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">MIN(0,D58+E57)</f>
-        <v>-120591.371825</v>
+        <v>-104373.151025</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">MIN(0,E58+F57)</f>
-        <v>-196845.53737625</v>
+        <v>-140355.10537625</v>
       </c>
       <c r="G58" s="0" t="n">
         <f aca="false">MIN(0,F58+G57)</f>
-        <v>-272644.002445063</v>
+        <v>-167498.908045063</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>296</v>
+        <v>322</v>
       </c>
       <c r="B59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B57)</f>
@@ -7842,7 +8256,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>297</v>
+        <v>323</v>
       </c>
       <c r="B60" s="0" t="n">
         <f aca="false">meses_cobro/meses_anio*B45</f>
@@ -7871,7 +8285,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>298</v>
+        <v>324</v>
       </c>
       <c r="B61" s="0" t="n">
         <f aca="false">B60</f>
@@ -7900,7 +8314,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="0" t="s">
-        <v>299</v>
+        <v>325</v>
       </c>
       <c r="G62" s="0" t="n">
         <f aca="false">G60</f>
@@ -7909,12 +8323,12 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>300</v>
+        <v>326</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>301</v>
+        <v>327</v>
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">B57-B59-B61+N(B62)</f>
@@ -7930,20 +8344,20 @@
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">E57-E59-E61+N(E62)</f>
-        <v>-51555.1279916667</v>
+        <v>-35336.9071916667</v>
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">F57-F59-F61+N(F62)</f>
-        <v>-80787.4988845833</v>
+        <v>-40515.2876845833</v>
       </c>
       <c r="G65" s="0" t="n">
         <f aca="false">G57-G59-G61+N(G62)</f>
-        <v>-65398.4650688125</v>
+        <v>-16743.8026688125</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>302</v>
+        <v>328</v>
       </c>
       <c r="B66" s="0" t="n">
         <f aca="false">1/(1+tasa_descuento)^B$3</f>
@@ -7972,7 +8386,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>303</v>
+        <v>329</v>
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">B65*B66</f>
@@ -7988,20 +8402,20 @@
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">E65*E66</f>
-        <v>-26396.2255317333</v>
+        <v>-18092.4964821333</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">F65*F66</f>
-        <v>-33090.5595431253</v>
+        <v>-16595.0618356053</v>
       </c>
       <c r="G67" s="0" t="n">
         <f aca="false">G65*G66</f>
-        <v>-21429.7690337485</v>
+        <v>-5486.60925851648</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="0" t="s">
-        <v>304</v>
+        <v>330</v>
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B65</f>
@@ -8017,20 +8431,20 @@
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">D68+E65</f>
-        <v>-126458.038491667</v>
+        <v>-110239.817691667</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">E68+F65</f>
-        <v>-207245.53737625</v>
+        <v>-150755.10537625</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">F68+G65</f>
-        <v>-272644.002445063</v>
+        <v>-167498.908045063</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>305</v>
+        <v>331</v>
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B67</f>
@@ -8046,20 +8460,20 @@
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E67</f>
-        <v>-80383.1236117333</v>
+        <v>-72079.3945621333</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F67</f>
-        <v>-113473.683154859</v>
+        <v>-88674.4563977387</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G67</f>
-        <v>-134903.452188607</v>
+        <v>-94161.0656562552</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>306</v>
+        <v>332</v>
       </c>
       <c r="C70" s="0" t="str">
         <f aca="false">IF(AND(B68&lt;0,C68&gt;=0),C$3-1+(-B68)/C65,"")</f>
@@ -8084,7 +8498,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
-        <v>307</v>
+        <v>333</v>
       </c>
       <c r="C71" s="0" t="str">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C67,"")</f>
@@ -8109,21 +8523,21 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>308</v>
+        <v>334</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">SUM(B67:G67)</f>
-        <v>-134903.452188607</v>
+        <v>-94161.0656562552</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B75" s="2" t="str">
         <f aca="false">IFERROR(IRR(B65:G65),"no definida")</f>
@@ -8132,7 +8546,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B76" s="0" t="str">
         <f aca="false">IF(COUNT(C70:G70)=0,"no se recupera",MIN(C70:G70))</f>
@@ -8141,7 +8555,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B77" s="0" t="str">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
@@ -8150,16 +8564,16 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="0" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">SUM(B67:G67)+MAX(0,G65-G62)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>-134903.452188607</v>
+        <v>-94161.0656562552</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B79" s="0" t="n">
         <f aca="false">IFERROR(G45/G36,"no definido")</f>
@@ -8168,11 +8582,11 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B80" s="0" t="n">
         <f aca="false">IFERROR(ROUNDUP(G54/B79,0),"no definido")</f>
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Usar fuentes primarias en el análisis financiero
- Tipo de cambio: Com. A 3500 del BCRA (1.528,76 ARS/USD al 28/09/2026)
  en lugar de El Cronista; dominio e INPI recalculados
- Riesgo país: cierre del EMBI según Rava Bursátil en lugar de Infobae
- Calendario electoral: solo la Constitución Nacional, sin La Nación
- Planilla regenerada y validada; tablas y sensibilidad reexportadas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -178,7 +178,7 @@
     <t xml:space="preserve">0/1</t>
   </si>
   <si>
-    <t xml:space="preserve">ConvencionConstituyente1994, LaNacion2026</t>
+    <t xml:space="preserve">ConvencionConstituyente1994</t>
   </si>
   <si>
     <t xml:space="preserve">Año 1 con elección nacional (1 = sí)</t>
@@ -214,7 +214,7 @@
     <t xml:space="preserve">Riesgo país de Argentina (EMBI, 628 pb)</t>
   </si>
   <si>
-    <t xml:space="preserve">Infobae2026</t>
+    <t xml:space="preserve">RavaBursatil2026</t>
   </si>
   <si>
     <t xml:space="preserve">prima_proyecto</t>
@@ -1975,7 +1975,7 @@
         <v>86</v>
       </c>
       <c r="D38" s="0" t="n">
-        <v>5.5</v>
+        <v>5.56</v>
       </c>
       <c r="H38" s="0" t="s">
         <v>90</v>
@@ -1992,7 +1992,7 @@
         <v>86</v>
       </c>
       <c r="D39" s="0" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H39" s="0" t="s">
         <v>93</v>
@@ -2082,7 +2082,7 @@
         <v>108</v>
       </c>
       <c r="D46" s="0" t="n">
-        <v>5.5</v>
+        <v>5.56</v>
       </c>
       <c r="H46" s="0" t="s">
         <v>90</v>
@@ -3234,15 +3234,15 @@
       </c>
       <c r="B2" s="0" t="n">
         <f aca="false">Optimista!B74</f>
-        <v>833353.475342681</v>
+        <v>833352.607260761</v>
       </c>
       <c r="C2" s="0" t="n">
         <f aca="false">Neutral!B74</f>
-        <v>63935.7622353104</v>
+        <v>63934.7785693904</v>
       </c>
       <c r="D2" s="0" t="n">
         <f aca="false">Pesimista!B74</f>
-        <v>-94161.0656562552</v>
+        <v>-94162.2870130552</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3251,11 +3251,11 @@
       </c>
       <c r="B3" s="2" t="n">
         <f aca="false">Optimista!B75</f>
-        <v>55.5453931939874</v>
+        <v>55.5120890005778</v>
       </c>
       <c r="C3" s="2" t="n">
         <f aca="false">Neutral!B75</f>
-        <v>0.725504464517237</v>
+        <v>0.725481790486073</v>
       </c>
       <c r="D3" s="2" t="str">
         <f aca="false">Pesimista!B75</f>
@@ -3268,11 +3268,11 @@
       </c>
       <c r="B4" s="0" t="n">
         <f aca="false">Optimista!B76</f>
-        <v>0.0184589758553011</v>
+        <v>0.0184703222077383</v>
       </c>
       <c r="C4" s="0" t="n">
         <f aca="false">Neutral!B76</f>
-        <v>2.93217357426835</v>
+        <v>2.93218828176455</v>
       </c>
       <c r="D4" s="0" t="str">
         <f aca="false">Pesimista!B76</f>
@@ -3285,11 +3285,11 @@
       </c>
       <c r="B5" s="0" t="n">
         <f aca="false">Optimista!B77</f>
-        <v>0.0230737198191263</v>
+        <v>0.0230879027596729</v>
       </c>
       <c r="C5" s="0" t="n">
         <f aca="false">Neutral!B77</f>
-        <v>3.46221348733306</v>
+        <v>3.46225271364738</v>
       </c>
       <c r="D5" s="0" t="str">
         <f aca="false">Pesimista!B77</f>
@@ -3336,15 +3336,15 @@
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">Optimista!B78</f>
-        <v>1609256.85245787</v>
+        <v>1609255.92770156</v>
       </c>
       <c r="C8" s="0" t="n">
         <f aca="false">Neutral!B78</f>
-        <v>199501.165457116</v>
+        <v>199500.125116803</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">Pesimista!B78</f>
-        <v>-94161.0656562552</v>
+        <v>-94162.2870130552</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4760,23 +4760,23 @@
       </c>
       <c r="C49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*C6/ua_escalado)+dominio_anual</f>
-        <v>305.5</v>
+        <v>305.56</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*D6/ua_escalado)+dominio_anual</f>
-        <v>485.5</v>
+        <v>485.56</v>
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*E6/ua_escalado)+dominio_anual</f>
-        <v>845.5</v>
+        <v>845.56</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*F6/ua_escalado)+dominio_anual</f>
-        <v>1445.5</v>
+        <v>1445.56</v>
       </c>
       <c r="G49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*G6/ua_escalado)+dominio_anual</f>
-        <v>2045.5</v>
+        <v>2045.56</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="B51" s="0" t="n">
         <f aca="false">inv_dominio+inv_marca_inpi+inv_legal</f>
-        <v>1558.5</v>
+        <v>1559.56</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4869,27 +4869,27 @@
       </c>
       <c r="B54" s="0" t="n">
         <f aca="false">SUM(B48:B53)</f>
-        <v>1714.5</v>
+        <v>1715.56</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">SUM(C48:C53)</f>
-        <v>47643.742</v>
+        <v>47643.802</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">SUM(D48:D53)</f>
-        <v>74659.9549</v>
+        <v>74660.0149</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">SUM(E48:E53)</f>
-        <v>104777.594125</v>
+        <v>104777.654125</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">SUM(F48:F53)</f>
-        <v>140354.42795125</v>
+        <v>140354.48795125</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">SUM(G48:G53)</f>
-        <v>173905.709868813</v>
+        <v>173905.769868813</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4903,27 +4903,27 @@
       </c>
       <c r="B57" s="0" t="n">
         <f aca="false">B45-B54</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C57" s="0" t="n">
         <f aca="false">C45-C54</f>
-        <v>207356.258</v>
+        <v>207356.198</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">D45-D54</f>
-        <v>398740.0451</v>
+        <v>398739.9851</v>
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">E45-E54</f>
-        <v>686622.405875</v>
+        <v>686622.345875</v>
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">F45-F54</f>
-        <v>708645.57204875</v>
+        <v>708645.51204875</v>
       </c>
       <c r="G57" s="0" t="n">
         <f aca="false">G45-G54</f>
-        <v>871894.290131188</v>
+        <v>871894.230131188</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">MIN(0,B57)</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">MIN(0,B58+C57)</f>
@@ -4965,23 +4965,23 @@
       </c>
       <c r="C59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,B58+C57)</f>
-        <v>71974.6153</v>
+        <v>71974.2233</v>
       </c>
       <c r="D59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,C58+D57)</f>
-        <v>139559.015785</v>
+        <v>139558.994785</v>
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,D58+E57)</f>
-        <v>240317.84205625</v>
+        <v>240317.82105625</v>
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,E58+F57)</f>
-        <v>248025.950217063</v>
+        <v>248025.929217062</v>
       </c>
       <c r="G59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,F58+G57)</f>
-        <v>305163.001545916</v>
+        <v>305162.980545916</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5062,27 +5062,27 @@
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">B57-B59-B61+N(B62)</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C65" s="0" t="n">
         <f aca="false">C57-C59-C61+N(C62)</f>
-        <v>92881.6427</v>
+        <v>92881.9747</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">D57-D59-D61+N(D62)</f>
-        <v>222781.029315</v>
+        <v>222780.990315</v>
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">E57-E59-E61+N(E62)</f>
-        <v>393304.56381875</v>
+        <v>393304.52481875</v>
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">F57-F59-F61+N(F62)</f>
-        <v>451019.621831688</v>
+        <v>451019.582831688</v>
       </c>
       <c r="G65" s="0" t="n">
         <f aca="false">G57-G59-G61+N(G62)</f>
-        <v>708231.288585272</v>
+        <v>708231.249585272</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5120,27 +5120,27 @@
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">B65*B66</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C67" s="0" t="n">
         <f aca="false">C65*C66</f>
-        <v>74305.31416</v>
+        <v>74305.57976</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">D65*D66</f>
-        <v>142579.8587616</v>
+        <v>142579.8338016</v>
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">E65*E66</f>
-        <v>201371.9366752</v>
+        <v>201371.9167072</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">F65*F66</f>
-        <v>184737.637102259</v>
+        <v>184737.621127859</v>
       </c>
       <c r="G67" s="0" t="n">
         <f aca="false">G65*G66</f>
-        <v>232073.228643622</v>
+        <v>232073.215864102</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5149,27 +5149,27 @@
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B65</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">B68+C65</f>
-        <v>91167.1427</v>
+        <v>91166.4147</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">C68+D65</f>
-        <v>313948.172015</v>
+        <v>313947.405015</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">D68+E65</f>
-        <v>707252.73583375</v>
+        <v>707251.92983375</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">E68+F65</f>
-        <v>1158272.35766544</v>
+        <v>1158271.51266544</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">F68+G65</f>
-        <v>1866503.64625071</v>
+        <v>1866502.76225071</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5178,27 +5178,27 @@
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B67</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">B69+C67</f>
-        <v>72590.81416</v>
+        <v>72590.01976</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">C69+D67</f>
-        <v>215170.6729216</v>
+        <v>215169.8535616</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E67</f>
-        <v>416542.6095968</v>
+        <v>416541.7702688</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F67</f>
-        <v>601280.246699059</v>
+        <v>601279.391396659</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G67</f>
-        <v>833353.475342681</v>
+        <v>833352.607260761</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="C70" s="0" t="n">
         <f aca="false">IF(AND(B68&lt;0,C68&gt;=0),C$3-1+(-B68)/C65,"")</f>
-        <v>0.0184589758553011</v>
+        <v>0.0184703222077383</v>
       </c>
       <c r="D70" s="0" t="str">
         <f aca="false">IF(AND(C68&lt;0,D68&gt;=0),D$3-1+(-C68)/D65,"")</f>
@@ -5232,7 +5232,7 @@
       </c>
       <c r="C71" s="0" t="n">
         <f aca="false">IF(AND(B69&lt;0,C69&gt;=0),C$3-1+(-B69)/C67,"")</f>
-        <v>0.0230737198191263</v>
+        <v>0.0230879027596729</v>
       </c>
       <c r="D71" s="0" t="str">
         <f aca="false">IF(AND(C69&lt;0,D69&gt;=0),D$3-1+(-C69)/D67,"")</f>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">SUM(B67:G67)</f>
-        <v>833353.475342681</v>
+        <v>833352.607260761</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B75" s="2" t="n">
         <f aca="false">IFERROR(IRR(B65:G65),"no definida")</f>
-        <v>55.5453931939874</v>
+        <v>55.5120890005778</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B76" s="0" t="n">
         <f aca="false">IF(COUNT(C70:G70)=0,"no se recupera",MIN(C70:G70))</f>
-        <v>0.0184589758553011</v>
+        <v>0.0184703222077383</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
-        <v>0.0230737198191263</v>
+        <v>0.0230879027596729</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">SUM(B67:G67)+MAX(0,G65-G62)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>1609256.85245787</v>
+        <v>1609255.92770156</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6395,23 +6395,23 @@
       </c>
       <c r="C49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*C6/ua_escalado)+dominio_anual</f>
-        <v>269.5</v>
+        <v>269.56</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*D6/ua_escalado)+dominio_anual</f>
-        <v>341.5</v>
+        <v>341.56</v>
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*E6/ua_escalado)+dominio_anual</f>
-        <v>485.5</v>
+        <v>485.56</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*F6/ua_escalado)+dominio_anual</f>
-        <v>725.5</v>
+        <v>725.56</v>
       </c>
       <c r="G49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*G6/ua_escalado)+dominio_anual</f>
-        <v>965.5</v>
+        <v>965.56</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="B51" s="0" t="n">
         <f aca="false">inv_dominio+inv_marca_inpi+inv_legal</f>
-        <v>1558.5</v>
+        <v>1559.56</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6504,27 +6504,27 @@
       </c>
       <c r="B54" s="0" t="n">
         <f aca="false">SUM(B48:B53)</f>
-        <v>1714.5</v>
+        <v>1715.56</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">SUM(C48:C53)</f>
-        <v>37125.806</v>
+        <v>37125.866</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">SUM(D48:D53)</f>
-        <v>61852.0957</v>
+        <v>61852.1557</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">SUM(E48:E53)</f>
-        <v>107014.291725</v>
+        <v>107014.351725</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">SUM(F48:F53)</f>
-        <v>154837.41675125</v>
+        <v>154837.47675125</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">SUM(G48:G53)</f>
-        <v>197777.165868813</v>
+        <v>197777.225868813</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6538,27 +6538,27 @@
       </c>
       <c r="B57" s="0" t="n">
         <f aca="false">B45-B54</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C57" s="0" t="n">
         <f aca="false">C45-C54</f>
-        <v>-37125.806</v>
+        <v>-37125.866</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">D45-D54</f>
-        <v>-4252.09570000001</v>
+        <v>-4252.1557</v>
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">E45-E54</f>
-        <v>102785.708275</v>
+        <v>102785.648275</v>
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">F45-F54</f>
-        <v>104962.58324875</v>
+        <v>104962.52324875</v>
       </c>
       <c r="G57" s="0" t="n">
         <f aca="false">G45-G54</f>
-        <v>171622.834131188</v>
+        <v>171622.774131188</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6567,15 +6567,15 @@
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">MIN(0,B57)</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">MIN(0,B58+C57)</f>
-        <v>-38840.306</v>
+        <v>-38841.426</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">MIN(0,C58+D57)</f>
-        <v>-43092.4017</v>
+        <v>-43093.5817</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">MIN(0,D58+E57)</f>
@@ -6608,15 +6608,15 @@
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,D58+E57)</f>
-        <v>20892.65730125</v>
+        <v>20892.22330125</v>
       </c>
       <c r="F59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,E58+F57)</f>
-        <v>36736.9041370625</v>
+        <v>36736.8831370625</v>
       </c>
       <c r="G59" s="0" t="n">
         <f aca="false">alicuota_ganancias*MAX(0,F58+G57)</f>
-        <v>60067.9919459156</v>
+        <v>60067.9709459156</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6697,27 +6697,27 @@
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">B57-B59-B61+N(B62)</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C65" s="0" t="n">
         <f aca="false">C57-C59-C61+N(C62)</f>
-        <v>-37125.806</v>
+        <v>-37125.866</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">D57-D59-D61+N(D62)</f>
-        <v>-13852.0957</v>
+        <v>-13852.1557</v>
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">E57-E59-E61+N(E62)</f>
-        <v>56526.3843070833</v>
+        <v>56526.7583070833</v>
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">F57-F59-F61+N(F62)</f>
-        <v>59892.3457783542</v>
+        <v>59892.3067783542</v>
       </c>
       <c r="G65" s="0" t="n">
         <f aca="false">G57-G59-G61+N(G62)</f>
-        <v>154854.842185272</v>
+        <v>154854.803185272</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6755,27 +6755,27 @@
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">B65*B66</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C67" s="0" t="n">
         <f aca="false">C65*C66</f>
-        <v>-29700.6448</v>
+        <v>-29700.6928</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">D65*D66</f>
-        <v>-8865.341248</v>
+        <v>-8865.379648</v>
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">E65*E66</f>
-        <v>28941.5087652267</v>
+        <v>28941.7002532267</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">F65*F66</f>
-        <v>24531.9048308139</v>
+        <v>24531.8888564139</v>
       </c>
       <c r="G67" s="0" t="n">
         <f aca="false">G65*G66</f>
-        <v>50742.8346872699</v>
+        <v>50742.8219077499</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6784,27 +6784,27 @@
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B65</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">B68+C65</f>
-        <v>-38840.306</v>
+        <v>-38841.426</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">C68+D65</f>
-        <v>-52692.4017</v>
+        <v>-52693.5817</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">D68+E65</f>
-        <v>3833.98260708334</v>
+        <v>3833.17660708334</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">E68+F65</f>
-        <v>63726.3283854375</v>
+        <v>63725.4833854375</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">F68+G65</f>
-        <v>218581.170570709</v>
+        <v>218580.286570709</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6813,27 +6813,27 @@
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B67</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">B69+C67</f>
-        <v>-31415.1448</v>
+        <v>-31416.2528</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">C69+D67</f>
-        <v>-40280.486048</v>
+        <v>-40281.632448</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E67</f>
-        <v>-11338.9772827733</v>
+        <v>-11339.9321947733</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F67</f>
-        <v>13192.9275480405</v>
+        <v>13191.9566616405</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G67</f>
-        <v>63935.7622353104</v>
+        <v>63934.7785693904</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">IF(AND(D68&lt;0,E68&gt;=0),E$3-1+(-D68)/E65,"")</f>
-        <v>2.93217357426835</v>
+        <v>2.93218828176455</v>
       </c>
       <c r="F70" s="0" t="str">
         <f aca="false">IF(AND(E68&lt;0,F68&gt;=0),F$3-1+(-E68)/F65,"")</f>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="F71" s="0" t="n">
         <f aca="false">IF(AND(E69&lt;0,F69&gt;=0),F$3-1+(-E69)/F67,"")</f>
-        <v>3.46221348733306</v>
+        <v>3.46225271364738</v>
       </c>
       <c r="G71" s="0" t="str">
         <f aca="false">IF(AND(F69&lt;0,G69&gt;=0),G$3-1+(-F69)/G67,"")</f>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">SUM(B67:G67)</f>
-        <v>63935.7622353104</v>
+        <v>63934.7785693904</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="B75" s="2" t="n">
         <f aca="false">IFERROR(IRR(B65:G65),"no definida")</f>
-        <v>0.725504464517237</v>
+        <v>0.725481790486073</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6915,7 +6915,7 @@
       </c>
       <c r="B76" s="0" t="n">
         <f aca="false">IF(COUNT(C70:G70)=0,"no se recupera",MIN(C70:G70))</f>
-        <v>2.93217357426835</v>
+        <v>2.93218828176455</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6924,7 +6924,7 @@
       </c>
       <c r="B77" s="0" t="n">
         <f aca="false">IF(COUNT(C71:G71)=0,"no se recupera",MIN(C71:G71))</f>
-        <v>3.46221348733306</v>
+        <v>3.46225271364738</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">SUM(B67:G67)+MAX(0,G65-G62)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>199501.165457116</v>
+        <v>199500.125116803</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8030,23 +8030,23 @@
       </c>
       <c r="C49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*C6/ua_escalado)+dominio_anual</f>
-        <v>251.5</v>
+        <v>251.56</v>
       </c>
       <c r="D49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*D6/ua_escalado)+dominio_anual</f>
-        <v>269.5</v>
+        <v>269.56</v>
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*E6/ua_escalado)+dominio_anual</f>
-        <v>305.5</v>
+        <v>305.56</v>
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*F6/ua_escalado)+dominio_anual</f>
-        <v>341.5</v>
+        <v>341.56</v>
       </c>
       <c r="G49" s="0" t="n">
         <f aca="false">meses_anio*(infra_base+infra_escalado*G6/ua_escalado)+dominio_anual</f>
-        <v>365.5</v>
+        <v>365.56</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="B51" s="0" t="n">
         <f aca="false">inv_dominio+inv_marca_inpi+inv_legal</f>
-        <v>1558.5</v>
+        <v>1559.56</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8139,27 +8139,27 @@
       </c>
       <c r="B54" s="0" t="n">
         <f aca="false">SUM(B48:B53)</f>
-        <v>1714.5</v>
+        <v>1715.56</v>
       </c>
       <c r="C54" s="0" t="n">
         <f aca="false">SUM(C48:C53)</f>
-        <v>33948.846</v>
+        <v>33948.906</v>
       </c>
       <c r="D54" s="0" t="n">
         <f aca="false">SUM(D48:D53)</f>
-        <v>39239.5645</v>
+        <v>39239.6245</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">SUM(E48:E53)</f>
-        <v>64670.240525</v>
+        <v>64670.300525</v>
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">SUM(F48:F53)</f>
-        <v>98381.95435125</v>
+        <v>98382.01435125</v>
       </c>
       <c r="G54" s="0" t="n">
         <f aca="false">SUM(G48:G53)</f>
-        <v>113943.802668813</v>
+        <v>113943.862668813</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8173,27 +8173,27 @@
       </c>
       <c r="B57" s="0" t="n">
         <f aca="false">B45-B54</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C57" s="0" t="n">
         <f aca="false">C45-C54</f>
-        <v>-33948.846</v>
+        <v>-33948.906</v>
       </c>
       <c r="D57" s="0" t="n">
         <f aca="false">D45-D54</f>
-        <v>-39239.5645</v>
+        <v>-39239.6245</v>
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">E45-E54</f>
-        <v>-29470.240525</v>
+        <v>-29470.300525</v>
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">F45-F54</f>
-        <v>-35981.95435125</v>
+        <v>-35982.01435125</v>
       </c>
       <c r="G57" s="0" t="n">
         <f aca="false">G45-G54</f>
-        <v>-27143.8026688125</v>
+        <v>-27143.8626688125</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8202,27 +8202,27 @@
       </c>
       <c r="B58" s="0" t="n">
         <f aca="false">MIN(0,B57)</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C58" s="0" t="n">
         <f aca="false">MIN(0,B58+C57)</f>
-        <v>-35663.346</v>
+        <v>-35664.466</v>
       </c>
       <c r="D58" s="0" t="n">
         <f aca="false">MIN(0,C58+D57)</f>
-        <v>-74902.9105</v>
+        <v>-74904.0905</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">MIN(0,D58+E57)</f>
-        <v>-104373.151025</v>
+        <v>-104374.391025</v>
       </c>
       <c r="F58" s="0" t="n">
         <f aca="false">MIN(0,E58+F57)</f>
-        <v>-140355.10537625</v>
+        <v>-140356.40537625</v>
       </c>
       <c r="G58" s="0" t="n">
         <f aca="false">MIN(0,F58+G57)</f>
-        <v>-167498.908045063</v>
+        <v>-167500.268045063</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8332,27 +8332,27 @@
       </c>
       <c r="B65" s="0" t="n">
         <f aca="false">B57-B59-B61+N(B62)</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C65" s="0" t="n">
         <f aca="false">C57-C59-C61+N(C62)</f>
-        <v>-33948.846</v>
+        <v>-33948.906</v>
       </c>
       <c r="D65" s="0" t="n">
         <f aca="false">D57-D59-D61+N(D62)</f>
-        <v>-39239.5645</v>
+        <v>-39239.6245</v>
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">E57-E59-E61+N(E62)</f>
-        <v>-35336.9071916667</v>
+        <v>-35336.9671916667</v>
       </c>
       <c r="F65" s="0" t="n">
         <f aca="false">F57-F59-F61+N(F62)</f>
-        <v>-40515.2876845833</v>
+        <v>-40515.3476845833</v>
       </c>
       <c r="G65" s="0" t="n">
         <f aca="false">G57-G59-G61+N(G62)</f>
-        <v>-16743.8026688125</v>
+        <v>-16743.8626688125</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8390,27 +8390,27 @@
       </c>
       <c r="B67" s="0" t="n">
         <f aca="false">B65*B66</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C67" s="0" t="n">
         <f aca="false">C65*C66</f>
-        <v>-27159.0768</v>
+        <v>-27159.1248</v>
       </c>
       <c r="D67" s="0" t="n">
         <f aca="false">D65*D66</f>
-        <v>-25113.32128</v>
+        <v>-25113.35968</v>
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">E65*E66</f>
-        <v>-18092.4964821333</v>
+        <v>-18092.5272021333</v>
       </c>
       <c r="F67" s="0" t="n">
         <f aca="false">F65*F66</f>
-        <v>-16595.0618356053</v>
+        <v>-16595.0864116053</v>
       </c>
       <c r="G67" s="0" t="n">
         <f aca="false">G65*G66</f>
-        <v>-5486.60925851648</v>
+        <v>-5486.62891931648</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8419,27 +8419,27 @@
       </c>
       <c r="B68" s="0" t="n">
         <f aca="false">B65</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C68" s="0" t="n">
         <f aca="false">B68+C65</f>
-        <v>-35663.346</v>
+        <v>-35664.466</v>
       </c>
       <c r="D68" s="0" t="n">
         <f aca="false">C68+D65</f>
-        <v>-74902.9105</v>
+        <v>-74904.0905</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">D68+E65</f>
-        <v>-110239.817691667</v>
+        <v>-110241.057691667</v>
       </c>
       <c r="F68" s="0" t="n">
         <f aca="false">E68+F65</f>
-        <v>-150755.10537625</v>
+        <v>-150756.40537625</v>
       </c>
       <c r="G68" s="0" t="n">
         <f aca="false">F68+G65</f>
-        <v>-167498.908045063</v>
+        <v>-167500.268045063</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8448,27 +8448,27 @@
       </c>
       <c r="B69" s="0" t="n">
         <f aca="false">B67</f>
-        <v>-1714.5</v>
+        <v>-1715.56</v>
       </c>
       <c r="C69" s="0" t="n">
         <f aca="false">B69+C67</f>
-        <v>-28873.5768</v>
+        <v>-28874.6848</v>
       </c>
       <c r="D69" s="0" t="n">
         <f aca="false">C69+D67</f>
-        <v>-53986.89808</v>
+        <v>-53988.04448</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">D69+E67</f>
-        <v>-72079.3945621333</v>
+        <v>-72080.5716821334</v>
       </c>
       <c r="F69" s="0" t="n">
         <f aca="false">E69+F67</f>
-        <v>-88674.4563977387</v>
+        <v>-88675.6580937387</v>
       </c>
       <c r="G69" s="0" t="n">
         <f aca="false">F69+G67</f>
-        <v>-94161.0656562552</v>
+        <v>-94162.2870130552</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="B74" s="0" t="n">
         <f aca="false">SUM(B67:G67)</f>
-        <v>-94161.0656562552</v>
+        <v>-94162.2870130552</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="B78" s="0" t="n">
         <f aca="false">SUM(B67:G67)+MAX(0,G65-G62)*(1+crecimiento_perpetuo)/(tasa_descuento-crecimiento_perpetuo)/(1+tasa_descuento)^5</f>
-        <v>-94161.0656562552</v>
+        <v>-94162.2870130552</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Corregir los defectos de la segunda ronda de evaluadores ciegos
- Cap. 4: quitar la contradicción sobre la ingesta y la memoria en 4.2.5,
  Tabla 4.XXIII en longtable y costo del LLM como cota, síntesis 4.3.6
  sin cifras repetidas
- Fig. 4.12: puntaje de confianza en lugar de probabilidad
- Anexo E: citas de la Constitución, Railway y la Ley 27.630 resueltas;
  ruta del script quitada; planilla regenerada y validada sin cambios
- Cap. 3: justificar el tipo de cambio de la encuesta para el sueldo
- Cap. 2: párrafo repetido de 2.1.2, fuentes de la Tabla 2.III y colores
  de la curva de valor
- wiki/sintesis/evaluacion-ciega-rubrica.md: 84,4 → 86,1

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -343,7 +343,7 @@
     <t xml:space="preserve">Impuesto a las ganancias, con quebrantos trasladables</t>
   </si>
   <si>
-    <t xml:space="preserve">Simplificación indicada por la cátedra</t>
+    <t xml:space="preserve">Alícuota máxima de la escala, CongresoNacion2021</t>
   </si>
   <si>
     <t xml:space="preserve">meses_cobro</t>
@@ -400,7 +400,7 @@
     <t xml:space="preserve">Base comercial: Railway Pro, con 20 USD de uso incluidos (API y clasificador, 13 USD/mes)</t>
   </si>
   <si>
-    <t xml:space="preserve">Railway2026</t>
+    <t xml:space="preserve">RailwayPrecios2026</t>
   </si>
   <si>
     <t xml:space="preserve">infra_escalado</t>
@@ -775,7 +775,7 @@
     <t xml:space="preserve">Churn anual: agencias</t>
   </si>
   <si>
-    <t xml:space="preserve">Sensibilidad (1 = caso base; los cambia scripts/sensibilidad_modelo_financiero.py)</t>
+    <t xml:space="preserve">Sensibilidad (1 = caso base)</t>
   </si>
   <si>
     <t xml:space="preserve">sens_costo_analisis</t>

</xml_diff>

<commit_message>
Corregir los defectos de la tercera ronda de evaluadores ciegos
- Cap. 4: remisión a la ingesta, fila de sqlite-vec en la Tabla 4.IX,
  orden de las Figs. 4.9 y 4.10, casos de prueba 1, 5, 6 y 7 y síntesis
- Cap. 2: quitar las frases valorativas del marco teórico
- Un término por concepto: combinador, tasa de bajas, período de
  recuperación, informe, ajuste fino, señal del texto y otros, también en
  c4-componentes, flujo-informacion y las tablas del financiero
- Cap. 1: objetivo 2 en oraciones cortas, con aviso de la reformulación
- wiki/sintesis/evaluacion-ciega-rubrica.md: ronda 3 (86,6)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/negocio/modelo-financiero.xlsx
+++ b/wiki/negocio/modelo-financiero.xlsx
@@ -274,7 +274,7 @@
     <t xml:space="preserve">sueldo_ars</t>
   </si>
   <si>
-    <t xml:space="preserve">Sueldo bruto mensual, developer semi senior</t>
+    <t xml:space="preserve">Sueldo bruto mensual, desarrollador semi senior</t>
   </si>
   <si>
     <t xml:space="preserve">ARS/mes</t>
@@ -748,31 +748,31 @@
     <t xml:space="preserve">churn_medios_grandes</t>
   </si>
   <si>
-    <t xml:space="preserve">Churn anual: medios de gran porte</t>
+    <t xml:space="preserve">Tasa de bajas anual: medios de gran porte</t>
   </si>
   <si>
     <t xml:space="preserve">churn_medios_chicos</t>
   </si>
   <si>
-    <t xml:space="preserve">Churn anual: resto de medios de ADEPA</t>
+    <t xml:space="preserve">Tasa de bajas anual: resto de medios de ADEPA</t>
   </si>
   <si>
     <t xml:space="preserve">churn_verificadores</t>
   </si>
   <si>
-    <t xml:space="preserve">Churn anual: verificadores</t>
+    <t xml:space="preserve">Tasa de bajas anual: verificadores</t>
   </si>
   <si>
     <t xml:space="preserve">churn_universidades</t>
   </si>
   <si>
-    <t xml:space="preserve">Churn anual: universidades</t>
+    <t xml:space="preserve">Tasa de bajas anual: universidades</t>
   </si>
   <si>
     <t xml:space="preserve">churn_agencias</t>
   </si>
   <si>
-    <t xml:space="preserve">Churn anual: agencias</t>
+    <t xml:space="preserve">Tasa de bajas anual: agencias</t>
   </si>
   <si>
     <t xml:space="preserve">Sensibilidad (1 = caso base)</t>

</xml_diff>